<commit_message>
Konteringsoppsett: full formelkjede for alle poster, lagreknapp og bytte av konto
- Innandørsmekanisering er nå en ekte formel (kontoer × andel), som maskinkostnader
- Fordelingsnøkler viser grunnlag og kan endres direkte i formelen
- Driftsmessige avskrivninger vises med riktig kilde (60xx etter korrigering)
- Totaløkonomi viser summer per produksjon kompakt, bare aktive produksjoner
- Automatiske poster viser kontoene som faktisk inngår
- Innstillinger: endringer lagres først med Lagre, kan forkastes
- Klikk en konto-brikke for å bytte den ut; dra over kontoer for intervall

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HrtCx2hBap2TXaC318T6kC
</commit_message>
<xml_diff>
--- a/excel/Analyse_jordbruk_produksjonar.xlsx
+++ b/excel/Analyse_jordbruk_produksjonar.xlsx
@@ -9023,7 +9023,7 @@
         </is>
       </c>
       <c r="C48" s="13">
-        <f>'Faste kostnader'!C65</f>
+        <f>'Faste kostnader'!C77</f>
         <v/>
       </c>
       <c r="D48" s="12" t="inlineStr">
@@ -9033,12 +9033,12 @@
       </c>
       <c r="E48" s="23" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Mjølk [Faste kostnader!C65]</t>
+          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Mjølk [Faste kostnader!C77]</t>
         </is>
       </c>
       <c r="F48" s="24" t="inlineStr">
         <is>
-          <t>='Faste kostnader'!C65</t>
+          <t>='Faste kostnader'!C77</t>
         </is>
       </c>
     </row>
@@ -11670,7 +11670,7 @@
         </is>
       </c>
       <c r="C45" s="13">
-        <f>'Faste kostnader'!C66</f>
+        <f>'Faste kostnader'!C78</f>
         <v/>
       </c>
       <c r="D45" s="12" t="inlineStr">
@@ -11680,12 +11680,12 @@
       </c>
       <c r="E45" s="23" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Oksar [Faste kostnader!C66]</t>
+          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Oksar [Faste kostnader!C78]</t>
         </is>
       </c>
       <c r="F45" s="24" t="inlineStr">
         <is>
-          <t>='Faste kostnader'!C66</t>
+          <t>='Faste kostnader'!C78</t>
         </is>
       </c>
     </row>
@@ -14162,7 +14162,7 @@
         </is>
       </c>
       <c r="C45" s="13">
-        <f>'Faste kostnader'!C67</f>
+        <f>'Faste kostnader'!C79</f>
         <v/>
       </c>
       <c r="D45" s="12" t="inlineStr">
@@ -14172,12 +14172,12 @@
       </c>
       <c r="E45" s="23" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Mellomkalv [Faste kostnader!C67]</t>
+          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Mellomkalv [Faste kostnader!C79]</t>
         </is>
       </c>
       <c r="F45" s="24" t="inlineStr">
         <is>
-          <t>='Faste kostnader'!C67</t>
+          <t>='Faste kostnader'!C79</t>
         </is>
       </c>
     </row>
@@ -16784,7 +16784,7 @@
         </is>
       </c>
       <c r="C50" s="13">
-        <f>'Faste kostnader'!C68</f>
+        <f>'Faste kostnader'!C80</f>
         <v/>
       </c>
       <c r="D50" s="12" t="inlineStr">
@@ -16794,12 +16794,12 @@
       </c>
       <c r="E50" s="23" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Ammekyr [Faste kostnader!C68]</t>
+          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Ammekyr [Faste kostnader!C80]</t>
         </is>
       </c>
       <c r="F50" s="24" t="inlineStr">
         <is>
-          <t>='Faste kostnader'!C68</t>
+          <t>='Faste kostnader'!C80</t>
         </is>
       </c>
     </row>
@@ -18900,7 +18900,7 @@
         </is>
       </c>
       <c r="C30" s="13">
-        <f>'Faste kostnader'!C69</f>
+        <f>'Faste kostnader'!C81</f>
         <v/>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -18910,12 +18910,12 @@
       </c>
       <c r="E30" s="23" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Smågris [Faste kostnader!C69]</t>
+          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Smågris [Faste kostnader!C81]</t>
         </is>
       </c>
       <c r="F30" s="24" t="inlineStr">
         <is>
-          <t>='Faste kostnader'!C69</t>
+          <t>='Faste kostnader'!C81</t>
         </is>
       </c>
     </row>
@@ -22108,7 +22108,7 @@
         </is>
       </c>
       <c r="C31" s="13">
-        <f>'Faste kostnader'!C70</f>
+        <f>'Faste kostnader'!C82</f>
         <v/>
       </c>
       <c r="D31" s="12" t="inlineStr">
@@ -22118,12 +22118,12 @@
       </c>
       <c r="E31" s="23" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Purkering [Faste kostnader!C70]</t>
+          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Purkering [Faste kostnader!C82]</t>
         </is>
       </c>
       <c r="F31" s="24" t="inlineStr">
         <is>
-          <t>='Faste kostnader'!C70</t>
+          <t>='Faste kostnader'!C82</t>
         </is>
       </c>
     </row>
@@ -24022,7 +24022,7 @@
         </is>
       </c>
       <c r="C27" s="13">
-        <f>'Faste kostnader'!C71</f>
+        <f>'Faste kostnader'!C83</f>
         <v/>
       </c>
       <c r="D27" s="12" t="inlineStr">
@@ -24032,12 +24032,12 @@
       </c>
       <c r="E27" s="23" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Slaktegris [Faste kostnader!C71]</t>
+          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Slaktegris [Faste kostnader!C83]</t>
         </is>
       </c>
       <c r="F27" s="24" t="inlineStr">
         <is>
-          <t>='Faste kostnader'!C71</t>
+          <t>='Faste kostnader'!C83</t>
         </is>
       </c>
     </row>
@@ -26397,7 +26397,7 @@
         </is>
       </c>
       <c r="C56" s="13">
-        <f>'Faste kostnader'!C72</f>
+        <f>'Faste kostnader'!C84</f>
         <v/>
       </c>
       <c r="D56" s="12" t="inlineStr">
@@ -26407,12 +26407,12 @@
       </c>
       <c r="E56" s="23" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Sau [Faste kostnader!C72]</t>
+          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Sau [Faste kostnader!C84]</t>
         </is>
       </c>
       <c r="F56" s="24" t="inlineStr">
         <is>
-          <t>='Faste kostnader'!C72</t>
+          <t>='Faste kostnader'!C84</t>
         </is>
       </c>
     </row>
@@ -28987,7 +28987,7 @@
         </is>
       </c>
       <c r="C44" s="13">
-        <f>'Faste kostnader'!C73</f>
+        <f>'Faste kostnader'!C85</f>
         <v/>
       </c>
       <c r="D44" s="12" t="inlineStr">
@@ -28997,12 +28997,12 @@
       </c>
       <c r="E44" s="23" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Geit [Faste kostnader!C73]</t>
+          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Geit [Faste kostnader!C85]</t>
         </is>
       </c>
       <c r="F44" s="24" t="inlineStr">
         <is>
-          <t>='Faste kostnader'!C73</t>
+          <t>='Faste kostnader'!C85</t>
         </is>
       </c>
     </row>
@@ -30926,7 +30926,7 @@
         </is>
       </c>
       <c r="C22" s="13">
-        <f>'Faste kostnader'!C74</f>
+        <f>'Faste kostnader'!C86</f>
         <v/>
       </c>
       <c r="D22" s="12" t="inlineStr">
@@ -30936,12 +30936,12 @@
       </c>
       <c r="E22" s="23" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Egg [Faste kostnader!C74]</t>
+          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Egg [Faste kostnader!C86]</t>
         </is>
       </c>
       <c r="F22" s="24" t="inlineStr">
         <is>
-          <t>='Faste kostnader'!C74</t>
+          <t>='Faste kostnader'!C86</t>
         </is>
       </c>
     </row>
@@ -32468,7 +32468,7 @@
         </is>
       </c>
       <c r="C27" s="13">
-        <f>'Faste kostnader'!C75</f>
+        <f>'Faste kostnader'!C87</f>
         <v/>
       </c>
       <c r="D27" s="12" t="inlineStr">
@@ -32478,12 +32478,12 @@
       </c>
       <c r="E27" s="23" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Slaktekylling [Faste kostnader!C75]</t>
+          <t>Innandørsmekanisering fordelt = Innandørsmekanisering – Slaktekylling [Faste kostnader!C87]</t>
         </is>
       </c>
       <c r="F27" s="24" t="inlineStr">
         <is>
-          <t>='Faste kostnader'!C75</t>
+          <t>='Faste kostnader'!C87</t>
         </is>
       </c>
     </row>
@@ -41526,7 +41526,7 @@
         </is>
       </c>
       <c r="C17" s="13">
-        <f>'Faste kostnader'!C90</f>
+        <f>'Faste kostnader'!C102</f>
         <v/>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -41536,12 +41536,12 @@
       </c>
       <c r="E17" s="23" t="inlineStr">
         <is>
-          <t>Sum faste kostnader = Sum faste kostnader jordbruk [Faste kostnader!C90]</t>
+          <t>Sum faste kostnader = Sum faste kostnader jordbruk [Faste kostnader!C102]</t>
         </is>
       </c>
       <c r="F17" s="24" t="inlineStr">
         <is>
-          <t>='Faste kostnader'!C90</t>
+          <t>='Faste kostnader'!C102</t>
         </is>
       </c>
     </row>
@@ -41617,16 +41617,16 @@
     <row r="21">
       <c r="A21" s="20" t="inlineStr">
         <is>
-          <t>Beholdningsendring buskap/varelager, skattemessig (+ = auke)</t>
+          <t>Driftsmessige avskrivingar</t>
         </is>
       </c>
       <c r="B21" s="24" t="inlineStr">
         <is>
-          <t>4090-4099, 4190-4199, 4290-4299, 4690-4699 (før korrigering)</t>
+          <t>60xx i saldobalansen (etter korrigering)</t>
         </is>
       </c>
       <c r="C21" s="31" t="n">
-        <v>-58135</v>
+        <v>246072.11</v>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
@@ -41635,7 +41635,7 @@
       </c>
       <c r="E21" s="24" t="inlineStr">
         <is>
-          <t>Input. Hentast frå: 4090-4099, 4190-4199, 4290-4299, 4690-4699 (før korrigering).</t>
+          <t>Input. Hentast frå: 60xx i saldobalansen (etter korrigering).</t>
         </is>
       </c>
       <c r="F21" s="32" t="n"/>
@@ -41643,16 +41643,16 @@
     <row r="22">
       <c r="A22" s="20" t="inlineStr">
         <is>
-          <t>Beholdningsendring buskap/varelager, driftsmessig (+ = auke)</t>
+          <t>Beholdningsendring buskap/varelager, skattemessig (+ = auke)</t>
         </is>
       </c>
       <c r="B22" s="24" t="inlineStr">
         <is>
-          <t>Etter korrigering til driftsmessige verdiar</t>
+          <t>4090-4099, 4190-4199, 4290-4299, 4690-4699 (før korrigering)</t>
         </is>
       </c>
       <c r="C22" s="31" t="n">
-        <v>3740</v>
+        <v>-58135</v>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
@@ -41661,7 +41661,7 @@
       </c>
       <c r="E22" s="24" t="inlineStr">
         <is>
-          <t>Input. Hentast frå: Etter korrigering til driftsmessige verdiar.</t>
+          <t>Input. Hentast frå: 4090-4099, 4190-4199, 4290-4299, 4690-4699 (før korrigering).</t>
         </is>
       </c>
       <c r="F22" s="32" t="n"/>
@@ -41669,71 +41669,66 @@
     <row r="23">
       <c r="A23" s="20" t="inlineStr">
         <is>
+          <t>Beholdningsendring buskap/varelager, driftsmessig (+ = auke)</t>
+        </is>
+      </c>
+      <c r="B23" s="24" t="inlineStr">
+        <is>
+          <t>Etter korrigering til driftsmessige verdiar</t>
+        </is>
+      </c>
+      <c r="C23" s="31" t="n">
+        <v>3740</v>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E23" s="24" t="inlineStr">
+        <is>
+          <t>Input. Hentast frå: Etter korrigering til driftsmessige verdiar.</t>
+        </is>
+      </c>
+      <c r="F23" s="32" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="20" t="inlineStr">
+        <is>
           <t>Driftsoverskot jordbruk i rekneskapen (skatt)</t>
         </is>
       </c>
-      <c r="B23" s="24" t="inlineStr">
+      <c r="B24" s="24" t="inlineStr">
         <is>
           <t>Næringsoppgåve / resultatrekneskap</t>
         </is>
       </c>
-      <c r="C23" s="31" t="n">
+      <c r="C24" s="31" t="n">
         <v>403480.85</v>
       </c>
-      <c r="D23" s="12" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E23" s="24" t="inlineStr">
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E24" s="24" t="inlineStr">
         <is>
           <t>Input. Hentast frå: Næringsoppgåve / resultatrekneskap.</t>
         </is>
       </c>
-      <c r="F23" s="32" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="F24" s="32" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="inlineStr">
         <is>
           <t>5. UTREKNING – Frå skattemessig til driftsmessig resultat</t>
         </is>
       </c>
-      <c r="B24" s="19" t="n"/>
-      <c r="C24" s="19" t="n"/>
-      <c r="D24" s="19" t="n"/>
-      <c r="E24" s="19" t="n"/>
-      <c r="F24" s="19" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="20" t="inlineStr">
-        <is>
-          <t>Driftsmessige avskrivingar</t>
-        </is>
-      </c>
-      <c r="B25" s="21" t="inlineStr">
-        <is>
-          <t>Lenkje frå anna ark</t>
-        </is>
-      </c>
-      <c r="C25" s="13">
-        <f>'Faste kostnader'!C91</f>
-        <v/>
-      </c>
-      <c r="D25" s="12" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E25" s="23" t="inlineStr">
-        <is>
-          <t>Driftsmessige avskrivingar = – herav driftsmessige avskrivingar [Faste kostnader!C91]</t>
-        </is>
-      </c>
-      <c r="F25" s="24" t="inlineStr">
-        <is>
-          <t>='Faste kostnader'!C91</t>
-        </is>
-      </c>
+      <c r="B25" s="19" t="n"/>
+      <c r="C25" s="19" t="n"/>
+      <c r="D25" s="19" t="n"/>
+      <c r="E25" s="19" t="n"/>
+      <c r="F25" s="19" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="20" t="inlineStr">
@@ -41747,7 +41742,7 @@
         </is>
       </c>
       <c r="C26" s="22">
-        <f>C20-C25</f>
+        <f>C20-C21</f>
         <v/>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -41757,12 +41752,12 @@
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
-          <t>Korrigering avskrivingar (skatt – drift) = Skattemessige avskrivingar [C20] − Driftsmessige avskrivingar [C25]</t>
+          <t>Korrigering avskrivingar (skatt – drift) = Skattemessige avskrivingar [C20] − Driftsmessige avskrivingar [C21]</t>
         </is>
       </c>
       <c r="F26" s="24" t="inlineStr">
         <is>
-          <t>=C20-C25</t>
+          <t>=C20-C21</t>
         </is>
       </c>
     </row>
@@ -41778,7 +41773,7 @@
         </is>
       </c>
       <c r="C27" s="22">
-        <f>C22-C21</f>
+        <f>C23-C22</f>
         <v/>
       </c>
       <c r="D27" s="12" t="inlineStr">
@@ -41788,12 +41783,12 @@
       </c>
       <c r="E27" s="23" t="inlineStr">
         <is>
-          <t>Korrigering beholdningsendring (drift – skatt) = Beholdningsendring buskap/varelager, driftsmessig (+ = auke) [C22] − Beholdningsendring buskap/varelager, skattemessig (+ = auke) [C21]</t>
+          <t>Korrigering beholdningsendring (drift – skatt) = Beholdningsendring buskap/varelager, driftsmessig (+ = auke) [C23] − Beholdningsendring buskap/varelager, skattemessig (+ = auke) [C22]</t>
         </is>
       </c>
       <c r="F27" s="24" t="inlineStr">
         <is>
-          <t>=C22-C21</t>
+          <t>=C23-C22</t>
         </is>
       </c>
     </row>
@@ -41840,7 +41835,7 @@
         </is>
       </c>
       <c r="C29" s="22">
-        <f>C23-C28</f>
+        <f>C24-C28</f>
         <v/>
       </c>
       <c r="D29" s="12" t="inlineStr">
@@ -41850,12 +41845,12 @@
       </c>
       <c r="E29" s="23" t="inlineStr">
         <is>
-          <t>Avvik mot rekneskapen (bør vere 0) = Driftsoverskot jordbruk i rekneskapen (skatt) [C23] − Driftsoverskot skattemessig, berekna [C28]   (Avvik kjem av postar som ikkje er lagt inn i analysen. Eksempelanalysen har same avvik (−329,66))</t>
+          <t>Avvik mot rekneskapen (bør vere 0) = Driftsoverskot jordbruk i rekneskapen (skatt) [C24] − Driftsoverskot skattemessig, berekna [C28]   (Avvik kjem av postar som ikkje er lagt inn i analysen. Eksempelanalysen har same avvik (−329,66))</t>
         </is>
       </c>
       <c r="F29" s="24" t="inlineStr">
         <is>
-          <t>=C23-C28</t>
+          <t>=C24-C28</t>
         </is>
       </c>
     </row>
@@ -42128,7 +42123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F93"/>
+  <dimension ref="A1:F105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -43779,16 +43774,16 @@
     <row r="65">
       <c r="A65" s="20" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering – Mjølk</t>
+          <t>Kostnader til innandørsmekanisering (kontoar)</t>
         </is>
       </c>
       <c r="B65" s="24" t="inlineStr">
         <is>
-          <t>6030, 6541, 6563, 6640 (fordelt med nøkkel)</t>
+          <t>6030, 6541, 6563, 6640</t>
         </is>
       </c>
       <c r="C65" s="31" t="n">
-        <v>0</v>
+        <v>95725.21000000001</v>
       </c>
       <c r="D65" s="12" t="inlineStr">
         <is>
@@ -43797,7 +43792,7 @@
       </c>
       <c r="E65" s="24" t="inlineStr">
         <is>
-          <t>Input. Hentast frå: 6030, 6541, 6563, 6640 (fordelt med nøkkel). Herav-post: kostnadene ligg alt i bygnings- og andre faste kostnader, her blir dei berre fordelte</t>
+          <t>Input. Hentast frå: 6030, 6541, 6563, 6640. Herav-post: kontoane er kopla til «Innandørsmek.» i kontoplanen og ligg alt i bygnings- og andre faste kostnader</t>
         </is>
       </c>
       <c r="F65" s="32" t="n"/>
@@ -43805,25 +43800,25 @@
     <row r="66">
       <c r="A66" s="20" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering – Oksar</t>
+          <t>Del innandørsmekanisering – Mjølk</t>
         </is>
       </c>
       <c r="B66" s="24" t="inlineStr">
         <is>
-          <t>6030, 6541, 6563, 6640 (fordelt med nøkkel)</t>
-        </is>
-      </c>
-      <c r="C66" s="31" t="n">
+          <t>Fordelingsnøkkel (fôr innandørs)</t>
+        </is>
+      </c>
+      <c r="C66" s="34" t="n">
         <v>0</v>
       </c>
       <c r="D66" s="12" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E66" s="24" t="inlineStr">
         <is>
-          <t>Input. Hentast frå: 6030, 6541, 6563, 6640 (fordelt med nøkkel). Herav-post: kostnadene ligg alt i bygnings- og andre faste kostnader, her blir dei berre fordelte</t>
+          <t>Input. Hentast frå: Fordelingsnøkkel (fôr innandørs).</t>
         </is>
       </c>
       <c r="F66" s="32" t="n"/>
@@ -43831,25 +43826,25 @@
     <row r="67">
       <c r="A67" s="20" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering – Mellomkalv</t>
+          <t>Del innandørsmekanisering – Oksar</t>
         </is>
       </c>
       <c r="B67" s="24" t="inlineStr">
         <is>
-          <t>6030, 6541, 6563, 6640 (fordelt med nøkkel)</t>
-        </is>
-      </c>
-      <c r="C67" s="31" t="n">
+          <t>Fordelingsnøkkel (fôr innandørs)</t>
+        </is>
+      </c>
+      <c r="C67" s="34" t="n">
         <v>0</v>
       </c>
       <c r="D67" s="12" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E67" s="24" t="inlineStr">
         <is>
-          <t>Input. Hentast frå: 6030, 6541, 6563, 6640 (fordelt med nøkkel). Herav-post: kostnadene ligg alt i bygnings- og andre faste kostnader, her blir dei berre fordelte</t>
+          <t>Input. Hentast frå: Fordelingsnøkkel (fôr innandørs).</t>
         </is>
       </c>
       <c r="F67" s="32" t="n"/>
@@ -43857,25 +43852,25 @@
     <row r="68">
       <c r="A68" s="20" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering – Ammekyr</t>
+          <t>Del innandørsmekanisering – Mellomkalv</t>
         </is>
       </c>
       <c r="B68" s="24" t="inlineStr">
         <is>
-          <t>6030, 6541, 6563, 6640 (fordelt med nøkkel)</t>
-        </is>
-      </c>
-      <c r="C68" s="31" t="n">
-        <v>72685.58</v>
+          <t>Fordelingsnøkkel (fôr innandørs)</t>
+        </is>
+      </c>
+      <c r="C68" s="34" t="n">
+        <v>0</v>
       </c>
       <c r="D68" s="12" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E68" s="24" t="inlineStr">
         <is>
-          <t>Input. Hentast frå: 6030, 6541, 6563, 6640 (fordelt med nøkkel). Herav-post: kostnadene ligg alt i bygnings- og andre faste kostnader, her blir dei berre fordelte</t>
+          <t>Input. Hentast frå: Fordelingsnøkkel (fôr innandørs).</t>
         </is>
       </c>
       <c r="F68" s="32" t="n"/>
@@ -43883,25 +43878,25 @@
     <row r="69">
       <c r="A69" s="20" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering – Smågris</t>
+          <t>Del innandørsmekanisering – Ammekyr</t>
         </is>
       </c>
       <c r="B69" s="24" t="inlineStr">
         <is>
-          <t>6030, 6541, 6563, 6640 (fordelt med nøkkel)</t>
-        </is>
-      </c>
-      <c r="C69" s="31" t="n">
-        <v>0</v>
+          <t>Fordelingsnøkkel (fôr innandørs)</t>
+        </is>
+      </c>
+      <c r="C69" s="34" t="n">
+        <v>0.7593149181913521</v>
       </c>
       <c r="D69" s="12" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E69" s="24" t="inlineStr">
         <is>
-          <t>Input. Hentast frå: 6030, 6541, 6563, 6640 (fordelt med nøkkel). Herav-post: kostnadene ligg alt i bygnings- og andre faste kostnader, her blir dei berre fordelte</t>
+          <t>Input. Hentast frå: Fordelingsnøkkel (fôr innandørs).</t>
         </is>
       </c>
       <c r="F69" s="32" t="n"/>
@@ -43909,25 +43904,25 @@
     <row r="70">
       <c r="A70" s="20" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering – Purkering</t>
+          <t>Del innandørsmekanisering – Smågris</t>
         </is>
       </c>
       <c r="B70" s="24" t="inlineStr">
         <is>
-          <t>6030, 6541, 6563, 6640 (fordelt med nøkkel)</t>
-        </is>
-      </c>
-      <c r="C70" s="31" t="n">
+          <t>Fordelingsnøkkel (fôr innandørs)</t>
+        </is>
+      </c>
+      <c r="C70" s="34" t="n">
         <v>0</v>
       </c>
       <c r="D70" s="12" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E70" s="24" t="inlineStr">
         <is>
-          <t>Input. Hentast frå: 6030, 6541, 6563, 6640 (fordelt med nøkkel). Herav-post: kostnadene ligg alt i bygnings- og andre faste kostnader, her blir dei berre fordelte</t>
+          <t>Input. Hentast frå: Fordelingsnøkkel (fôr innandørs).</t>
         </is>
       </c>
       <c r="F70" s="32" t="n"/>
@@ -43935,25 +43930,25 @@
     <row r="71">
       <c r="A71" s="20" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering – Slaktegris</t>
+          <t>Del innandørsmekanisering – Purkering</t>
         </is>
       </c>
       <c r="B71" s="24" t="inlineStr">
         <is>
-          <t>6030, 6541, 6563, 6640 (fordelt med nøkkel)</t>
-        </is>
-      </c>
-      <c r="C71" s="31" t="n">
+          <t>Fordelingsnøkkel (fôr innandørs)</t>
+        </is>
+      </c>
+      <c r="C71" s="34" t="n">
         <v>0</v>
       </c>
       <c r="D71" s="12" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E71" s="24" t="inlineStr">
         <is>
-          <t>Input. Hentast frå: 6030, 6541, 6563, 6640 (fordelt med nøkkel). Herav-post: kostnadene ligg alt i bygnings- og andre faste kostnader, her blir dei berre fordelte</t>
+          <t>Input. Hentast frå: Fordelingsnøkkel (fôr innandørs).</t>
         </is>
       </c>
       <c r="F71" s="32" t="n"/>
@@ -43961,25 +43956,25 @@
     <row r="72">
       <c r="A72" s="20" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering – Sau</t>
+          <t>Del innandørsmekanisering – Slaktegris</t>
         </is>
       </c>
       <c r="B72" s="24" t="inlineStr">
         <is>
-          <t>6030, 6541, 6563, 6640 (fordelt med nøkkel)</t>
-        </is>
-      </c>
-      <c r="C72" s="31" t="n">
-        <v>23039.63</v>
+          <t>Fordelingsnøkkel (fôr innandørs)</t>
+        </is>
+      </c>
+      <c r="C72" s="34" t="n">
+        <v>0</v>
       </c>
       <c r="D72" s="12" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E72" s="24" t="inlineStr">
         <is>
-          <t>Input. Hentast frå: 6030, 6541, 6563, 6640 (fordelt med nøkkel). Herav-post: kostnadene ligg alt i bygnings- og andre faste kostnader, her blir dei berre fordelte</t>
+          <t>Input. Hentast frå: Fordelingsnøkkel (fôr innandørs).</t>
         </is>
       </c>
       <c r="F72" s="32" t="n"/>
@@ -43987,25 +43982,25 @@
     <row r="73">
       <c r="A73" s="20" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering – Geit</t>
+          <t>Del innandørsmekanisering – Sau</t>
         </is>
       </c>
       <c r="B73" s="24" t="inlineStr">
         <is>
-          <t>6030, 6541, 6563, 6640 (fordelt med nøkkel)</t>
-        </is>
-      </c>
-      <c r="C73" s="31" t="n">
-        <v>0</v>
+          <t>Fordelingsnøkkel (fôr innandørs)</t>
+        </is>
+      </c>
+      <c r="C73" s="34" t="n">
+        <v>0.2406850818086479</v>
       </c>
       <c r="D73" s="12" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E73" s="24" t="inlineStr">
         <is>
-          <t>Input. Hentast frå: 6030, 6541, 6563, 6640 (fordelt med nøkkel). Herav-post: kostnadene ligg alt i bygnings- og andre faste kostnader, her blir dei berre fordelte</t>
+          <t>Input. Hentast frå: Fordelingsnøkkel (fôr innandørs).</t>
         </is>
       </c>
       <c r="F73" s="32" t="n"/>
@@ -44013,25 +44008,25 @@
     <row r="74">
       <c r="A74" s="20" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering – Egg</t>
+          <t>Del innandørsmekanisering – Geit</t>
         </is>
       </c>
       <c r="B74" s="24" t="inlineStr">
         <is>
-          <t>6030, 6541, 6563, 6640 (fordelt med nøkkel)</t>
-        </is>
-      </c>
-      <c r="C74" s="31" t="n">
+          <t>Fordelingsnøkkel (fôr innandørs)</t>
+        </is>
+      </c>
+      <c r="C74" s="34" t="n">
         <v>0</v>
       </c>
       <c r="D74" s="12" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E74" s="24" t="inlineStr">
         <is>
-          <t>Input. Hentast frå: 6030, 6541, 6563, 6640 (fordelt med nøkkel). Herav-post: kostnadene ligg alt i bygnings- og andre faste kostnader, her blir dei berre fordelte</t>
+          <t>Input. Hentast frå: Fordelingsnøkkel (fôr innandørs).</t>
         </is>
       </c>
       <c r="F74" s="32" t="n"/>
@@ -44039,25 +44034,25 @@
     <row r="75">
       <c r="A75" s="20" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering – Slaktekylling</t>
+          <t>Del innandørsmekanisering – Egg</t>
         </is>
       </c>
       <c r="B75" s="24" t="inlineStr">
         <is>
-          <t>6030, 6541, 6563, 6640 (fordelt med nøkkel)</t>
-        </is>
-      </c>
-      <c r="C75" s="31" t="n">
+          <t>Fordelingsnøkkel (fôr innandørs)</t>
+        </is>
+      </c>
+      <c r="C75" s="34" t="n">
         <v>0</v>
       </c>
       <c r="D75" s="12" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E75" s="24" t="inlineStr">
         <is>
-          <t>Input. Hentast frå: 6030, 6541, 6563, 6640 (fordelt med nøkkel). Herav-post: kostnadene ligg alt i bygnings- og andre faste kostnader, her blir dei berre fordelte</t>
+          <t>Input. Hentast frå: Fordelingsnøkkel (fôr innandørs).</t>
         </is>
       </c>
       <c r="F75" s="32" t="n"/>
@@ -44065,306 +44060,374 @@
     <row r="76">
       <c r="A76" s="20" t="inlineStr">
         <is>
-          <t>Sum innandørsmekanisering (herav, inngår i summane ovanfor)</t>
-        </is>
-      </c>
-      <c r="B76" s="21" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C76" s="22">
-        <f>C65+C66+C67+C68+C69+C70+C71+C72+C73+C74+C75</f>
-        <v/>
+          <t>Del innandørsmekanisering – Slaktekylling</t>
+        </is>
+      </c>
+      <c r="B76" s="24" t="inlineStr">
+        <is>
+          <t>Fordelingsnøkkel (fôr innandørs)</t>
+        </is>
+      </c>
+      <c r="C76" s="34" t="n">
+        <v>0</v>
       </c>
       <c r="D76" s="12" t="inlineStr">
         <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E76" s="23" t="inlineStr">
-        <is>
-          <t>Sum innandørsmekanisering (herav, inngår i summane ovanfor) = Innandørsmekanisering – Mjølk [C65] + Innandørsmekanisering – Oksar [C66] + Innandørsmekanisering – Mellomkalv [C67] + Innandørsmekanisering – Ammekyr [C68] + Innandørsmekanisering – Smågris [C69] + Innandørsmekanisering – Purkering [C70] + Innandørsmekanisering – Slaktegris [C71] + Innandørsmekanisering – Sau [C72] + Innandørsmekanisering – Geit [C73] + Innandørsmekanisering – Egg [C74] + Innandørsmekanisering – Slaktekylling [C75]</t>
-        </is>
-      </c>
-      <c r="F76" s="24" t="inlineStr">
-        <is>
-          <t>=C65+C66+C67+C68+C69+C70+C71+C72+C73+C74+C75</t>
-        </is>
-      </c>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E76" s="24" t="inlineStr">
+        <is>
+          <t>Input. Hentast frå: Fordelingsnøkkel (fôr innandørs).</t>
+        </is>
+      </c>
+      <c r="F76" s="32" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="18" t="inlineStr">
-        <is>
-          <t>6. INPUT – Andre faste kostnader</t>
-        </is>
-      </c>
-      <c r="B77" s="19" t="n"/>
-      <c r="C77" s="19" t="n"/>
-      <c r="D77" s="19" t="n"/>
-      <c r="E77" s="19" t="n"/>
-      <c r="F77" s="19" t="n"/>
+      <c r="A77" s="20" t="inlineStr">
+        <is>
+          <t>Innandørsmekanisering – Mjølk</t>
+        </is>
+      </c>
+      <c r="B77" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C77" s="22">
+        <f>C65*C66</f>
+        <v/>
+      </c>
+      <c r="D77" s="12" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E77" s="23" t="inlineStr">
+        <is>
+          <t>Innandørsmekanisering – Mjølk = Kostnader til innandørsmekanisering (kontoar) [C65] × Del innandørsmekanisering – Mjølk [C66]</t>
+        </is>
+      </c>
+      <c r="F77" s="24" t="inlineStr">
+        <is>
+          <t>=C65*C66</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="20" t="inlineStr">
         <is>
-          <t>Leigd hjelp / løn / avløysar</t>
-        </is>
-      </c>
-      <c r="B78" s="24" t="inlineStr">
-        <is>
-          <t>4570-4580, 5000-5599, 5700-5999, !5800-5899</t>
-        </is>
-      </c>
-      <c r="C78" s="31" t="n">
-        <v>78672.8</v>
+          <t>Innandørsmekanisering – Oksar</t>
+        </is>
+      </c>
+      <c r="B78" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C78" s="22">
+        <f>C65*C67</f>
+        <v/>
       </c>
       <c r="D78" s="12" t="inlineStr">
         <is>
           <t>kr</t>
         </is>
       </c>
-      <c r="E78" s="24" t="inlineStr">
-        <is>
-          <t>Input. Hentast frå: 4570-4580, 5000-5599, 5700-5999, !5800-5899.</t>
-        </is>
-      </c>
-      <c r="F78" s="32" t="n"/>
+      <c r="E78" s="23" t="inlineStr">
+        <is>
+          <t>Innandørsmekanisering – Oksar = Kostnader til innandørsmekanisering (kontoar) [C65] × Del innandørsmekanisering – Oksar [C67]</t>
+        </is>
+      </c>
+      <c r="F78" s="24" t="inlineStr">
+        <is>
+          <t>=C65*C67</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="20" t="inlineStr">
         <is>
-          <t>Arbeidsvederlag i selskap</t>
-        </is>
-      </c>
-      <c r="B79" s="24" t="inlineStr">
-        <is>
-          <t>5600-5699</t>
-        </is>
-      </c>
-      <c r="C79" s="31" t="n">
-        <v>0</v>
+          <t>Innandørsmekanisering – Mellomkalv</t>
+        </is>
+      </c>
+      <c r="B79" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C79" s="22">
+        <f>C65*C68</f>
+        <v/>
       </c>
       <c r="D79" s="12" t="inlineStr">
         <is>
           <t>kr</t>
         </is>
       </c>
-      <c r="E79" s="24" t="inlineStr">
-        <is>
-          <t>Input. Hentast frå: 5600-5699.</t>
-        </is>
-      </c>
-      <c r="F79" s="32" t="n"/>
+      <c r="E79" s="23" t="inlineStr">
+        <is>
+          <t>Innandørsmekanisering – Mellomkalv = Kostnader til innandørsmekanisering (kontoar) [C65] × Del innandørsmekanisering – Mellomkalv [C68]</t>
+        </is>
+      </c>
+      <c r="F79" s="24" t="inlineStr">
+        <is>
+          <t>=C65*C68</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="20" t="inlineStr">
         <is>
-          <t>Refusjon avløysar / sjukdom (-)</t>
-        </is>
-      </c>
-      <c r="B80" s="24" t="inlineStr">
-        <is>
-          <t>3440-3442, 5800-5899</t>
-        </is>
-      </c>
-      <c r="C80" s="31" t="n">
-        <v>-62681</v>
+          <t>Innandørsmekanisering – Ammekyr</t>
+        </is>
+      </c>
+      <c r="B80" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C80" s="22">
+        <f>C65*C69</f>
+        <v/>
       </c>
       <c r="D80" s="12" t="inlineStr">
         <is>
           <t>kr</t>
         </is>
       </c>
-      <c r="E80" s="24" t="inlineStr">
-        <is>
-          <t>Input. Hentast frå: 3440-3442, 5800-5899.</t>
-        </is>
-      </c>
-      <c r="F80" s="32" t="n"/>
+      <c r="E80" s="23" t="inlineStr">
+        <is>
+          <t>Innandørsmekanisering – Ammekyr = Kostnader til innandørsmekanisering (kontoar) [C65] × Del innandørsmekanisering – Ammekyr [C69]</t>
+        </is>
+      </c>
+      <c r="F80" s="24" t="inlineStr">
+        <is>
+          <t>=C65*C69</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="20" t="inlineStr">
         <is>
-          <t>Leige av jord, beite og mjølkekvote</t>
-        </is>
-      </c>
-      <c r="B81" s="24" t="inlineStr">
-        <is>
-          <t>6471, 6472, 6475</t>
-        </is>
-      </c>
-      <c r="C81" s="31" t="n">
-        <v>0</v>
+          <t>Innandørsmekanisering – Smågris</t>
+        </is>
+      </c>
+      <c r="B81" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C81" s="22">
+        <f>C65*C70</f>
+        <v/>
       </c>
       <c r="D81" s="12" t="inlineStr">
         <is>
           <t>kr</t>
         </is>
       </c>
-      <c r="E81" s="24" t="inlineStr">
-        <is>
-          <t>Input. Hentast frå: 6471, 6472, 6475.</t>
-        </is>
-      </c>
-      <c r="F81" s="32" t="n"/>
+      <c r="E81" s="23" t="inlineStr">
+        <is>
+          <t>Innandørsmekanisering – Smågris = Kostnader til innandørsmekanisering (kontoar) [C65] × Del innandørsmekanisering – Smågris [C70]</t>
+        </is>
+      </c>
+      <c r="F81" s="24" t="inlineStr">
+        <is>
+          <t>=C65*C70</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="20" t="inlineStr">
         <is>
-          <t>Vedlikehald jord, vegar, grøfter og anna</t>
-        </is>
-      </c>
-      <c r="B82" s="24" t="inlineStr">
-        <is>
-          <t>6650-6699</t>
-        </is>
-      </c>
-      <c r="C82" s="31" t="n">
-        <v>5000</v>
+          <t>Innandørsmekanisering – Purkering</t>
+        </is>
+      </c>
+      <c r="B82" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C82" s="22">
+        <f>C65*C71</f>
+        <v/>
       </c>
       <c r="D82" s="12" t="inlineStr">
         <is>
           <t>kr</t>
         </is>
       </c>
-      <c r="E82" s="24" t="inlineStr">
-        <is>
-          <t>Input. Hentast frå: 6650-6699.</t>
-        </is>
-      </c>
-      <c r="F82" s="32" t="n"/>
+      <c r="E82" s="23" t="inlineStr">
+        <is>
+          <t>Innandørsmekanisering – Purkering = Kostnader til innandørsmekanisering (kontoar) [C65] × Del innandørsmekanisering – Purkering [C71]</t>
+        </is>
+      </c>
+      <c r="F82" s="24" t="inlineStr">
+        <is>
+          <t>=C65*C71</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="20" t="inlineStr">
         <is>
-          <t>Energi (straum, brensel) som ikkje er fordelt</t>
-        </is>
-      </c>
-      <c r="B83" s="24" t="inlineStr">
-        <is>
-          <t>6200-6249</t>
-        </is>
-      </c>
-      <c r="C83" s="31" t="n">
-        <v>23734.87</v>
+          <t>Innandørsmekanisering – Slaktegris</t>
+        </is>
+      </c>
+      <c r="B83" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C83" s="22">
+        <f>C65*C72</f>
+        <v/>
       </c>
       <c r="D83" s="12" t="inlineStr">
         <is>
           <t>kr</t>
         </is>
       </c>
-      <c r="E83" s="24" t="inlineStr">
-        <is>
-          <t>Input. Hentast frå: 6200-6249.</t>
-        </is>
-      </c>
-      <c r="F83" s="32" t="n"/>
+      <c r="E83" s="23" t="inlineStr">
+        <is>
+          <t>Innandørsmekanisering – Slaktegris = Kostnader til innandørsmekanisering (kontoar) [C65] × Del innandørsmekanisering – Slaktegris [C72]</t>
+        </is>
+      </c>
+      <c r="F83" s="24" t="inlineStr">
+        <is>
+          <t>=C65*C72</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="20" t="inlineStr">
         <is>
-          <t>Administrasjon (rekneskap, kontor, telefon, kontingentar, forsikring)</t>
-        </is>
-      </c>
-      <c r="B84" s="24" t="inlineStr">
-        <is>
-          <t>6700-6999, 7100-7499, 7500, 7502, 7509, 7600-7799</t>
-        </is>
-      </c>
-      <c r="C84" s="31" t="n">
-        <v>156309.53</v>
+          <t>Innandørsmekanisering – Sau</t>
+        </is>
+      </c>
+      <c r="B84" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C84" s="22">
+        <f>C65*C73</f>
+        <v/>
       </c>
       <c r="D84" s="12" t="inlineStr">
         <is>
           <t>kr</t>
         </is>
       </c>
-      <c r="E84" s="24" t="inlineStr">
-        <is>
-          <t>Input. Hentast frå: 6700-6999, 7100-7499, 7500, 7502, 7509, 7600-7799.</t>
-        </is>
-      </c>
-      <c r="F84" s="32" t="n"/>
+      <c r="E84" s="23" t="inlineStr">
+        <is>
+          <t>Innandørsmekanisering – Sau = Kostnader til innandørsmekanisering (kontoar) [C65] × Del innandørsmekanisering – Sau [C73]</t>
+        </is>
+      </c>
+      <c r="F84" s="24" t="inlineStr">
+        <is>
+          <t>=C65*C73</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="20" t="inlineStr">
         <is>
-          <t>Bil og transportmiddel</t>
-        </is>
-      </c>
-      <c r="B85" s="24" t="inlineStr">
-        <is>
-          <t>6011-6014, 7000-7099</t>
-        </is>
-      </c>
-      <c r="C85" s="31" t="n">
-        <v>0</v>
+          <t>Innandørsmekanisering – Geit</t>
+        </is>
+      </c>
+      <c r="B85" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C85" s="22">
+        <f>C65*C74</f>
+        <v/>
       </c>
       <c r="D85" s="12" t="inlineStr">
         <is>
           <t>kr</t>
         </is>
       </c>
-      <c r="E85" s="24" t="inlineStr">
-        <is>
-          <t>Input. Hentast frå: 6011-6014, 7000-7099.</t>
-        </is>
-      </c>
-      <c r="F85" s="32" t="n"/>
+      <c r="E85" s="23" t="inlineStr">
+        <is>
+          <t>Innandørsmekanisering – Geit = Kostnader til innandørsmekanisering (kontoar) [C65] × Del innandørsmekanisering – Geit [C74]</t>
+        </is>
+      </c>
+      <c r="F85" s="24" t="inlineStr">
+        <is>
+          <t>=C65*C74</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="20" t="inlineStr">
         <is>
-          <t>Andre avskrivingar (driftsmessige)</t>
-        </is>
-      </c>
-      <c r="B86" s="24" t="inlineStr">
-        <is>
-          <t>6015-6019</t>
-        </is>
-      </c>
-      <c r="C86" s="31" t="n">
-        <v>0</v>
+          <t>Innandørsmekanisering – Egg</t>
+        </is>
+      </c>
+      <c r="B86" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C86" s="22">
+        <f>C65*C75</f>
+        <v/>
       </c>
       <c r="D86" s="12" t="inlineStr">
         <is>
           <t>kr</t>
         </is>
       </c>
-      <c r="E86" s="24" t="inlineStr">
-        <is>
-          <t>Input. Hentast frå: 6015-6019.</t>
-        </is>
-      </c>
-      <c r="F86" s="32" t="n"/>
+      <c r="E86" s="23" t="inlineStr">
+        <is>
+          <t>Innandørsmekanisering – Egg = Kostnader til innandørsmekanisering (kontoar) [C65] × Del innandørsmekanisering – Egg [C75]</t>
+        </is>
+      </c>
+      <c r="F86" s="24" t="inlineStr">
+        <is>
+          <t>=C65*C75</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="20" t="inlineStr">
         <is>
-          <t>Annan fast kostnad (resten av 5000–7999)</t>
-        </is>
-      </c>
-      <c r="B87" s="24" t="inlineStr"/>
-      <c r="C87" s="31" t="n">
-        <v>66370.83</v>
+          <t>Innandørsmekanisering – Slaktekylling</t>
+        </is>
+      </c>
+      <c r="B87" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C87" s="22">
+        <f>C65*C76</f>
+        <v/>
       </c>
       <c r="D87" s="12" t="inlineStr">
         <is>
           <t>kr</t>
         </is>
       </c>
-      <c r="E87" s="24" t="inlineStr">
-        <is>
-          <t>Input.</t>
-        </is>
-      </c>
-      <c r="F87" s="32" t="n"/>
+      <c r="E87" s="23" t="inlineStr">
+        <is>
+          <t>Innandørsmekanisering – Slaktekylling = Kostnader til innandørsmekanisering (kontoar) [C65] × Del innandørsmekanisering – Slaktekylling [C76]</t>
+        </is>
+      </c>
+      <c r="F87" s="24" t="inlineStr">
+        <is>
+          <t>=C65*C76</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="20" t="inlineStr">
         <is>
-          <t>Sum andre faste kostnader</t>
+          <t>Sum innandørsmekanisering (herav, inngår i summane ovanfor)</t>
         </is>
       </c>
       <c r="B88" s="21" t="inlineStr">
@@ -44373,7 +44436,7 @@
         </is>
       </c>
       <c r="C88" s="22">
-        <f>C78+C79+C80+C81+C82+C83+C84+C85+C86+C87</f>
+        <f>C77+C78+C79+C80+C81+C82+C83+C84+C85+C86+C87</f>
         <v/>
       </c>
       <c r="D88" s="12" t="inlineStr">
@@ -44383,19 +44446,19 @@
       </c>
       <c r="E88" s="23" t="inlineStr">
         <is>
-          <t>Sum andre faste kostnader = Leigd hjelp / løn / avløysar [C78] + Arbeidsvederlag i selskap [C79] + Refusjon avløysar / sjukdom (-) [C80] + Leige av jord, beite og mjølkekvote [C81] + Vedlikehald jord, vegar, grøfter og anna [C82] + Energi (straum, brensel) som ikkje er fordelt [C83] + Administrasjon (rekneskap, kontor, telefon, kontingentar, forsikring) [C84] + Bil og transportmiddel [C85] + Andre avskrivingar (driftsmessige) [C86] + Annan fast kostnad (resten av 5000–7999) [C87]</t>
+          <t>Sum innandørsmekanisering (herav, inngår i summane ovanfor) = Innandørsmekanisering – Mjølk [C77] + Innandørsmekanisering – Oksar [C78] + Innandørsmekanisering – Mellomkalv [C79] + Innandørsmekanisering – Ammekyr [C80] + Innandørsmekanisering – Smågris [C81] + Innandørsmekanisering – Purkering [C82] + Innandørsmekanisering – Slaktegris [C83] + Innandørsmekanisering – Sau [C84] + Innandørsmekanisering – Geit [C85] + Innandørsmekanisering – Egg [C86] + Innandørsmekanisering – Slaktekylling [C87]</t>
         </is>
       </c>
       <c r="F88" s="24" t="inlineStr">
         <is>
-          <t>=C78+C79+C80+C81+C82+C83+C84+C85+C86+C87</t>
+          <t>=C77+C78+C79+C80+C81+C82+C83+C84+C85+C86+C87</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="18" t="inlineStr">
         <is>
-          <t>7. OUTPUT – Sum faste kostnader</t>
+          <t>6. INPUT – Andre faste kostnader</t>
         </is>
       </c>
       <c r="B89" s="19" t="n"/>
@@ -44405,126 +44468,425 @@
       <c r="F89" s="19" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="25" t="inlineStr">
-        <is>
-          <t>Sum faste kostnader jordbruk</t>
-        </is>
-      </c>
-      <c r="B90" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C90" s="27">
-        <f>C13+C63+C88</f>
-        <v/>
-      </c>
-      <c r="D90" s="28" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E90" s="29" t="inlineStr">
-        <is>
-          <t>Sum faste kostnader jordbruk = Sum maskinkostnader [C13] + Sum bygningskostnader [C63] + Sum andre faste kostnader [C88]   (Innandørsmekanisering er ein herav-post og blir ikkje lagd til (same som eksempelanalysen))</t>
-        </is>
-      </c>
-      <c r="F90" s="30" t="inlineStr">
-        <is>
-          <t>=C13+C63+C88</t>
-        </is>
-      </c>
+      <c r="A90" s="20" t="inlineStr">
+        <is>
+          <t>Leigd hjelp / løn / avløysar</t>
+        </is>
+      </c>
+      <c r="B90" s="24" t="inlineStr">
+        <is>
+          <t>4570-4580, 5000-5599, 5700-5999, !5800-5899</t>
+        </is>
+      </c>
+      <c r="C90" s="31" t="n">
+        <v>78672.8</v>
+      </c>
+      <c r="D90" s="12" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E90" s="24" t="inlineStr">
+        <is>
+          <t>Input. Hentast frå: 4570-4580, 5000-5599, 5700-5999, !5800-5899.</t>
+        </is>
+      </c>
+      <c r="F90" s="32" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="20" t="inlineStr">
         <is>
+          <t>Arbeidsvederlag i selskap</t>
+        </is>
+      </c>
+      <c r="B91" s="24" t="inlineStr">
+        <is>
+          <t>5600-5699</t>
+        </is>
+      </c>
+      <c r="C91" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D91" s="12" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E91" s="24" t="inlineStr">
+        <is>
+          <t>Input. Hentast frå: 5600-5699.</t>
+        </is>
+      </c>
+      <c r="F91" s="32" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="20" t="inlineStr">
+        <is>
+          <t>Refusjon avløysar / sjukdom (-)</t>
+        </is>
+      </c>
+      <c r="B92" s="24" t="inlineStr">
+        <is>
+          <t>3440-3442, 5800-5899</t>
+        </is>
+      </c>
+      <c r="C92" s="31" t="n">
+        <v>-62681</v>
+      </c>
+      <c r="D92" s="12" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E92" s="24" t="inlineStr">
+        <is>
+          <t>Input. Hentast frå: 3440-3442, 5800-5899.</t>
+        </is>
+      </c>
+      <c r="F92" s="32" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="20" t="inlineStr">
+        <is>
+          <t>Leige av jord, beite og mjølkekvote</t>
+        </is>
+      </c>
+      <c r="B93" s="24" t="inlineStr">
+        <is>
+          <t>6471, 6472, 6475</t>
+        </is>
+      </c>
+      <c r="C93" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D93" s="12" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E93" s="24" t="inlineStr">
+        <is>
+          <t>Input. Hentast frå: 6471, 6472, 6475.</t>
+        </is>
+      </c>
+      <c r="F93" s="32" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="20" t="inlineStr">
+        <is>
+          <t>Vedlikehald jord, vegar, grøfter og anna</t>
+        </is>
+      </c>
+      <c r="B94" s="24" t="inlineStr">
+        <is>
+          <t>6650-6699</t>
+        </is>
+      </c>
+      <c r="C94" s="31" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D94" s="12" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E94" s="24" t="inlineStr">
+        <is>
+          <t>Input. Hentast frå: 6650-6699.</t>
+        </is>
+      </c>
+      <c r="F94" s="32" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="20" t="inlineStr">
+        <is>
+          <t>Energi (straum, brensel) som ikkje er fordelt</t>
+        </is>
+      </c>
+      <c r="B95" s="24" t="inlineStr">
+        <is>
+          <t>6200-6249</t>
+        </is>
+      </c>
+      <c r="C95" s="31" t="n">
+        <v>23734.87</v>
+      </c>
+      <c r="D95" s="12" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E95" s="24" t="inlineStr">
+        <is>
+          <t>Input. Hentast frå: 6200-6249.</t>
+        </is>
+      </c>
+      <c r="F95" s="32" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="20" t="inlineStr">
+        <is>
+          <t>Administrasjon (rekneskap, kontor, telefon, kontingentar, forsikring)</t>
+        </is>
+      </c>
+      <c r="B96" s="24" t="inlineStr">
+        <is>
+          <t>6700-6999, 7100-7499, 7500, 7502, 7509, 7600-7799</t>
+        </is>
+      </c>
+      <c r="C96" s="31" t="n">
+        <v>156309.53</v>
+      </c>
+      <c r="D96" s="12" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E96" s="24" t="inlineStr">
+        <is>
+          <t>Input. Hentast frå: 6700-6999, 7100-7499, 7500, 7502, 7509, 7600-7799.</t>
+        </is>
+      </c>
+      <c r="F96" s="32" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="20" t="inlineStr">
+        <is>
+          <t>Bil og transportmiddel</t>
+        </is>
+      </c>
+      <c r="B97" s="24" t="inlineStr">
+        <is>
+          <t>6011-6014, 7000-7099</t>
+        </is>
+      </c>
+      <c r="C97" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D97" s="12" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E97" s="24" t="inlineStr">
+        <is>
+          <t>Input. Hentast frå: 6011-6014, 7000-7099.</t>
+        </is>
+      </c>
+      <c r="F97" s="32" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="20" t="inlineStr">
+        <is>
+          <t>Andre avskrivingar (driftsmessige)</t>
+        </is>
+      </c>
+      <c r="B98" s="24" t="inlineStr">
+        <is>
+          <t>6015-6019</t>
+        </is>
+      </c>
+      <c r="C98" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D98" s="12" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E98" s="24" t="inlineStr">
+        <is>
+          <t>Input. Hentast frå: 6015-6019.</t>
+        </is>
+      </c>
+      <c r="F98" s="32" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="20" t="inlineStr">
+        <is>
+          <t>Annan fast kostnad (resten av 5000–7999)</t>
+        </is>
+      </c>
+      <c r="B99" s="24" t="inlineStr"/>
+      <c r="C99" s="31" t="n">
+        <v>66370.83</v>
+      </c>
+      <c r="D99" s="12" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E99" s="24" t="inlineStr">
+        <is>
+          <t>Input.</t>
+        </is>
+      </c>
+      <c r="F99" s="32" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="20" t="inlineStr">
+        <is>
+          <t>Sum andre faste kostnader</t>
+        </is>
+      </c>
+      <c r="B100" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C100" s="22">
+        <f>C90+C91+C92+C93+C94+C95+C96+C97+C98+C99</f>
+        <v/>
+      </c>
+      <c r="D100" s="12" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E100" s="23" t="inlineStr">
+        <is>
+          <t>Sum andre faste kostnader = Leigd hjelp / løn / avløysar [C90] + Arbeidsvederlag i selskap [C91] + Refusjon avløysar / sjukdom (-) [C92] + Leige av jord, beite og mjølkekvote [C93] + Vedlikehald jord, vegar, grøfter og anna [C94] + Energi (straum, brensel) som ikkje er fordelt [C95] + Administrasjon (rekneskap, kontor, telefon, kontingentar, forsikring) [C96] + Bil og transportmiddel [C97] + Andre avskrivingar (driftsmessige) [C98] + Annan fast kostnad (resten av 5000–7999) [C99]</t>
+        </is>
+      </c>
+      <c r="F100" s="24" t="inlineStr">
+        <is>
+          <t>=C90+C91+C92+C93+C94+C95+C96+C97+C98+C99</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="18" t="inlineStr">
+        <is>
+          <t>7. OUTPUT – Sum faste kostnader</t>
+        </is>
+      </c>
+      <c r="B101" s="19" t="n"/>
+      <c r="C101" s="19" t="n"/>
+      <c r="D101" s="19" t="n"/>
+      <c r="E101" s="19" t="n"/>
+      <c r="F101" s="19" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="25" t="inlineStr">
+        <is>
+          <t>Sum faste kostnader jordbruk</t>
+        </is>
+      </c>
+      <c r="B102" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C102" s="27">
+        <f>C13+C63+C100</f>
+        <v/>
+      </c>
+      <c r="D102" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E102" s="29" t="inlineStr">
+        <is>
+          <t>Sum faste kostnader jordbruk = Sum maskinkostnader [C13] + Sum bygningskostnader [C63] + Sum andre faste kostnader [C100]   (Innandørsmekanisering er ein herav-post og blir ikkje lagd til (same som eksempelanalysen))</t>
+        </is>
+      </c>
+      <c r="F102" s="30" t="inlineStr">
+        <is>
+          <t>=C13+C63+C100</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="20" t="inlineStr">
+        <is>
           <t>– herav driftsmessige avskrivingar</t>
         </is>
       </c>
-      <c r="B91" s="21" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C91" s="22">
-        <f>C11+C60+C86</f>
-        <v/>
-      </c>
-      <c r="D91" s="12" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E91" s="23" t="inlineStr">
-        <is>
-          <t>– herav driftsmessige avskrivingar = Avskrivingar maskiner og reiskap (driftsmessige) [C11] + Avskrivingar bygningar og anlegg (driftsmessige) [C60] + Andre avskrivingar (driftsmessige) [C86]</t>
-        </is>
-      </c>
-      <c r="F91" s="24" t="inlineStr">
-        <is>
-          <t>=C11+C60+C86</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="25" t="inlineStr">
+      <c r="B103" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C103" s="22">
+        <f>C11+C60+C98</f>
+        <v/>
+      </c>
+      <c r="D103" s="12" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E103" s="23" t="inlineStr">
+        <is>
+          <t>– herav driftsmessige avskrivingar = Avskrivingar maskiner og reiskap (driftsmessige) [C11] + Avskrivingar bygningar og anlegg (driftsmessige) [C60] + Andre avskrivingar (driftsmessige) [C98]</t>
+        </is>
+      </c>
+      <c r="F103" s="24" t="inlineStr">
+        <is>
+          <t>=C11+C60+C98</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="25" t="inlineStr">
         <is>
           <t>Maskinkostnader i % av faste kostnader</t>
         </is>
       </c>
-      <c r="B92" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C92" s="33">
-        <f>IF((C90)=0,0,(C13)/(C90))</f>
-        <v/>
-      </c>
-      <c r="D92" s="28" t="inlineStr">
+      <c r="B104" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C104" s="33">
+        <f>IF((C102)=0,0,(C13)/(C102))</f>
+        <v/>
+      </c>
+      <c r="D104" s="28" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E92" s="29" t="inlineStr">
-        <is>
-          <t>Maskinkostnader i % av faste kostnader = Sum maskinkostnader [C13] ÷ Sum faste kostnader jordbruk [C90]</t>
-        </is>
-      </c>
-      <c r="F92" s="30" t="inlineStr">
-        <is>
-          <t>=IF((C90)=0,0,(C13)/(C90))</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="25" t="inlineStr">
+      <c r="E104" s="29" t="inlineStr">
+        <is>
+          <t>Maskinkostnader i % av faste kostnader = Sum maskinkostnader [C13] ÷ Sum faste kostnader jordbruk [C102]</t>
+        </is>
+      </c>
+      <c r="F104" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C102)=0,0,(C13)/(C102))</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="25" t="inlineStr">
         <is>
           <t>Bygningskostnader i % av faste kostnader</t>
         </is>
       </c>
-      <c r="B93" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C93" s="33">
-        <f>IF((C90)=0,0,(C63)/(C90))</f>
-        <v/>
-      </c>
-      <c r="D93" s="28" t="inlineStr">
+      <c r="B105" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C105" s="33">
+        <f>IF((C102)=0,0,(C63)/(C102))</f>
+        <v/>
+      </c>
+      <c r="D105" s="28" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E93" s="29" t="inlineStr">
-        <is>
-          <t>Bygningskostnader i % av faste kostnader = Sum bygningskostnader [C63] ÷ Sum faste kostnader jordbruk [C90]</t>
-        </is>
-      </c>
-      <c r="F93" s="30" t="inlineStr">
-        <is>
-          <t>=IF((C90)=0,0,(C63)/(C90))</t>
+      <c r="E105" s="29" t="inlineStr">
+        <is>
+          <t>Bygningskostnader i % av faste kostnader = Sum bygningskostnader [C63] ÷ Sum faste kostnader jordbruk [C102]</t>
+        </is>
+      </c>
+      <c r="F105" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C102)=0,0,(C63)/(C102))</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rapport etter gullstandard-oppsett, færre sider; nye beregninger
- PDF: Totaløkonomi (fra skattemessig til nettoinntekt, fjorår/i år, graf og
  korrigeringsbokser), Dekningsbidrag, Areal og grovfôr, Faste kostnader,
  produksjoner. Store produksjoner får egen side med nøkkeltall, graf,
  kommentar og DB per enhet; små blir kompakte og deler side. Vedlegg samlet.
- Nye beregninger: driftsresultat skog/pelsdyr (avd. 30/50) skilt fra annen
  næring, kueiningar storfe/småfe, korrigert areal per del (kulturbeite ÷2,5/÷10),
  utmarksbeite storfe/småfe, korrigerte dekar per kueining i produksjonen

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HrtCx2hBap2TXaC318T6kC
</commit_message>
<xml_diff>
--- a/excel/Analyse_jordbruk_produksjonar.xlsx
+++ b/excel/Analyse_jordbruk_produksjonar.xlsx
@@ -7920,7 +7920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F103"/>
+  <dimension ref="A1:F104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -10211,7 +10211,7 @@
         </is>
       </c>
       <c r="C90" s="39">
-        <f>IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C53)/('Grovfôr'!C38)))=0,0,(C56)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C53)/('Grovfôr'!C38))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C53)/('Grovfôr'!C46)))=0,0,(C56)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C53)/('Grovfôr'!C46))))</f>
         <v/>
       </c>
       <c r="D90" s="28" t="inlineStr">
@@ -10221,12 +10221,12 @@
       </c>
       <c r="E90" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C56] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C21] × Sum eigen grovfôrproduksjon (utan lagerendring) [C53] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C38])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
+          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C56] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C53] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
         </is>
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C53)/('Grovfôr'!C38)))=0,0,(C56)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C53)/('Grovfôr'!C38))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C53)/('Grovfôr'!C46)))=0,0,(C56)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C53)/('Grovfôr'!C46))))</t>
         </is>
       </c>
     </row>
@@ -10242,7 +10242,7 @@
         </is>
       </c>
       <c r="C91" s="39">
-        <f>IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C53)/('Grovfôr'!C38)))=0,0,(C57)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C53)/('Grovfôr'!C38))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C53)/('Grovfôr'!C46)))=0,0,(C57)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C53)/('Grovfôr'!C46))))</f>
         <v/>
       </c>
       <c r="D91" s="28" t="inlineStr">
@@ -10252,12 +10252,12 @@
       </c>
       <c r="E91" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C57] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C21] × Sum eigen grovfôrproduksjon (utan lagerendring) [C53] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C38])</t>
+          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C57] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C53] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])</t>
         </is>
       </c>
       <c r="F91" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C53)/('Grovfôr'!C38)))=0,0,(C57)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C53)/('Grovfôr'!C38))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C53)/('Grovfôr'!C46)))=0,0,(C57)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C53)/('Grovfôr'!C46))))</t>
         </is>
       </c>
     </row>
@@ -10273,7 +10273,7 @@
         </is>
       </c>
       <c r="C92" s="40">
-        <f>'Grovfôr'!C52</f>
+        <f>'Grovfôr'!C60</f>
         <v/>
       </c>
       <c r="D92" s="28" t="inlineStr">
@@ -10283,12 +10283,12 @@
       </c>
       <c r="E92" s="29" t="inlineStr">
         <is>
-          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C52]</t>
+          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C60]</t>
         </is>
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C52</t>
+          <t>='Grovfôr'!C60</t>
         </is>
       </c>
     </row>
@@ -10304,7 +10304,7 @@
         </is>
       </c>
       <c r="C93" s="40">
-        <f>'Grovfôr'!C53</f>
+        <f>'Grovfôr'!C61</f>
         <v/>
       </c>
       <c r="D93" s="28" t="inlineStr">
@@ -10314,19 +10314,19 @@
       </c>
       <c r="E93" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C53]</t>
+          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C61]</t>
         </is>
       </c>
       <c r="F93" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C53</t>
+          <t>='Grovfôr'!C61</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="25" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining»</t>
+          <t>Korrigerte dekar pr «kueining» (heile garden)</t>
         </is>
       </c>
       <c r="B94" s="26" t="inlineStr">
@@ -10335,7 +10335,7 @@
         </is>
       </c>
       <c r="C94" s="40">
-        <f>'Grovfôr'!C54</f>
+        <f>'Grovfôr'!C62</f>
         <v/>
       </c>
       <c r="D94" s="28" t="inlineStr">
@@ -10345,19 +10345,19 @@
       </c>
       <c r="E94" s="29" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining» = Korrigerte dekar pr «kueining» [Grovfôr!C54]</t>
+          <t>Korrigerte dekar pr «kueining» (heile garden) = Korrigerte dekar pr «kueining» [Grovfôr!C62]</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C54</t>
+          <t>='Grovfôr'!C62</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="25" t="inlineStr">
         <is>
-          <t>Oppnådd mjølkepris pr liter (u/distriktstilskot)</t>
+          <t>Korrigerte dekar pr «kueining» i produksjonen</t>
         </is>
       </c>
       <c r="B95" s="26" t="inlineStr">
@@ -10366,29 +10366,29 @@
         </is>
       </c>
       <c r="C95" s="39">
-        <f>IF((C8)=0,0,(C22-C27)/(C8))</f>
+        <f>IF((C59)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C53)/('Grovfôr'!C46)))/(C59))</f>
         <v/>
       </c>
       <c r="D95" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>da</t>
         </is>
       </c>
       <c r="E95" s="29" t="inlineStr">
         <is>
-          <t>Oppnådd mjølkepris pr liter (u/distriktstilskot) = (Mjølk [C22] − Herav distriktstilskot mjølk [C27]) ÷ Levert mjølk [C8]</t>
+          <t>Korrigerte dekar pr «kueining» i produksjonen = (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C53] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46]) ÷ «Kueiningar» [C59]   (Grovfôrarealet produksjonen får (etter eigen grovfôrkostnad) delt på kueiningane i produksjonen)</t>
         </is>
       </c>
       <c r="F95" s="30" t="inlineStr">
         <is>
-          <t>=IF((C8)=0,0,(C22-C27)/(C8))</t>
+          <t>=IF((C59)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C53)/('Grovfôr'!C46)))/(C59))</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="25" t="inlineStr">
         <is>
-          <t>Oppnådd slaktepris pr kg (u/distriktstilskot)</t>
+          <t>Oppnådd mjølkepris pr liter (u/distriktstilskot)</t>
         </is>
       </c>
       <c r="B96" s="26" t="inlineStr">
@@ -10397,7 +10397,7 @@
         </is>
       </c>
       <c r="C96" s="39">
-        <f>IF((C10)=0,0,(C23-C28)/(C10))</f>
+        <f>IF((C8)=0,0,(C22-C27)/(C8))</f>
         <v/>
       </c>
       <c r="D96" s="28" t="inlineStr">
@@ -10407,19 +10407,19 @@
       </c>
       <c r="E96" s="29" t="inlineStr">
         <is>
-          <t>Oppnådd slaktepris pr kg (u/distriktstilskot) = (Slakt [C23] − Herav distriktstilskot kjøt [C28]) ÷ Kg slakt storfe (mjølkeproduksjonen) [C10]</t>
+          <t>Oppnådd mjølkepris pr liter (u/distriktstilskot) = (Mjølk [C22] − Herav distriktstilskot mjølk [C27]) ÷ Levert mjølk [C8]</t>
         </is>
       </c>
       <c r="F96" s="30" t="inlineStr">
         <is>
-          <t>=IF((C10)=0,0,(C23-C28)/(C10))</t>
+          <t>=IF((C8)=0,0,(C22-C27)/(C8))</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="25" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr liter</t>
+          <t>Oppnådd slaktepris pr kg (u/distriktstilskot)</t>
         </is>
       </c>
       <c r="B97" s="26" t="inlineStr">
@@ -10428,7 +10428,7 @@
         </is>
       </c>
       <c r="C97" s="39">
-        <f>IF((C8)=0,0,(C47)/(C8))</f>
+        <f>IF((C10)=0,0,(C23-C28)/(C10))</f>
         <v/>
       </c>
       <c r="D97" s="28" t="inlineStr">
@@ -10438,19 +10438,19 @@
       </c>
       <c r="E97" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr liter = Maskinkostnader fordelt [C47] ÷ Levert mjølk [C8]</t>
+          <t>Oppnådd slaktepris pr kg (u/distriktstilskot) = (Slakt [C23] − Herav distriktstilskot kjøt [C28]) ÷ Kg slakt storfe (mjølkeproduksjonen) [C10]</t>
         </is>
       </c>
       <c r="F97" s="30" t="inlineStr">
         <is>
-          <t>=IF((C8)=0,0,(C47)/(C8))</t>
+          <t>=IF((C10)=0,0,(C23-C28)/(C10))</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="25" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr liter</t>
+          <t>Maskinkostnader pr liter</t>
         </is>
       </c>
       <c r="B98" s="26" t="inlineStr">
@@ -10459,7 +10459,7 @@
         </is>
       </c>
       <c r="C98" s="39">
-        <f>IF((C8)=0,0,(C48)/(C8))</f>
+        <f>IF((C8)=0,0,(C47)/(C8))</f>
         <v/>
       </c>
       <c r="D98" s="28" t="inlineStr">
@@ -10469,19 +10469,19 @@
       </c>
       <c r="E98" s="29" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr liter = Innandørsmekanisering fordelt [C48] ÷ Levert mjølk [C8]</t>
+          <t>Maskinkostnader pr liter = Maskinkostnader fordelt [C47] ÷ Levert mjølk [C8]</t>
         </is>
       </c>
       <c r="F98" s="30" t="inlineStr">
         <is>
-          <t>=IF((C8)=0,0,(C48)/(C8))</t>
+          <t>=IF((C8)=0,0,(C47)/(C8))</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="25" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr årsku</t>
+          <t>Innandørsmekanisering pr liter</t>
         </is>
       </c>
       <c r="B99" s="26" t="inlineStr">
@@ -10490,7 +10490,7 @@
         </is>
       </c>
       <c r="C99" s="39">
-        <f>IF((C7)=0,0,(C48)/(C7))</f>
+        <f>IF((C8)=0,0,(C48)/(C8))</f>
         <v/>
       </c>
       <c r="D99" s="28" t="inlineStr">
@@ -10500,19 +10500,19 @@
       </c>
       <c r="E99" s="29" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr årsku = Innandørsmekanisering fordelt [C48] ÷ Tal årskyr [C7]</t>
+          <t>Innandørsmekanisering pr liter = Innandørsmekanisering fordelt [C48] ÷ Levert mjølk [C8]</t>
         </is>
       </c>
       <c r="F99" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C48)/(C7))</t>
+          <t>=IF((C8)=0,0,(C48)/(C8))</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="25" t="inlineStr">
         <is>
-          <t>Levert mjølk pr årsku (liter)</t>
+          <t>Innandørsmekanisering pr årsku</t>
         </is>
       </c>
       <c r="B100" s="26" t="inlineStr">
@@ -10520,30 +10520,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C100" s="27">
-        <f>IF((C7)=0,0,(C8)/(C7))</f>
+      <c r="C100" s="39">
+        <f>IF((C7)=0,0,(C48)/(C7))</f>
         <v/>
       </c>
       <c r="D100" s="28" t="inlineStr">
         <is>
-          <t>liter</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E100" s="29" t="inlineStr">
         <is>
-          <t>Levert mjølk pr årsku (liter) = Levert mjølk [C8] ÷ Tal årskyr [C7]</t>
+          <t>Innandørsmekanisering pr årsku = Innandørsmekanisering fordelt [C48] ÷ Tal årskyr [C7]</t>
         </is>
       </c>
       <c r="F100" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C8)/(C7))</t>
+          <t>=IF((C7)=0,0,(C48)/(C7))</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="25" t="inlineStr">
         <is>
-          <t>Påsettprosent</t>
+          <t>Levert mjølk pr årsku (liter)</t>
         </is>
       </c>
       <c r="B101" s="26" t="inlineStr">
@@ -10551,30 +10551,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C101" s="33">
-        <f>C60</f>
+      <c r="C101" s="27">
+        <f>IF((C7)=0,0,(C8)/(C7))</f>
         <v/>
       </c>
       <c r="D101" s="28" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>liter</t>
         </is>
       </c>
       <c r="E101" s="29" t="inlineStr">
         <is>
-          <t>Påsettprosent = Påsettprosent [C60]</t>
+          <t>Levert mjølk pr årsku (liter) = Levert mjølk [C8] ÷ Tal årskyr [C7]</t>
         </is>
       </c>
       <c r="F101" s="30" t="inlineStr">
         <is>
-          <t>=C60</t>
+          <t>=IF((C7)=0,0,(C8)/(C7))</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="25" t="inlineStr">
         <is>
-          <t>Kvoteoppfylling</t>
+          <t>Påsettprosent</t>
         </is>
       </c>
       <c r="B102" s="26" t="inlineStr">
@@ -10583,7 +10583,7 @@
         </is>
       </c>
       <c r="C102" s="33">
-        <f>IF((C9)=0,0,(C8)/(C9))</f>
+        <f>C60</f>
         <v/>
       </c>
       <c r="D102" s="28" t="inlineStr">
@@ -10593,41 +10593,72 @@
       </c>
       <c r="E102" s="29" t="inlineStr">
         <is>
-          <t>Kvoteoppfylling = Levert mjølk [C8] ÷ Disponibel mjølkekvote [C9]</t>
+          <t>Påsettprosent = Påsettprosent [C60]</t>
         </is>
       </c>
       <c r="F102" s="30" t="inlineStr">
         <is>
-          <t>=IF((C9)=0,0,(C8)/(C9))</t>
+          <t>=C60</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="25" t="inlineStr">
         <is>
+          <t>Kvoteoppfylling</t>
+        </is>
+      </c>
+      <c r="B103" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C103" s="33">
+        <f>IF((C9)=0,0,(C8)/(C9))</f>
+        <v/>
+      </c>
+      <c r="D103" s="28" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E103" s="29" t="inlineStr">
+        <is>
+          <t>Kvoteoppfylling = Levert mjølk [C8] ÷ Disponibel mjølkekvote [C9]</t>
+        </is>
+      </c>
+      <c r="F103" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C9)=0,0,(C8)/(C9))</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="25" t="inlineStr">
+        <is>
           <t>Analysegruppe (påsett)</t>
         </is>
       </c>
-      <c r="B103" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C103" s="41">
+      <c r="B104" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C104" s="41">
         <f>IF(C60&lt;=0.8,"Påsett &lt; 80 %",IF(C60&lt;1.2,"Påsett 80–120 %","Påsett &gt; 120 %"))</f>
         <v/>
       </c>
-      <c r="D103" s="28" t="inlineStr">
+      <c r="D104" s="28" t="inlineStr">
         <is>
           <t>tekst</t>
         </is>
       </c>
-      <c r="E103" s="29" t="inlineStr">
+      <c r="E104" s="29" t="inlineStr">
         <is>
           <t>Analysegruppe (påsett) = HVIS(Påsettprosent [C60]&lt;=0,8; "Påsett &lt; 80 %"; HVIS(Påsettprosent [C60]&lt;1,2; "Påsett 80–120 %"; "Påsett &gt; 120 %"))   (Tilsvarar arka «Mjølk &lt;80%», «Mjølk 80-120%» og «Mjølk &gt;120%» i eksempelanalysen)</t>
         </is>
       </c>
-      <c r="F103" s="30" t="inlineStr">
+      <c r="F104" s="30" t="inlineStr">
         <is>
           <t>=IF(C60&lt;=0.8,"Påsett &lt; 80 %",IF(C60&lt;1.2,"Påsett 80–120 %","Påsett &gt; 120 %"))</t>
         </is>
@@ -10645,7 +10676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -12765,7 +12796,7 @@
         </is>
       </c>
       <c r="C84" s="39">
-        <f>IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C50)/('Grovfôr'!C38)))=0,0,(C53)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C50)/('Grovfôr'!C38))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))=0,0,(C53)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46))))</f>
         <v/>
       </c>
       <c r="D84" s="28" t="inlineStr">
@@ -12775,12 +12806,12 @@
       </c>
       <c r="E84" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C53] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C21] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C38])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
+          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C53] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
         </is>
       </c>
       <c r="F84" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C50)/('Grovfôr'!C38)))=0,0,(C53)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C50)/('Grovfôr'!C38))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))=0,0,(C53)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46))))</t>
         </is>
       </c>
     </row>
@@ -12796,7 +12827,7 @@
         </is>
       </c>
       <c r="C85" s="39">
-        <f>IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C50)/('Grovfôr'!C38)))=0,0,(C54)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C50)/('Grovfôr'!C38))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))=0,0,(C54)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46))))</f>
         <v/>
       </c>
       <c r="D85" s="28" t="inlineStr">
@@ -12806,12 +12837,12 @@
       </c>
       <c r="E85" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C54] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C21] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C38])</t>
+          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C54] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])</t>
         </is>
       </c>
       <c r="F85" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C50)/('Grovfôr'!C38)))=0,0,(C54)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C50)/('Grovfôr'!C38))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))=0,0,(C54)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46))))</t>
         </is>
       </c>
     </row>
@@ -12827,7 +12858,7 @@
         </is>
       </c>
       <c r="C86" s="40">
-        <f>'Grovfôr'!C52</f>
+        <f>'Grovfôr'!C60</f>
         <v/>
       </c>
       <c r="D86" s="28" t="inlineStr">
@@ -12837,12 +12868,12 @@
       </c>
       <c r="E86" s="29" t="inlineStr">
         <is>
-          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C52]</t>
+          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C60]</t>
         </is>
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C52</t>
+          <t>='Grovfôr'!C60</t>
         </is>
       </c>
     </row>
@@ -12858,7 +12889,7 @@
         </is>
       </c>
       <c r="C87" s="40">
-        <f>'Grovfôr'!C53</f>
+        <f>'Grovfôr'!C61</f>
         <v/>
       </c>
       <c r="D87" s="28" t="inlineStr">
@@ -12868,19 +12899,19 @@
       </c>
       <c r="E87" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C53]</t>
+          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C61]</t>
         </is>
       </c>
       <c r="F87" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C53</t>
+          <t>='Grovfôr'!C61</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="25" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining»</t>
+          <t>Korrigerte dekar pr «kueining» (heile garden)</t>
         </is>
       </c>
       <c r="B88" s="26" t="inlineStr">
@@ -12889,7 +12920,7 @@
         </is>
       </c>
       <c r="C88" s="40">
-        <f>'Grovfôr'!C54</f>
+        <f>'Grovfôr'!C62</f>
         <v/>
       </c>
       <c r="D88" s="28" t="inlineStr">
@@ -12899,19 +12930,19 @@
       </c>
       <c r="E88" s="29" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining» = Korrigerte dekar pr «kueining» [Grovfôr!C54]</t>
+          <t>Korrigerte dekar pr «kueining» (heile garden) = Korrigerte dekar pr «kueining» [Grovfôr!C62]</t>
         </is>
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C54</t>
+          <t>='Grovfôr'!C62</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="25" t="inlineStr">
         <is>
-          <t>Snitt slaktepris pr okse</t>
+          <t>Korrigerte dekar pr «kueining» i produksjonen</t>
         </is>
       </c>
       <c r="B89" s="26" t="inlineStr">
@@ -12920,29 +12951,29 @@
         </is>
       </c>
       <c r="C89" s="39">
-        <f>IF((C9)=0,0,(C21)/(C9))</f>
+        <f>IF((C56)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))/(C56))</f>
         <v/>
       </c>
       <c r="D89" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>da</t>
         </is>
       </c>
       <c r="E89" s="29" t="inlineStr">
         <is>
-          <t>Snitt slaktepris pr okse = Slakt [C21] ÷ Tal slakta oksar [C9]</t>
+          <t>Korrigerte dekar pr «kueining» i produksjonen = (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46]) ÷ «Kueiningar» [C56]   (Grovfôrarealet produksjonen får (etter eigen grovfôrkostnad) delt på kueiningane i produksjonen)</t>
         </is>
       </c>
       <c r="F89" s="30" t="inlineStr">
         <is>
-          <t>=IF((C9)=0,0,(C21)/(C9))</t>
+          <t>=IF((C56)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))/(C56))</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="25" t="inlineStr">
         <is>
-          <t>Snitt kjøpspris pr kalv</t>
+          <t>Snitt slaktepris pr okse</t>
         </is>
       </c>
       <c r="B90" s="26" t="inlineStr">
@@ -12951,7 +12982,7 @@
         </is>
       </c>
       <c r="C90" s="39">
-        <f>IF((C11)=0,0,(C41)/(C11))</f>
+        <f>IF((C9)=0,0,(C21)/(C9))</f>
         <v/>
       </c>
       <c r="D90" s="28" t="inlineStr">
@@ -12961,19 +12992,19 @@
       </c>
       <c r="E90" s="29" t="inlineStr">
         <is>
-          <t>Snitt kjøpspris pr kalv = Innkjøp dyr [C41] ÷ Tal kjøpte kalvar [C11]</t>
+          <t>Snitt slaktepris pr okse = Slakt [C21] ÷ Tal slakta oksar [C9]</t>
         </is>
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>=IF((C11)=0,0,(C41)/(C11))</t>
+          <t>=IF((C9)=0,0,(C21)/(C9))</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="25" t="inlineStr">
         <is>
-          <t>Slaktepris – kjøpspris pr okse</t>
+          <t>Snitt kjøpspris pr kalv</t>
         </is>
       </c>
       <c r="B91" s="26" t="inlineStr">
@@ -12982,7 +13013,7 @@
         </is>
       </c>
       <c r="C91" s="39">
-        <f>IF((C9)=0,0,(C21)/(C9))-IF((C11)=0,0,(C41)/(C11))</f>
+        <f>IF((C11)=0,0,(C41)/(C11))</f>
         <v/>
       </c>
       <c r="D91" s="28" t="inlineStr">
@@ -12992,19 +13023,19 @@
       </c>
       <c r="E91" s="29" t="inlineStr">
         <is>
-          <t>Slaktepris – kjøpspris pr okse = Slakt [C21] ÷ Tal slakta oksar [C9] − Innkjøp dyr [C41] ÷ Tal kjøpte kalvar [C11]</t>
+          <t>Snitt kjøpspris pr kalv = Innkjøp dyr [C41] ÷ Tal kjøpte kalvar [C11]</t>
         </is>
       </c>
       <c r="F91" s="30" t="inlineStr">
         <is>
-          <t>=IF((C9)=0,0,(C21)/(C9))-IF((C11)=0,0,(C41)/(C11))</t>
+          <t>=IF((C11)=0,0,(C41)/(C11))</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="25" t="inlineStr">
         <is>
-          <t>Oppnådd pris pr kg slakt (u/distriktstilskot)</t>
+          <t>Slaktepris – kjøpspris pr okse</t>
         </is>
       </c>
       <c r="B92" s="26" t="inlineStr">
@@ -13013,7 +13044,7 @@
         </is>
       </c>
       <c r="C92" s="39">
-        <f>IF((C8)=0,0,(C21-C25)/(C8))</f>
+        <f>IF((C9)=0,0,(C21)/(C9))-IF((C11)=0,0,(C41)/(C11))</f>
         <v/>
       </c>
       <c r="D92" s="28" t="inlineStr">
@@ -13023,19 +13054,19 @@
       </c>
       <c r="E92" s="29" t="inlineStr">
         <is>
-          <t>Oppnådd pris pr kg slakt (u/distriktstilskot) = (Slakt [C21] − Herav distriktstilskot kjøt [C25]) ÷ Kg slakt [C8]</t>
+          <t>Slaktepris – kjøpspris pr okse = Slakt [C21] ÷ Tal slakta oksar [C9] − Innkjøp dyr [C41] ÷ Tal kjøpte kalvar [C11]</t>
         </is>
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>=IF((C8)=0,0,(C21-C25)/(C8))</t>
+          <t>=IF((C9)=0,0,(C21)/(C9))-IF((C11)=0,0,(C41)/(C11))</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="25" t="inlineStr">
         <is>
-          <t>Slaktevekt pr okse (kg)</t>
+          <t>Oppnådd pris pr kg slakt (u/distriktstilskot)</t>
         </is>
       </c>
       <c r="B93" s="26" t="inlineStr">
@@ -13043,30 +13074,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C93" s="37">
-        <f>IF((C9)=0,0,(C8)/(C9))</f>
+      <c r="C93" s="39">
+        <f>IF((C8)=0,0,(C21-C25)/(C8))</f>
         <v/>
       </c>
       <c r="D93" s="28" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E93" s="29" t="inlineStr">
         <is>
-          <t>Slaktevekt pr okse (kg) = Kg slakt [C8] ÷ Tal slakta oksar [C9]</t>
+          <t>Oppnådd pris pr kg slakt (u/distriktstilskot) = (Slakt [C21] − Herav distriktstilskot kjøt [C25]) ÷ Kg slakt [C8]</t>
         </is>
       </c>
       <c r="F93" s="30" t="inlineStr">
         <is>
-          <t>=IF((C9)=0,0,(C8)/(C9))</t>
+          <t>=IF((C8)=0,0,(C21-C25)/(C8))</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="25" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr okse</t>
+          <t>Slaktevekt pr okse (kg)</t>
         </is>
       </c>
       <c r="B94" s="26" t="inlineStr">
@@ -13074,52 +13105,83 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C94" s="39">
-        <f>IF((C7)=0,0,(C45)/(C7))</f>
+      <c r="C94" s="37">
+        <f>IF((C9)=0,0,(C8)/(C9))</f>
         <v/>
       </c>
       <c r="D94" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E94" s="29" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr okse = Innandørsmekanisering fordelt [C45] ÷ Tal produserte oksar [C7]</t>
+          <t>Slaktevekt pr okse (kg) = Kg slakt [C8] ÷ Tal slakta oksar [C9]</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C45)/(C7))</t>
+          <t>=IF((C9)=0,0,(C8)/(C9))</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="25" t="inlineStr">
         <is>
+          <t>Innandørsmekanisering pr okse</t>
+        </is>
+      </c>
+      <c r="B95" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C95" s="39">
+        <f>IF((C7)=0,0,(C45)/(C7))</f>
+        <v/>
+      </c>
+      <c r="D95" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E95" s="29" t="inlineStr">
+        <is>
+          <t>Innandørsmekanisering pr okse = Innandørsmekanisering fordelt [C45] ÷ Tal produserte oksar [C7]</t>
+        </is>
+      </c>
+      <c r="F95" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C7)=0,0,(C45)/(C7))</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="25" t="inlineStr">
+        <is>
           <t>Tapsprosent</t>
         </is>
       </c>
-      <c r="B95" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C95" s="33">
+      <c r="B96" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C96" s="33">
         <f>MAX(0,IF((C12+C14+C11)=0,0,((C12+C14+C11)-(C13+C15+C9+C10))/(C12+C14+C11)))</f>
         <v/>
       </c>
-      <c r="D95" s="28" t="inlineStr">
+      <c r="D96" s="28" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E95" s="29" t="inlineStr">
+      <c r="E96" s="29" t="inlineStr">
         <is>
           <t>Tapsprosent = MAKS(0; ((Oksar over 12 md pr 1.1. [C12] + Oksar/kalvar under 12 md pr 1.1. [C14] + Tal kjøpte kalvar [C11]) − (Oksar over 12 md pr 31.12. [C13] + Oksar/kalvar under 12 md pr 31.12. [C15] + Tal slakta oksar [C9] + Tal storfe selt til liv [C10])) ÷ (Oksar over 12 md pr 1.1. [C12] + Oksar/kalvar under 12 md pr 1.1. [C14] + Tal kjøpte kalvar [C11]))   ((Inngåande dyr + kjøpte) – (utgåande dyr + slakta + selde), delt på inngåande + kjøpte)</t>
         </is>
       </c>
-      <c r="F95" s="30" t="inlineStr">
+      <c r="F96" s="30" t="inlineStr">
         <is>
           <t>=MAX(0,IF((C12+C14+C11)=0,0,((C12+C14+C11)-(C13+C15+C9+C10))/(C12+C14+C11)))</t>
         </is>
@@ -13137,7 +13199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -15257,7 +15319,7 @@
         </is>
       </c>
       <c r="C84" s="39">
-        <f>IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C50)/('Grovfôr'!C38)))=0,0,(C53)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C50)/('Grovfôr'!C38))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))=0,0,(C53)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46))))</f>
         <v/>
       </c>
       <c r="D84" s="28" t="inlineStr">
@@ -15267,12 +15329,12 @@
       </c>
       <c r="E84" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C53] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C21] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C38])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
+          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C53] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
         </is>
       </c>
       <c r="F84" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C50)/('Grovfôr'!C38)))=0,0,(C53)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C50)/('Grovfôr'!C38))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))=0,0,(C53)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46))))</t>
         </is>
       </c>
     </row>
@@ -15288,7 +15350,7 @@
         </is>
       </c>
       <c r="C85" s="39">
-        <f>IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C50)/('Grovfôr'!C38)))=0,0,(C54)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C50)/('Grovfôr'!C38))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))=0,0,(C54)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46))))</f>
         <v/>
       </c>
       <c r="D85" s="28" t="inlineStr">
@@ -15298,12 +15360,12 @@
       </c>
       <c r="E85" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C54] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C21] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C38])</t>
+          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C54] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])</t>
         </is>
       </c>
       <c r="F85" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C50)/('Grovfôr'!C38)))=0,0,(C54)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C50)/('Grovfôr'!C38))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))=0,0,(C54)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46))))</t>
         </is>
       </c>
     </row>
@@ -15319,7 +15381,7 @@
         </is>
       </c>
       <c r="C86" s="40">
-        <f>'Grovfôr'!C52</f>
+        <f>'Grovfôr'!C60</f>
         <v/>
       </c>
       <c r="D86" s="28" t="inlineStr">
@@ -15329,12 +15391,12 @@
       </c>
       <c r="E86" s="29" t="inlineStr">
         <is>
-          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C52]</t>
+          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C60]</t>
         </is>
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C52</t>
+          <t>='Grovfôr'!C60</t>
         </is>
       </c>
     </row>
@@ -15350,7 +15412,7 @@
         </is>
       </c>
       <c r="C87" s="40">
-        <f>'Grovfôr'!C53</f>
+        <f>'Grovfôr'!C61</f>
         <v/>
       </c>
       <c r="D87" s="28" t="inlineStr">
@@ -15360,19 +15422,19 @@
       </c>
       <c r="E87" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C53]</t>
+          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C61]</t>
         </is>
       </c>
       <c r="F87" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C53</t>
+          <t>='Grovfôr'!C61</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="25" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining»</t>
+          <t>Korrigerte dekar pr «kueining» (heile garden)</t>
         </is>
       </c>
       <c r="B88" s="26" t="inlineStr">
@@ -15381,7 +15443,7 @@
         </is>
       </c>
       <c r="C88" s="40">
-        <f>'Grovfôr'!C54</f>
+        <f>'Grovfôr'!C62</f>
         <v/>
       </c>
       <c r="D88" s="28" t="inlineStr">
@@ -15391,19 +15453,19 @@
       </c>
       <c r="E88" s="29" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining» = Korrigerte dekar pr «kueining» [Grovfôr!C54]</t>
+          <t>Korrigerte dekar pr «kueining» (heile garden) = Korrigerte dekar pr «kueining» [Grovfôr!C62]</t>
         </is>
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C54</t>
+          <t>='Grovfôr'!C62</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="25" t="inlineStr">
         <is>
-          <t>Snitt slaktepris pr kalv (u/distriktstilskot)</t>
+          <t>Korrigerte dekar pr «kueining» i produksjonen</t>
         </is>
       </c>
       <c r="B89" s="26" t="inlineStr">
@@ -15412,29 +15474,29 @@
         </is>
       </c>
       <c r="C89" s="39">
-        <f>IF((C9)=0,0,(C21-C25)/(C9))</f>
+        <f>IF((C56)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))/(C56))</f>
         <v/>
       </c>
       <c r="D89" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>da</t>
         </is>
       </c>
       <c r="E89" s="29" t="inlineStr">
         <is>
-          <t>Snitt slaktepris pr kalv (u/distriktstilskot) = (Slakt [C21] − Herav distriktstilskot kjøt [C25]) ÷ Tal slakta kalvar [C9]</t>
+          <t>Korrigerte dekar pr «kueining» i produksjonen = (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46]) ÷ «Kueiningar» [C56]   (Grovfôrarealet produksjonen får (etter eigen grovfôrkostnad) delt på kueiningane i produksjonen)</t>
         </is>
       </c>
       <c r="F89" s="30" t="inlineStr">
         <is>
-          <t>=IF((C9)=0,0,(C21-C25)/(C9))</t>
+          <t>=IF((C56)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))/(C56))</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="25" t="inlineStr">
         <is>
-          <t>Snitt kjøpspris pr kalv</t>
+          <t>Snitt slaktepris pr kalv (u/distriktstilskot)</t>
         </is>
       </c>
       <c r="B90" s="26" t="inlineStr">
@@ -15443,7 +15505,7 @@
         </is>
       </c>
       <c r="C90" s="39">
-        <f>IF((C11)=0,0,(C41)/(C11))</f>
+        <f>IF((C9)=0,0,(C21-C25)/(C9))</f>
         <v/>
       </c>
       <c r="D90" s="28" t="inlineStr">
@@ -15453,19 +15515,19 @@
       </c>
       <c r="E90" s="29" t="inlineStr">
         <is>
-          <t>Snitt kjøpspris pr kalv = Innkjøp dyr [C41] ÷ Tal kjøpte kalvar [C11]</t>
+          <t>Snitt slaktepris pr kalv (u/distriktstilskot) = (Slakt [C21] − Herav distriktstilskot kjøt [C25]) ÷ Tal slakta kalvar [C9]</t>
         </is>
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>=IF((C11)=0,0,(C41)/(C11))</t>
+          <t>=IF((C9)=0,0,(C21-C25)/(C9))</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="25" t="inlineStr">
         <is>
-          <t>Slaktepris – kjøpspris pr kalv</t>
+          <t>Snitt kjøpspris pr kalv</t>
         </is>
       </c>
       <c r="B91" s="26" t="inlineStr">
@@ -15474,7 +15536,7 @@
         </is>
       </c>
       <c r="C91" s="39">
-        <f>IF((C9)=0,0,(C21)/(C9))-IF((C11)=0,0,(C41)/(C11))</f>
+        <f>IF((C11)=0,0,(C41)/(C11))</f>
         <v/>
       </c>
       <c r="D91" s="28" t="inlineStr">
@@ -15484,19 +15546,19 @@
       </c>
       <c r="E91" s="29" t="inlineStr">
         <is>
-          <t>Slaktepris – kjøpspris pr kalv = Slakt [C21] ÷ Tal slakta kalvar [C9] − Innkjøp dyr [C41] ÷ Tal kjøpte kalvar [C11]</t>
+          <t>Snitt kjøpspris pr kalv = Innkjøp dyr [C41] ÷ Tal kjøpte kalvar [C11]</t>
         </is>
       </c>
       <c r="F91" s="30" t="inlineStr">
         <is>
-          <t>=IF((C9)=0,0,(C21)/(C9))-IF((C11)=0,0,(C41)/(C11))</t>
+          <t>=IF((C11)=0,0,(C41)/(C11))</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="25" t="inlineStr">
         <is>
-          <t>Oppnådd pris pr kg slakt (u/distriktstilskot)</t>
+          <t>Slaktepris – kjøpspris pr kalv</t>
         </is>
       </c>
       <c r="B92" s="26" t="inlineStr">
@@ -15505,7 +15567,7 @@
         </is>
       </c>
       <c r="C92" s="39">
-        <f>IF((C8)=0,0,(C21-C25)/(C8))</f>
+        <f>IF((C9)=0,0,(C21)/(C9))-IF((C11)=0,0,(C41)/(C11))</f>
         <v/>
       </c>
       <c r="D92" s="28" t="inlineStr">
@@ -15515,19 +15577,19 @@
       </c>
       <c r="E92" s="29" t="inlineStr">
         <is>
-          <t>Oppnådd pris pr kg slakt (u/distriktstilskot) = (Slakt [C21] − Herav distriktstilskot kjøt [C25]) ÷ Kg slakt [C8]</t>
+          <t>Slaktepris – kjøpspris pr kalv = Slakt [C21] ÷ Tal slakta kalvar [C9] − Innkjøp dyr [C41] ÷ Tal kjøpte kalvar [C11]</t>
         </is>
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>=IF((C8)=0,0,(C21-C25)/(C8))</t>
+          <t>=IF((C9)=0,0,(C21)/(C9))-IF((C11)=0,0,(C41)/(C11))</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="25" t="inlineStr">
         <is>
-          <t>Slaktevekt pr kalv (kg)</t>
+          <t>Oppnådd pris pr kg slakt (u/distriktstilskot)</t>
         </is>
       </c>
       <c r="B93" s="26" t="inlineStr">
@@ -15535,30 +15597,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C93" s="37">
-        <f>IF((C9)=0,0,(C8)/(C9))</f>
+      <c r="C93" s="39">
+        <f>IF((C8)=0,0,(C21-C25)/(C8))</f>
         <v/>
       </c>
       <c r="D93" s="28" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E93" s="29" t="inlineStr">
         <is>
-          <t>Slaktevekt pr kalv (kg) = Kg slakt [C8] ÷ Tal slakta kalvar [C9]</t>
+          <t>Oppnådd pris pr kg slakt (u/distriktstilskot) = (Slakt [C21] − Herav distriktstilskot kjøt [C25]) ÷ Kg slakt [C8]</t>
         </is>
       </c>
       <c r="F93" s="30" t="inlineStr">
         <is>
-          <t>=IF((C9)=0,0,(C8)/(C9))</t>
+          <t>=IF((C8)=0,0,(C21-C25)/(C8))</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="25" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr kalv</t>
+          <t>Slaktevekt pr kalv (kg)</t>
         </is>
       </c>
       <c r="B94" s="26" t="inlineStr">
@@ -15566,52 +15628,83 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C94" s="39">
-        <f>IF((C7)=0,0,(C45)/(C7))</f>
+      <c r="C94" s="37">
+        <f>IF((C9)=0,0,(C8)/(C9))</f>
         <v/>
       </c>
       <c r="D94" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E94" s="29" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr kalv = Innandørsmekanisering fordelt [C45] ÷ Tal produserte kalvar [C7]</t>
+          <t>Slaktevekt pr kalv (kg) = Kg slakt [C8] ÷ Tal slakta kalvar [C9]</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C45)/(C7))</t>
+          <t>=IF((C9)=0,0,(C8)/(C9))</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="25" t="inlineStr">
         <is>
+          <t>Innandørsmekanisering pr kalv</t>
+        </is>
+      </c>
+      <c r="B95" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C95" s="39">
+        <f>IF((C7)=0,0,(C45)/(C7))</f>
+        <v/>
+      </c>
+      <c r="D95" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E95" s="29" t="inlineStr">
+        <is>
+          <t>Innandørsmekanisering pr kalv = Innandørsmekanisering fordelt [C45] ÷ Tal produserte kalvar [C7]</t>
+        </is>
+      </c>
+      <c r="F95" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C7)=0,0,(C45)/(C7))</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="25" t="inlineStr">
+        <is>
           <t>Tapsprosent</t>
         </is>
       </c>
-      <c r="B95" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C95" s="33">
+      <c r="B96" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C96" s="33">
         <f>MAX(0,IF((C12+C14+C11)=0,0,((C12+C14+C11)-(C13+C15+C9+C10))/(C12+C14+C11)))</f>
         <v/>
       </c>
-      <c r="D95" s="28" t="inlineStr">
+      <c r="D96" s="28" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E95" s="29" t="inlineStr">
+      <c r="E96" s="29" t="inlineStr">
         <is>
           <t>Tapsprosent = MAKS(0; ((Ungdyr over 12 md pr 1.1. [C12] + Kalvar under 12 md pr 1.1. [C14] + Tal kjøpte kalvar [C11]) − (Ungdyr over 12 md pr 31.12. [C13] + Kalvar under 12 md pr 31.12. [C15] + Tal slakta kalvar [C9] + Tal selt til liv [C10])) ÷ (Ungdyr over 12 md pr 1.1. [C12] + Kalvar under 12 md pr 1.1. [C14] + Tal kjøpte kalvar [C11]))</t>
         </is>
       </c>
-      <c r="F95" s="30" t="inlineStr">
+      <c r="F96" s="30" t="inlineStr">
         <is>
           <t>=MAX(0,IF((C12+C14+C11)=0,0,((C12+C14+C11)-(C13+C15+C9+C10))/(C12+C14+C11)))</t>
         </is>
@@ -15629,7 +15722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F100"/>
+  <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -17910,7 +18003,7 @@
         </is>
       </c>
       <c r="C90" s="39">
-        <f>IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C55)/('Grovfôr'!C38)))=0,0,(C58)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C55)/('Grovfôr'!C38))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C55)/('Grovfôr'!C46)))=0,0,(C58)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C55)/('Grovfôr'!C46))))</f>
         <v/>
       </c>
       <c r="D90" s="28" t="inlineStr">
@@ -17920,12 +18013,12 @@
       </c>
       <c r="E90" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C58] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C21] × Sum eigen grovfôrproduksjon (utan lagerendring) [C55] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C38])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
+          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C58] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C55] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
         </is>
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C55)/('Grovfôr'!C38)))=0,0,(C58)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C55)/('Grovfôr'!C38))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C55)/('Grovfôr'!C46)))=0,0,(C58)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C55)/('Grovfôr'!C46))))</t>
         </is>
       </c>
     </row>
@@ -17941,7 +18034,7 @@
         </is>
       </c>
       <c r="C91" s="39">
-        <f>IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C55)/('Grovfôr'!C38)))=0,0,(C59)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C55)/('Grovfôr'!C38))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C55)/('Grovfôr'!C46)))=0,0,(C59)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C55)/('Grovfôr'!C46))))</f>
         <v/>
       </c>
       <c r="D91" s="28" t="inlineStr">
@@ -17951,12 +18044,12 @@
       </c>
       <c r="E91" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C59] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C21] × Sum eigen grovfôrproduksjon (utan lagerendring) [C55] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C38])</t>
+          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C59] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C55] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])</t>
         </is>
       </c>
       <c r="F91" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C55)/('Grovfôr'!C38)))=0,0,(C59)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C55)/('Grovfôr'!C38))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C55)/('Grovfôr'!C46)))=0,0,(C59)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C55)/('Grovfôr'!C46))))</t>
         </is>
       </c>
     </row>
@@ -17972,7 +18065,7 @@
         </is>
       </c>
       <c r="C92" s="40">
-        <f>'Grovfôr'!C52</f>
+        <f>'Grovfôr'!C60</f>
         <v/>
       </c>
       <c r="D92" s="28" t="inlineStr">
@@ -17982,12 +18075,12 @@
       </c>
       <c r="E92" s="29" t="inlineStr">
         <is>
-          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C52]</t>
+          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C60]</t>
         </is>
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C52</t>
+          <t>='Grovfôr'!C60</t>
         </is>
       </c>
     </row>
@@ -18003,7 +18096,7 @@
         </is>
       </c>
       <c r="C93" s="40">
-        <f>'Grovfôr'!C53</f>
+        <f>'Grovfôr'!C61</f>
         <v/>
       </c>
       <c r="D93" s="28" t="inlineStr">
@@ -18013,19 +18106,19 @@
       </c>
       <c r="E93" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C53]</t>
+          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C61]</t>
         </is>
       </c>
       <c r="F93" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C53</t>
+          <t>='Grovfôr'!C61</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="25" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining»</t>
+          <t>Korrigerte dekar pr «kueining» (heile garden)</t>
         </is>
       </c>
       <c r="B94" s="26" t="inlineStr">
@@ -18034,7 +18127,7 @@
         </is>
       </c>
       <c r="C94" s="40">
-        <f>'Grovfôr'!C54</f>
+        <f>'Grovfôr'!C62</f>
         <v/>
       </c>
       <c r="D94" s="28" t="inlineStr">
@@ -18044,19 +18137,19 @@
       </c>
       <c r="E94" s="29" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining» = Korrigerte dekar pr «kueining» [Grovfôr!C54]</t>
+          <t>Korrigerte dekar pr «kueining» (heile garden) = Korrigerte dekar pr «kueining» [Grovfôr!C62]</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C54</t>
+          <t>='Grovfôr'!C62</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="25" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr ammeku</t>
+          <t>Korrigerte dekar pr «kueining» i produksjonen</t>
         </is>
       </c>
       <c r="B95" s="26" t="inlineStr">
@@ -18065,29 +18158,29 @@
         </is>
       </c>
       <c r="C95" s="39">
-        <f>IF((C7)=0,0,(C50)/(C7))</f>
+        <f>IF((C61)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C55)/('Grovfôr'!C46)))/(C61))</f>
         <v/>
       </c>
       <c r="D95" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>da</t>
         </is>
       </c>
       <c r="E95" s="29" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr ammeku = Innandørsmekanisering fordelt [C50] ÷ Tal ammekyr [C7]</t>
+          <t>Korrigerte dekar pr «kueining» i produksjonen = (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C55] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46]) ÷ «Kueiningar» [C61]   (Grovfôrarealet produksjonen får (etter eigen grovfôrkostnad) delt på kueiningane i produksjonen)</t>
         </is>
       </c>
       <c r="F95" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C50)/(C7))</t>
+          <t>=IF((C61)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C55)/('Grovfôr'!C46)))/(C61))</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="25" t="inlineStr">
         <is>
-          <t>Påsettprosent</t>
+          <t>Innandørsmekanisering pr ammeku</t>
         </is>
       </c>
       <c r="B96" s="26" t="inlineStr">
@@ -18095,30 +18188,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C96" s="33">
-        <f>C62</f>
+      <c r="C96" s="39">
+        <f>IF((C7)=0,0,(C50)/(C7))</f>
         <v/>
       </c>
       <c r="D96" s="28" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E96" s="29" t="inlineStr">
         <is>
-          <t>Påsettprosent = Påsettprosent [C62]</t>
+          <t>Innandørsmekanisering pr ammeku = Innandørsmekanisering fordelt [C50] ÷ Tal ammekyr [C7]</t>
         </is>
       </c>
       <c r="F96" s="30" t="inlineStr">
         <is>
-          <t>=C62</t>
+          <t>=IF((C7)=0,0,(C50)/(C7))</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="25" t="inlineStr">
         <is>
-          <t>Snitt slaktevekt kyr (kg)</t>
+          <t>Påsettprosent</t>
         </is>
       </c>
       <c r="B97" s="26" t="inlineStr">
@@ -18126,30 +18219,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C97" s="37">
-        <f>IF((C17)=0,0,(C16)/(C17))</f>
+      <c r="C97" s="33">
+        <f>C62</f>
         <v/>
       </c>
       <c r="D97" s="28" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E97" s="29" t="inlineStr">
         <is>
-          <t>Snitt slaktevekt kyr (kg) = Kg slakt kyr [C16] ÷ Tal slakta kyr [C17]</t>
+          <t>Påsettprosent = Påsettprosent [C62]</t>
         </is>
       </c>
       <c r="F97" s="30" t="inlineStr">
         <is>
-          <t>=IF((C17)=0,0,(C16)/(C17))</t>
+          <t>=C62</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="25" t="inlineStr">
         <is>
-          <t>Nyttbar kalv pr ku</t>
+          <t>Snitt slaktevekt kyr (kg)</t>
         </is>
       </c>
       <c r="B98" s="26" t="inlineStr">
@@ -18157,30 +18250,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C98" s="39">
-        <f>IF((C7)=0,0,((C9+C11+C13+C15)+C19-C20-(C8+C10+C12+C14))/(C7))</f>
+      <c r="C98" s="37">
+        <f>IF((C17)=0,0,(C16)/(C17))</f>
         <v/>
       </c>
       <c r="D98" s="28" t="inlineStr">
         <is>
-          <t>stk</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E98" s="29" t="inlineStr">
         <is>
-          <t>Nyttbar kalv pr ku = ((Ammekyr pr 31.12. [C9] + Avlsokse pr 31.12. [C11] + Ungdyr over 12 md pr 31.12. [C13] + Kalvar/ungdyr under 12 md pr 31.12. [C15]) + Tal dyr slakta / selt til liv [C19] − Tal kjøpte dyr [C20] − (Ammekyr pr 1.1. [C8] + Avlsokse pr 1.1. [C10] + Ungdyr over 12 md pr 1.1. [C12] + Kalvar/ungdyr under 12 md pr 1.1. [C14])) ÷ Tal ammekyr [C7]   ((Dyr 31.12. + slakta/selde – kjøpte – dyr 1.1.) delt på tal ammekyr)</t>
+          <t>Snitt slaktevekt kyr (kg) = Kg slakt kyr [C16] ÷ Tal slakta kyr [C17]</t>
         </is>
       </c>
       <c r="F98" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,((C9+C11+C13+C15)+C19-C20-(C8+C10+C12+C14))/(C7))</t>
+          <t>=IF((C17)=0,0,(C16)/(C17))</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="25" t="inlineStr">
         <is>
-          <t>Oppnådd pris pr kg slakt (u/distriktstilskot)</t>
+          <t>Nyttbar kalv pr ku</t>
         </is>
       </c>
       <c r="B99" s="26" t="inlineStr">
@@ -18189,51 +18282,82 @@
         </is>
       </c>
       <c r="C99" s="39">
-        <f>IF((C18)=0,0,(C27-C30)/(C18))</f>
+        <f>IF((C7)=0,0,((C9+C11+C13+C15)+C19-C20-(C8+C10+C12+C14))/(C7))</f>
         <v/>
       </c>
       <c r="D99" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>stk</t>
         </is>
       </c>
       <c r="E99" s="29" t="inlineStr">
         <is>
-          <t>Oppnådd pris pr kg slakt (u/distriktstilskot) = (Slakt [C27] − Herav distriktstilskot kjøt [C30]) ÷ Kg slakt totalt [C18]</t>
+          <t>Nyttbar kalv pr ku = ((Ammekyr pr 31.12. [C9] + Avlsokse pr 31.12. [C11] + Ungdyr over 12 md pr 31.12. [C13] + Kalvar/ungdyr under 12 md pr 31.12. [C15]) + Tal dyr slakta / selt til liv [C19] − Tal kjøpte dyr [C20] − (Ammekyr pr 1.1. [C8] + Avlsokse pr 1.1. [C10] + Ungdyr over 12 md pr 1.1. [C12] + Kalvar/ungdyr under 12 md pr 1.1. [C14])) ÷ Tal ammekyr [C7]   ((Dyr 31.12. + slakta/selde – kjøpte – dyr 1.1.) delt på tal ammekyr)</t>
         </is>
       </c>
       <c r="F99" s="30" t="inlineStr">
         <is>
-          <t>=IF((C18)=0,0,(C27-C30)/(C18))</t>
+          <t>=IF((C7)=0,0,((C9+C11+C13+C15)+C19-C20-(C8+C10+C12+C14))/(C7))</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="25" t="inlineStr">
         <is>
+          <t>Oppnådd pris pr kg slakt (u/distriktstilskot)</t>
+        </is>
+      </c>
+      <c r="B100" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C100" s="39">
+        <f>IF((C18)=0,0,(C27-C30)/(C18))</f>
+        <v/>
+      </c>
+      <c r="D100" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E100" s="29" t="inlineStr">
+        <is>
+          <t>Oppnådd pris pr kg slakt (u/distriktstilskot) = (Slakt [C27] − Herav distriktstilskot kjøt [C30]) ÷ Kg slakt totalt [C18]</t>
+        </is>
+      </c>
+      <c r="F100" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C18)=0,0,(C27-C30)/(C18))</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="25" t="inlineStr">
+        <is>
           <t>Analysegruppe (påsett)</t>
         </is>
       </c>
-      <c r="B100" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C100" s="41">
+      <c r="B101" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C101" s="41">
         <f>IF(C62&gt;0.5,"Påsett &gt; 50 %","Påsett &lt; 50 %")</f>
         <v/>
       </c>
-      <c r="D100" s="28" t="inlineStr">
+      <c r="D101" s="28" t="inlineStr">
         <is>
           <t>tekst</t>
         </is>
       </c>
-      <c r="E100" s="29" t="inlineStr">
+      <c r="E101" s="29" t="inlineStr">
         <is>
           <t>Analysegruppe (påsett) = HVIS(Påsettprosent [C62]&gt;0,5; "Påsett &gt; 50 %"; "Påsett &lt; 50 %")   (Tilsvarar arka «Ammekyr &lt;50%» og «Ammekyr &gt;50%» i eksempelanalysen)</t>
         </is>
       </c>
-      <c r="F100" s="30" t="inlineStr">
+      <c r="F101" s="30" t="inlineStr">
         <is>
           <t>=IF(C62&gt;0.5,"Påsett &gt; 50 %","Påsett &lt; 50 %")</t>
         </is>
@@ -25086,7 +25210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F110"/>
+  <dimension ref="A1:F111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -27647,7 +27771,7 @@
         </is>
       </c>
       <c r="C100" s="39">
-        <f>IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C61)/('Grovfôr'!C38)))=0,0,(C64)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C61)/('Grovfôr'!C38))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C61)/('Grovfôr'!C46)))=0,0,(C64)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C61)/('Grovfôr'!C46))))</f>
         <v/>
       </c>
       <c r="D100" s="28" t="inlineStr">
@@ -27657,12 +27781,12 @@
       </c>
       <c r="E100" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C64] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C21] × Sum eigen grovfôrproduksjon (utan lagerendring) [C61] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C38])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
+          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C64] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C61] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
         </is>
       </c>
       <c r="F100" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C61)/('Grovfôr'!C38)))=0,0,(C64)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C61)/('Grovfôr'!C38))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C61)/('Grovfôr'!C46)))=0,0,(C64)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C61)/('Grovfôr'!C46))))</t>
         </is>
       </c>
     </row>
@@ -27678,7 +27802,7 @@
         </is>
       </c>
       <c r="C101" s="39">
-        <f>IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C61)/('Grovfôr'!C38)))=0,0,(C65)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C61)/('Grovfôr'!C38))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C61)/('Grovfôr'!C46)))=0,0,(C65)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C61)/('Grovfôr'!C46))))</f>
         <v/>
       </c>
       <c r="D101" s="28" t="inlineStr">
@@ -27688,12 +27812,12 @@
       </c>
       <c r="E101" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C65] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C21] × Sum eigen grovfôrproduksjon (utan lagerendring) [C61] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C38])</t>
+          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C65] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C61] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])</t>
         </is>
       </c>
       <c r="F101" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C61)/('Grovfôr'!C38)))=0,0,(C65)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C61)/('Grovfôr'!C38))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C61)/('Grovfôr'!C46)))=0,0,(C65)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C61)/('Grovfôr'!C46))))</t>
         </is>
       </c>
     </row>
@@ -27709,7 +27833,7 @@
         </is>
       </c>
       <c r="C102" s="40">
-        <f>'Grovfôr'!C52</f>
+        <f>'Grovfôr'!C60</f>
         <v/>
       </c>
       <c r="D102" s="28" t="inlineStr">
@@ -27719,12 +27843,12 @@
       </c>
       <c r="E102" s="29" t="inlineStr">
         <is>
-          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C52]</t>
+          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C60]</t>
         </is>
       </c>
       <c r="F102" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C52</t>
+          <t>='Grovfôr'!C60</t>
         </is>
       </c>
     </row>
@@ -27740,7 +27864,7 @@
         </is>
       </c>
       <c r="C103" s="40">
-        <f>'Grovfôr'!C53</f>
+        <f>'Grovfôr'!C61</f>
         <v/>
       </c>
       <c r="D103" s="28" t="inlineStr">
@@ -27750,19 +27874,19 @@
       </c>
       <c r="E103" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C53]</t>
+          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C61]</t>
         </is>
       </c>
       <c r="F103" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C53</t>
+          <t>='Grovfôr'!C61</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="25" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining»</t>
+          <t>Korrigerte dekar pr «kueining» (heile garden)</t>
         </is>
       </c>
       <c r="B104" s="26" t="inlineStr">
@@ -27771,7 +27895,7 @@
         </is>
       </c>
       <c r="C104" s="40">
-        <f>'Grovfôr'!C54</f>
+        <f>'Grovfôr'!C62</f>
         <v/>
       </c>
       <c r="D104" s="28" t="inlineStr">
@@ -27781,19 +27905,19 @@
       </c>
       <c r="E104" s="29" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining» = Korrigerte dekar pr «kueining» [Grovfôr!C54]</t>
+          <t>Korrigerte dekar pr «kueining» (heile garden) = Korrigerte dekar pr «kueining» [Grovfôr!C62]</t>
         </is>
       </c>
       <c r="F104" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C54</t>
+          <t>='Grovfôr'!C62</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="25" t="inlineStr">
         <is>
-          <t>Snitt kjøtpris pr kg slakt (u/distriktstilskot)</t>
+          <t>Korrigerte dekar pr «kueining» i produksjonen</t>
         </is>
       </c>
       <c r="B105" s="26" t="inlineStr">
@@ -27802,29 +27926,29 @@
         </is>
       </c>
       <c r="C105" s="39">
-        <f>IF((C8)=0,0,(IF(C36&gt;0,C36,C31-C35))/(C8))</f>
+        <f>IF((C67)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C61)/('Grovfôr'!C46)))/(C67))</f>
         <v/>
       </c>
       <c r="D105" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>da</t>
         </is>
       </c>
       <c r="E105" s="29" t="inlineStr">
         <is>
-          <t>Snitt kjøtpris pr kg slakt (u/distriktstilskot) = (HVIS(Herav slakteinntekt til kjøtpris (3040–3046, 3048–3049) [C36]&gt;0; Herav slakteinntekt til kjøtpris (3040–3046, 3048–3049) [C36]; Slakt [C31] − Herav distriktstilskot kjøt [C35])) ÷ Kg slakt (sau og lam) [C8]</t>
+          <t>Korrigerte dekar pr «kueining» i produksjonen = (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C61] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46]) ÷ «Kueiningar» [C67]   (Grovfôrarealet produksjonen får (etter eigen grovfôrkostnad) delt på kueiningane i produksjonen)</t>
         </is>
       </c>
       <c r="F105" s="30" t="inlineStr">
         <is>
-          <t>=IF((C8)=0,0,(IF(C36&gt;0,C36,C31-C35))/(C8))</t>
+          <t>=IF((C67)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C61)/('Grovfôr'!C46)))/(C67))</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="25" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr sau</t>
+          <t>Snitt kjøtpris pr kg slakt (u/distriktstilskot)</t>
         </is>
       </c>
       <c r="B106" s="26" t="inlineStr">
@@ -27833,7 +27957,7 @@
         </is>
       </c>
       <c r="C106" s="39">
-        <f>IF((C7)=0,0,(C56)/(C7))</f>
+        <f>IF((C8)=0,0,(IF(C36&gt;0,C36,C31-C35))/(C8))</f>
         <v/>
       </c>
       <c r="D106" s="28" t="inlineStr">
@@ -27843,19 +27967,19 @@
       </c>
       <c r="E106" s="29" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr sau = Innandørsmekanisering fordelt [C56] ÷ Tal vinterfôra sau [C7]</t>
+          <t>Snitt kjøtpris pr kg slakt (u/distriktstilskot) = (HVIS(Herav slakteinntekt til kjøtpris (3040–3046, 3048–3049) [C36]&gt;0; Herav slakteinntekt til kjøtpris (3040–3046, 3048–3049) [C36]; Slakt [C31] − Herav distriktstilskot kjøt [C35])) ÷ Kg slakt (sau og lam) [C8]</t>
         </is>
       </c>
       <c r="F106" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C56)/(C7))</t>
+          <t>=IF((C8)=0,0,(IF(C36&gt;0,C36,C31-C35))/(C8))</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="25" t="inlineStr">
         <is>
-          <t>Kg slakt pr vf. sau</t>
+          <t>Innandørsmekanisering pr sau</t>
         </is>
       </c>
       <c r="B107" s="26" t="inlineStr">
@@ -27863,30 +27987,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C107" s="37">
-        <f>IF(C9&gt;0,C9,IF((C7)=0,0,(C8)/(C7)))</f>
+      <c r="C107" s="39">
+        <f>IF((C7)=0,0,(C56)/(C7))</f>
         <v/>
       </c>
       <c r="D107" s="28" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E107" s="29" t="inlineStr">
         <is>
-          <t>Kg slakt pr vf. sau = HVIS(Kg slakt pr vf. sau frå produksjonstabellen (0 = rekna ut) [C9]&gt;0; Kg slakt pr vf. sau frå produksjonstabellen (0 = rekna ut) [C9]; Kg slakt (sau og lam) [C8] ÷ Tal vinterfôra sau [C7])</t>
+          <t>Innandørsmekanisering pr sau = Innandørsmekanisering fordelt [C56] ÷ Tal vinterfôra sau [C7]</t>
         </is>
       </c>
       <c r="F107" s="30" t="inlineStr">
         <is>
-          <t>=IF(C9&gt;0,C9,IF((C7)=0,0,(C8)/(C7)))</t>
+          <t>=IF((C7)=0,0,(C56)/(C7))</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="25" t="inlineStr">
         <is>
-          <t>Gagnslam pr vf. sau</t>
+          <t>Kg slakt pr vf. sau</t>
         </is>
       </c>
       <c r="B108" s="26" t="inlineStr">
@@ -27894,30 +28018,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C108" s="39">
-        <f>IF((C7)=0,0,(C11+C18-C10)/(C7))</f>
+      <c r="C108" s="37">
+        <f>IF(C9&gt;0,C9,IF((C7)=0,0,(C8)/(C7)))</f>
         <v/>
       </c>
       <c r="D108" s="28" t="inlineStr">
         <is>
-          <t>stk</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E108" s="29" t="inlineStr">
         <is>
-          <t>Gagnslam pr vf. sau = (Tal slakta/selde årslam (mai–des) [C11] + Sau/lam under 12 md pr 31.12. (stk) [C18] − Tal kjøpte lam (mai–des) [C10]) ÷ Tal vinterfôra sau [C7]   ((Selde/slakta årslam + lam på lager 31.12. – kjøpte lam) delt på vf. sau)</t>
+          <t>Kg slakt pr vf. sau = HVIS(Kg slakt pr vf. sau frå produksjonstabellen (0 = rekna ut) [C9]&gt;0; Kg slakt pr vf. sau frå produksjonstabellen (0 = rekna ut) [C9]; Kg slakt (sau og lam) [C8] ÷ Tal vinterfôra sau [C7])</t>
         </is>
       </c>
       <c r="F108" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C11+C18-C10)/(C7))</t>
+          <t>=IF(C9&gt;0,C9,IF((C7)=0,0,(C8)/(C7)))</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="25" t="inlineStr">
         <is>
-          <t>Del dyr på utmarksbeite</t>
+          <t>Gagnslam pr vf. sau</t>
         </is>
       </c>
       <c r="B109" s="26" t="inlineStr">
@@ -27925,52 +28049,83 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C109" s="33">
-        <f>IF((C16+C17+C18+C12)=0,0,('Grovfôr'!C12+'Grovfôr'!C13)/(C16+C17+C18+C12))</f>
+      <c r="C109" s="39">
+        <f>IF((C7)=0,0,(C11+C18-C10)/(C7))</f>
         <v/>
       </c>
       <c r="D109" s="28" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>stk</t>
         </is>
       </c>
       <c r="E109" s="29" t="inlineStr">
         <is>
-          <t>Del dyr på utmarksbeite = (Sau på utmarksbeite (1,05 FEm/dag, 95 dagar) [Grovfôr!C12] + Lam på utmarksbeite (1 FEm/dag, 90 dagar) [Grovfôr!C13]) ÷ (Sauer frå inngåande balanse pr 31.12. (stk) [C16] + Sauer tilført i året pr 31.12. (stk) [C17] + Sau/lam under 12 md pr 31.12. (stk) [C18] + Tal slakta/selde sau og lam (juli–des) [C12])</t>
+          <t>Gagnslam pr vf. sau = (Tal slakta/selde årslam (mai–des) [C11] + Sau/lam under 12 md pr 31.12. (stk) [C18] − Tal kjøpte lam (mai–des) [C10]) ÷ Tal vinterfôra sau [C7]   ((Selde/slakta årslam + lam på lager 31.12. – kjøpte lam) delt på vf. sau)</t>
         </is>
       </c>
       <c r="F109" s="30" t="inlineStr">
         <is>
-          <t>=IF((C16+C17+C18+C12)=0,0,('Grovfôr'!C12+'Grovfôr'!C13)/(C16+C17+C18+C12))</t>
+          <t>=IF((C7)=0,0,(C11+C18-C10)/(C7))</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="25" t="inlineStr">
         <is>
+          <t>Del dyr på utmarksbeite</t>
+        </is>
+      </c>
+      <c r="B110" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C110" s="33">
+        <f>IF((C16+C17+C18+C12)=0,0,('Grovfôr'!C12+'Grovfôr'!C13)/(C16+C17+C18+C12))</f>
+        <v/>
+      </c>
+      <c r="D110" s="28" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E110" s="29" t="inlineStr">
+        <is>
+          <t>Del dyr på utmarksbeite = (Sau på utmarksbeite (1,05 FEm/dag, 95 dagar) [Grovfôr!C12] + Lam på utmarksbeite (1 FEm/dag, 90 dagar) [Grovfôr!C13]) ÷ (Sauer frå inngåande balanse pr 31.12. (stk) [C16] + Sauer tilført i året pr 31.12. (stk) [C17] + Sau/lam under 12 md pr 31.12. (stk) [C18] + Tal slakta/selde sau og lam (juli–des) [C12])</t>
+        </is>
+      </c>
+      <c r="F110" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C16+C17+C18+C12)=0,0,('Grovfôr'!C12+'Grovfôr'!C13)/(C16+C17+C18+C12))</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="25" t="inlineStr">
+        <is>
           <t>Endra DB pr vf. sau grunna prisendring på dyr</t>
         </is>
       </c>
-      <c r="B110" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C110" s="39">
+      <c r="B111" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C111" s="39">
         <f>ROUND(IF((C7)=0,0,(C71)/(C7)),0)</f>
         <v/>
       </c>
-      <c r="D110" s="28" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E110" s="29" t="inlineStr">
+      <c r="D111" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E111" s="29" t="inlineStr">
         <is>
           <t>Endra DB pr vf. sau grunna prisendring på dyr = AVRUND(Endring i buskapsverdi grunna prisendring [C71] ÷ Tal vinterfôra sau [C7]; 0)   (Positivt tal = auka DB fordi verdien pr dyr har gått opp)</t>
         </is>
       </c>
-      <c r="F110" s="30" t="inlineStr">
+      <c r="F111" s="30" t="inlineStr">
         <is>
           <t>=ROUND(IF((C7)=0,0,(C71)/(C7)),0)</t>
         </is>
@@ -27988,7 +28143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -30144,7 +30299,7 @@
         </is>
       </c>
       <c r="C85" s="39">
-        <f>IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C49)/('Grovfôr'!C38)))=0,0,(C52)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C49)/('Grovfôr'!C38))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C49)/('Grovfôr'!C46)))=0,0,(C52)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C49)/('Grovfôr'!C46))))</f>
         <v/>
       </c>
       <c r="D85" s="28" t="inlineStr">
@@ -30154,12 +30309,12 @@
       </c>
       <c r="E85" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C52] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C21] × Sum eigen grovfôrproduksjon (utan lagerendring) [C49] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C38])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
+          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C52] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C49] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
         </is>
       </c>
       <c r="F85" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C49)/('Grovfôr'!C38)))=0,0,(C52)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C49)/('Grovfôr'!C38))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C49)/('Grovfôr'!C46)))=0,0,(C52)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C49)/('Grovfôr'!C46))))</t>
         </is>
       </c>
     </row>
@@ -30175,7 +30330,7 @@
         </is>
       </c>
       <c r="C86" s="39">
-        <f>IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C49)/('Grovfôr'!C38)))=0,0,(C53)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C49)/('Grovfôr'!C38))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C49)/('Grovfôr'!C46)))=0,0,(C53)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C49)/('Grovfôr'!C46))))</f>
         <v/>
       </c>
       <c r="D86" s="28" t="inlineStr">
@@ -30185,12 +30340,12 @@
       </c>
       <c r="E86" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C53] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C21] × Sum eigen grovfôrproduksjon (utan lagerendring) [C49] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C38])</t>
+          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C53] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C49] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])</t>
         </is>
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C49)/('Grovfôr'!C38)))=0,0,(C53)/('Grovfôr'!C21*IF(('Grovfôr'!C38)=0,0,(C49)/('Grovfôr'!C38))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C49)/('Grovfôr'!C46)))=0,0,(C53)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C49)/('Grovfôr'!C46))))</t>
         </is>
       </c>
     </row>
@@ -30206,7 +30361,7 @@
         </is>
       </c>
       <c r="C87" s="40">
-        <f>'Grovfôr'!C52</f>
+        <f>'Grovfôr'!C60</f>
         <v/>
       </c>
       <c r="D87" s="28" t="inlineStr">
@@ -30216,12 +30371,12 @@
       </c>
       <c r="E87" s="29" t="inlineStr">
         <is>
-          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C52]</t>
+          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C60]</t>
         </is>
       </c>
       <c r="F87" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C52</t>
+          <t>='Grovfôr'!C60</t>
         </is>
       </c>
     </row>
@@ -30237,7 +30392,7 @@
         </is>
       </c>
       <c r="C88" s="40">
-        <f>'Grovfôr'!C53</f>
+        <f>'Grovfôr'!C61</f>
         <v/>
       </c>
       <c r="D88" s="28" t="inlineStr">
@@ -30247,19 +30402,19 @@
       </c>
       <c r="E88" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C53]</t>
+          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C61]</t>
         </is>
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C53</t>
+          <t>='Grovfôr'!C61</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="25" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining»</t>
+          <t>Korrigerte dekar pr «kueining» (heile garden)</t>
         </is>
       </c>
       <c r="B89" s="26" t="inlineStr">
@@ -30268,7 +30423,7 @@
         </is>
       </c>
       <c r="C89" s="40">
-        <f>'Grovfôr'!C54</f>
+        <f>'Grovfôr'!C62</f>
         <v/>
       </c>
       <c r="D89" s="28" t="inlineStr">
@@ -30278,19 +30433,19 @@
       </c>
       <c r="E89" s="29" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining» = Korrigerte dekar pr «kueining» [Grovfôr!C54]</t>
+          <t>Korrigerte dekar pr «kueining» (heile garden) = Korrigerte dekar pr «kueining» [Grovfôr!C62]</t>
         </is>
       </c>
       <c r="F89" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C54</t>
+          <t>='Grovfôr'!C62</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="25" t="inlineStr">
         <is>
-          <t>Oppnådd mjølkepris pr liter (u/distriktstilskot)</t>
+          <t>Korrigerte dekar pr «kueining» i produksjonen</t>
         </is>
       </c>
       <c r="B90" s="26" t="inlineStr">
@@ -30299,29 +30454,29 @@
         </is>
       </c>
       <c r="C90" s="39">
-        <f>IF((C8)=0,0,(C19-C24)/(C8))</f>
+        <f>IF((C55)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C49)/('Grovfôr'!C46)))/(C55))</f>
         <v/>
       </c>
       <c r="D90" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>da</t>
         </is>
       </c>
       <c r="E90" s="29" t="inlineStr">
         <is>
-          <t>Oppnådd mjølkepris pr liter (u/distriktstilskot) = (Mjølk [C19] − Herav distriktstilskot mjølk [C24]) ÷ Levert mjølk [C8]</t>
+          <t>Korrigerte dekar pr «kueining» i produksjonen = (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C49] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46]) ÷ «Kueiningar» [C55]   (Grovfôrarealet produksjonen får (etter eigen grovfôrkostnad) delt på kueiningane i produksjonen)</t>
         </is>
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>=IF((C8)=0,0,(C19-C24)/(C8))</t>
+          <t>=IF((C55)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C49)/('Grovfôr'!C46)))/(C55))</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="25" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr liter</t>
+          <t>Oppnådd mjølkepris pr liter (u/distriktstilskot)</t>
         </is>
       </c>
       <c r="B91" s="26" t="inlineStr">
@@ -30330,7 +30485,7 @@
         </is>
       </c>
       <c r="C91" s="39">
-        <f>IF((C8)=0,0,(C43)/(C8))</f>
+        <f>IF((C8)=0,0,(C19-C24)/(C8))</f>
         <v/>
       </c>
       <c r="D91" s="28" t="inlineStr">
@@ -30340,19 +30495,19 @@
       </c>
       <c r="E91" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr liter = Maskinkostnader fordelt [C43] ÷ Levert mjølk [C8]</t>
+          <t>Oppnådd mjølkepris pr liter (u/distriktstilskot) = (Mjølk [C19] − Herav distriktstilskot mjølk [C24]) ÷ Levert mjølk [C8]</t>
         </is>
       </c>
       <c r="F91" s="30" t="inlineStr">
         <is>
-          <t>=IF((C8)=0,0,(C43)/(C8))</t>
+          <t>=IF((C8)=0,0,(C19-C24)/(C8))</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="25" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr liter</t>
+          <t>Maskinkostnader pr liter</t>
         </is>
       </c>
       <c r="B92" s="26" t="inlineStr">
@@ -30361,7 +30516,7 @@
         </is>
       </c>
       <c r="C92" s="39">
-        <f>IF((C8)=0,0,(C44)/(C8))</f>
+        <f>IF((C8)=0,0,(C43)/(C8))</f>
         <v/>
       </c>
       <c r="D92" s="28" t="inlineStr">
@@ -30371,19 +30526,19 @@
       </c>
       <c r="E92" s="29" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr liter = Innandørsmekanisering fordelt [C44] ÷ Levert mjølk [C8]</t>
+          <t>Maskinkostnader pr liter = Maskinkostnader fordelt [C43] ÷ Levert mjølk [C8]</t>
         </is>
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>=IF((C8)=0,0,(C44)/(C8))</t>
+          <t>=IF((C8)=0,0,(C43)/(C8))</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="25" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr geit</t>
+          <t>Innandørsmekanisering pr liter</t>
         </is>
       </c>
       <c r="B93" s="26" t="inlineStr">
@@ -30392,7 +30547,7 @@
         </is>
       </c>
       <c r="C93" s="39">
-        <f>IF((C7)=0,0,(C44)/(C7))</f>
+        <f>IF((C8)=0,0,(C44)/(C8))</f>
         <v/>
       </c>
       <c r="D93" s="28" t="inlineStr">
@@ -30402,19 +30557,19 @@
       </c>
       <c r="E93" s="29" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr geit = Innandørsmekanisering fordelt [C44] ÷ Tal årsgeiter [C7]</t>
+          <t>Innandørsmekanisering pr liter = Innandørsmekanisering fordelt [C44] ÷ Levert mjølk [C8]</t>
         </is>
       </c>
       <c r="F93" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C44)/(C7))</t>
+          <t>=IF((C8)=0,0,(C44)/(C8))</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="25" t="inlineStr">
         <is>
-          <t>Levert mjølk pr geit (liter)</t>
+          <t>Innandørsmekanisering pr geit</t>
         </is>
       </c>
       <c r="B94" s="26" t="inlineStr">
@@ -30422,52 +30577,83 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C94" s="27">
-        <f>IF((C7)=0,0,(C8)/(C7))</f>
+      <c r="C94" s="39">
+        <f>IF((C7)=0,0,(C44)/(C7))</f>
         <v/>
       </c>
       <c r="D94" s="28" t="inlineStr">
         <is>
-          <t>liter</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E94" s="29" t="inlineStr">
         <is>
-          <t>Levert mjølk pr geit (liter) = Levert mjølk [C8] ÷ Tal årsgeiter [C7]</t>
+          <t>Innandørsmekanisering pr geit = Innandørsmekanisering fordelt [C44] ÷ Tal årsgeiter [C7]</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C8)/(C7))</t>
+          <t>=IF((C7)=0,0,(C44)/(C7))</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="25" t="inlineStr">
         <is>
+          <t>Levert mjølk pr geit (liter)</t>
+        </is>
+      </c>
+      <c r="B95" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C95" s="27">
+        <f>IF((C7)=0,0,(C8)/(C7))</f>
+        <v/>
+      </c>
+      <c r="D95" s="28" t="inlineStr">
+        <is>
+          <t>liter</t>
+        </is>
+      </c>
+      <c r="E95" s="29" t="inlineStr">
+        <is>
+          <t>Levert mjølk pr geit (liter) = Levert mjølk [C8] ÷ Tal årsgeiter [C7]</t>
+        </is>
+      </c>
+      <c r="F95" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C7)=0,0,(C8)/(C7))</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="25" t="inlineStr">
+        <is>
           <t>Kvoteoppfylling</t>
         </is>
       </c>
-      <c r="B95" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C95" s="33">
+      <c r="B96" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C96" s="33">
         <f>IF((C9)=0,0,(C8)/(C9))</f>
         <v/>
       </c>
-      <c r="D95" s="28" t="inlineStr">
+      <c r="D96" s="28" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E95" s="29" t="inlineStr">
+      <c r="E96" s="29" t="inlineStr">
         <is>
           <t>Kvoteoppfylling = Levert mjølk [C8] ÷ Disponibel mjølkekvote [C9]</t>
         </is>
       </c>
-      <c r="F95" s="30" t="inlineStr">
+      <c r="F96" s="30" t="inlineStr">
         <is>
           <t>=IF((C9)=0,0,(C8)/(C9))</t>
         </is>
@@ -41181,7 +41367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -41869,16 +42055,16 @@
     <row r="31">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>Driftsoverskot andre næringar (skog, leigekøyring o.l.)</t>
+          <t>Driftsoverskot skog/pelsdyr</t>
         </is>
       </c>
       <c r="B31" s="24" t="inlineStr">
         <is>
-          <t>Avdeling 30/70 o.l.</t>
+          <t>Avdeling 30 (skogbruk) og 50 (pelsdyr)</t>
         </is>
       </c>
       <c r="C31" s="31" t="n">
-        <v>117592.22</v>
+        <v>0</v>
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
@@ -41887,7 +42073,7 @@
       </c>
       <c r="E31" s="24" t="inlineStr">
         <is>
-          <t>Input. Hentast frå: Avdeling 30/70 o.l..</t>
+          <t>Input. Hentast frå: Avdeling 30 (skogbruk) og 50 (pelsdyr).</t>
         </is>
       </c>
       <c r="F31" s="32" t="n"/>
@@ -41895,16 +42081,16 @@
     <row r="32">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>Renteinntekter</t>
+          <t>Driftsoverskot annan næring (leigekøyring, utleige o.l.)</t>
         </is>
       </c>
       <c r="B32" s="24" t="inlineStr">
         <is>
-          <t>80xx</t>
+          <t>Andre avdelingar enn jordbruk, skog og pelsdyr</t>
         </is>
       </c>
       <c r="C32" s="31" t="n">
-        <v>117</v>
+        <v>117592.22</v>
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
@@ -41913,7 +42099,7 @@
       </c>
       <c r="E32" s="24" t="inlineStr">
         <is>
-          <t>Input. Hentast frå: 80xx.</t>
+          <t>Input. Hentast frå: Andre avdelingar enn jordbruk, skog og pelsdyr.</t>
         </is>
       </c>
       <c r="F32" s="32" t="n"/>
@@ -41921,107 +42107,102 @@
     <row r="33">
       <c r="A33" s="20" t="inlineStr">
         <is>
+          <t>Renteinntekter</t>
+        </is>
+      </c>
+      <c r="B33" s="24" t="inlineStr">
+        <is>
+          <t>80xx</t>
+        </is>
+      </c>
+      <c r="C33" s="31" t="n">
+        <v>117</v>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E33" s="24" t="inlineStr">
+        <is>
+          <t>Input. Hentast frå: 80xx.</t>
+        </is>
+      </c>
+      <c r="F33" s="32" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="20" t="inlineStr">
+        <is>
           <t>Renteutgifter</t>
         </is>
       </c>
-      <c r="B33" s="24" t="inlineStr">
+      <c r="B34" s="24" t="inlineStr">
         <is>
           <t>8100-8179</t>
         </is>
       </c>
-      <c r="C33" s="31" t="n">
+      <c r="C34" s="31" t="n">
         <v>190284.05</v>
       </c>
-      <c r="D33" s="12" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E33" s="24" t="inlineStr">
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E34" s="24" t="inlineStr">
         <is>
           <t>Input. Hentast frå: 8100-8179.</t>
         </is>
       </c>
-      <c r="F33" s="32" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="25" t="inlineStr">
+      <c r="F34" s="32" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="25" t="inlineStr">
         <is>
           <t>Nettoinntekt næring (driftsmessig)</t>
         </is>
       </c>
-      <c r="B34" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C34" s="27">
-        <f>C18+C31+C32-C33</f>
-        <v/>
-      </c>
-      <c r="D34" s="28" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E34" s="29" t="inlineStr">
-        <is>
-          <t>Nettoinntekt næring (driftsmessig) = Driftsoverskot jordbruk, driftsmessig [C18] + Driftsoverskot andre næringar (skog, leigekøyring o.l.) [C31] + Renteinntekter [C32] − Renteutgifter [C33]</t>
-        </is>
-      </c>
-      <c r="F34" s="30" t="inlineStr">
-        <is>
-          <t>=C18+C31+C32-C33</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="18" t="inlineStr">
+      <c r="B35" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C35" s="27">
+        <f>C18+C31+C32+C33-C34</f>
+        <v/>
+      </c>
+      <c r="D35" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E35" s="29" t="inlineStr">
+        <is>
+          <t>Nettoinntekt næring (driftsmessig) = Driftsoverskot jordbruk, driftsmessig [C18] + Driftsoverskot skog/pelsdyr [C31] + Driftsoverskot annan næring (leigekøyring, utleige o.l.) [C32] + Renteinntekter [C33] − Renteutgifter [C34]</t>
+        </is>
+      </c>
+      <c r="F35" s="30" t="inlineStr">
+        <is>
+          <t>=C18+C31+C32+C33-C34</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="18" t="inlineStr">
         <is>
           <t>7. OUTPUT – Nøkkeltal totaløkonomi</t>
         </is>
       </c>
-      <c r="B35" s="19" t="n"/>
-      <c r="C35" s="19" t="n"/>
-      <c r="D35" s="19" t="n"/>
-      <c r="E35" s="19" t="n"/>
-      <c r="F35" s="19" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="25" t="inlineStr">
-        <is>
-          <t>DB m/tilskot i % av produksjonsinntekter og tilskot</t>
-        </is>
-      </c>
-      <c r="B36" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C36" s="33">
-        <f>IF((C7+C10)=0,0,(C11)/(C7+C10))</f>
-        <v/>
-      </c>
-      <c r="D36" s="28" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E36" s="29" t="inlineStr">
-        <is>
-          <t>DB m/tilskot i % av produksjonsinntekter og tilskot = Sum DB med tilskot [C11] ÷ (Sum produksjonsinntekter [C7] + Sum tilskot fordelt på produksjonane [C10])</t>
-        </is>
-      </c>
-      <c r="F36" s="30" t="inlineStr">
-        <is>
-          <t>=IF((C7+C10)=0,0,(C11)/(C7+C10))</t>
-        </is>
-      </c>
+      <c r="B36" s="19" t="n"/>
+      <c r="C36" s="19" t="n"/>
+      <c r="D36" s="19" t="n"/>
+      <c r="E36" s="19" t="n"/>
+      <c r="F36" s="19" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="25" t="inlineStr">
         <is>
-          <t>Tilskot i % av DB m/tilskot</t>
+          <t>DB m/tilskot i % av produksjonsinntekter og tilskot</t>
         </is>
       </c>
       <c r="B37" s="26" t="inlineStr">
@@ -42030,7 +42211,7 @@
         </is>
       </c>
       <c r="C37" s="33">
-        <f>IF((C11)=0,0,(C10)/(C11))</f>
+        <f>IF((C7+C10)=0,0,(C11)/(C7+C10))</f>
         <v/>
       </c>
       <c r="D37" s="28" t="inlineStr">
@@ -42040,19 +42221,19 @@
       </c>
       <c r="E37" s="29" t="inlineStr">
         <is>
-          <t>Tilskot i % av DB m/tilskot = Sum tilskot fordelt på produksjonane [C10] ÷ Sum DB med tilskot [C11]</t>
+          <t>DB m/tilskot i % av produksjonsinntekter og tilskot = Sum DB med tilskot [C11] ÷ (Sum produksjonsinntekter [C7] + Sum tilskot fordelt på produksjonane [C10])</t>
         </is>
       </c>
       <c r="F37" s="30" t="inlineStr">
         <is>
-          <t>=IF((C11)=0,0,(C10)/(C11))</t>
+          <t>=IF((C7+C10)=0,0,(C11)/(C7+C10))</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="25" t="inlineStr">
         <is>
-          <t>Faste kostnader i % av DB m/tilskot</t>
+          <t>Tilskot i % av DB m/tilskot</t>
         </is>
       </c>
       <c r="B38" s="26" t="inlineStr">
@@ -42061,7 +42242,7 @@
         </is>
       </c>
       <c r="C38" s="33">
-        <f>IF((C11)=0,0,(C17)/(C11))</f>
+        <f>IF((C11)=0,0,(C10)/(C11))</f>
         <v/>
       </c>
       <c r="D38" s="28" t="inlineStr">
@@ -42071,43 +42252,74 @@
       </c>
       <c r="E38" s="29" t="inlineStr">
         <is>
-          <t>Faste kostnader i % av DB m/tilskot = Sum faste kostnader [C17] ÷ Sum DB med tilskot [C11]</t>
+          <t>Tilskot i % av DB m/tilskot = Sum tilskot fordelt på produksjonane [C10] ÷ Sum DB med tilskot [C11]</t>
         </is>
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>=IF((C11)=0,0,(C17)/(C11))</t>
+          <t>=IF((C11)=0,0,(C10)/(C11))</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="25" t="inlineStr">
         <is>
+          <t>Faste kostnader i % av DB m/tilskot</t>
+        </is>
+      </c>
+      <c r="B39" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C39" s="33">
+        <f>IF((C11)=0,0,(C17)/(C11))</f>
+        <v/>
+      </c>
+      <c r="D39" s="28" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E39" s="29" t="inlineStr">
+        <is>
+          <t>Faste kostnader i % av DB m/tilskot = Sum faste kostnader [C17] ÷ Sum DB med tilskot [C11]</t>
+        </is>
+      </c>
+      <c r="F39" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C11)=0,0,(C17)/(C11))</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="25" t="inlineStr">
+        <is>
           <t>Renteutgifter i % av driftsoverskot</t>
         </is>
       </c>
-      <c r="B39" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C39" s="33">
-        <f>IF((C18)=0,0,(C33)/(C18))</f>
-        <v/>
-      </c>
-      <c r="D39" s="28" t="inlineStr">
+      <c r="B40" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C40" s="33">
+        <f>IF((C18)=0,0,(C34)/(C18))</f>
+        <v/>
+      </c>
+      <c r="D40" s="28" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E39" s="29" t="inlineStr">
-        <is>
-          <t>Renteutgifter i % av driftsoverskot = Renteutgifter [C33] ÷ Driftsoverskot jordbruk, driftsmessig [C18]</t>
-        </is>
-      </c>
-      <c r="F39" s="30" t="inlineStr">
-        <is>
-          <t>=IF((C18)=0,0,(C33)/(C18))</t>
+      <c r="E40" s="29" t="inlineStr">
+        <is>
+          <t>Renteutgifter i % av driftsoverskot = Renteutgifter [C34] ÷ Driftsoverskot jordbruk, driftsmessig [C18]</t>
+        </is>
+      </c>
+      <c r="F40" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C18)=0,0,(C34)/(C18))</t>
         </is>
       </c>
     </row>
@@ -44902,7 +45114,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -45306,7 +45518,7 @@
     <row r="20">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t>Dekar grovfôr – maskinkostnadsgrunnlag (overflate/2 + fulldyrka + kulturbeite×10 %)</t>
+          <t>Overflatedyrka korrigert til «fulldyrka» (delt på 1,25)</t>
         </is>
       </c>
       <c r="B20" s="21" t="inlineStr">
@@ -45315,7 +45527,7 @@
         </is>
       </c>
       <c r="C20" s="36">
-        <f>C7/2+C18+C19*0.1</f>
+        <f>C7/1.25</f>
         <v/>
       </c>
       <c r="D20" s="12" t="inlineStr">
@@ -45325,81 +45537,81 @@
       </c>
       <c r="E20" s="23" t="inlineStr">
         <is>
-          <t>Dekar grovfôr – maskinkostnadsgrunnlag (overflate/2 + fulldyrka + kulturbeite×10 %) = Overflatedyrka jord til eng og beite [C7] / 2 + Fulldyrka til eigen grovfôrbasert husdyrproduksjon [C18] + Kulturbeite til eige bruk [C19] × 0,1</t>
+          <t>Overflatedyrka korrigert til «fulldyrka» (delt på 1,25) = Overflatedyrka jord til eng og beite [C7] / 1,25</t>
         </is>
       </c>
       <c r="F20" s="24" t="inlineStr">
         <is>
-          <t>=C7/2+C18+C19*0.1</t>
+          <t>=C7/1.25</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="25" t="inlineStr">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>Kulturbeite korrigert til «fulldyrka» (delt på 2,5)</t>
+        </is>
+      </c>
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C21" s="36">
+        <f>C19/2.5</f>
+        <v/>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>da</t>
+        </is>
+      </c>
+      <c r="E21" s="23" t="inlineStr">
+        <is>
+          <t>Kulturbeite korrigert til «fulldyrka» (delt på 2,5) = Kulturbeite til eige bruk [C19] / 2,5</t>
+        </is>
+      </c>
+      <c r="F21" s="24" t="inlineStr">
+        <is>
+          <t>=C19/2.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="25" t="inlineStr">
         <is>
           <t>Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5)</t>
         </is>
       </c>
-      <c r="B21" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C21" s="37">
-        <f>C7/1.25+C18+C19/2.5</f>
-        <v/>
-      </c>
-      <c r="D21" s="28" t="inlineStr">
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C22" s="37">
+        <f>C20+C18+C21</f>
+        <v/>
+      </c>
+      <c r="D22" s="28" t="inlineStr">
         <is>
           <t>da</t>
         </is>
       </c>
-      <c r="E21" s="29" t="inlineStr">
-        <is>
-          <t>Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) = Overflatedyrka jord til eng og beite [C7] / 1,25 + Fulldyrka til eigen grovfôrbasert husdyrproduksjon [C18] + Kulturbeite til eige bruk [C19] / 2,5</t>
-        </is>
-      </c>
-      <c r="F21" s="30" t="inlineStr">
-        <is>
-          <t>=C7/1.25+C18+C19/2.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="20" t="inlineStr">
-        <is>
-          <t>Fôreiningar (FEm) henta frå utmark</t>
-        </is>
-      </c>
-      <c r="B22" s="21" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C22" s="22">
-        <f>C12*1.05*95+C13*1*90+C14*7.2*92+C15*4.8*92</f>
-        <v/>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>FEm</t>
-        </is>
-      </c>
-      <c r="E22" s="23" t="inlineStr">
-        <is>
-          <t>Fôreiningar (FEm) henta frå utmark = Sau på utmarksbeite (1,05 FEm/dag, 95 dagar) [C12] × 1,05 × 95 + Lam på utmarksbeite (1 FEm/dag, 90 dagar) [C13] × 1 × 90 + Kyr på utmarksbeite (7,2 FEm/dag, 92 dagar) [C14] × 7,2 × 92 + Ungdyr på utmarksbeite (4,8 FEm/dag, 92 dagar) [C15] × 4,8 × 92</t>
-        </is>
-      </c>
-      <c r="F22" s="24" t="inlineStr">
-        <is>
-          <t>=C12*1.05*95+C13*1*90+C14*7.2*92+C15*4.8*92</t>
+      <c r="E22" s="29" t="inlineStr">
+        <is>
+          <t>Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) = Overflatedyrka korrigert til «fulldyrka» (delt på 1,25) [C20] + Fulldyrka til eigen grovfôrbasert husdyrproduksjon [C18] + Kulturbeite korrigert til «fulldyrka» (delt på 2,5) [C21]</t>
+        </is>
+      </c>
+      <c r="F22" s="30" t="inlineStr">
+        <is>
+          <t>=C20+C18+C21</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="20" t="inlineStr">
         <is>
-          <t>Utmark omrekna til «fulldyrka» dekar (900 FEm/da)</t>
+          <t>Overflatedyrka korrigert for maskinkostnader (delt på 2)</t>
         </is>
       </c>
       <c r="B23" s="21" t="inlineStr">
@@ -45408,7 +45620,7 @@
         </is>
       </c>
       <c r="C23" s="36">
-        <f>C22/900</f>
+        <f>C7/2</f>
         <v/>
       </c>
       <c r="D23" s="12" t="inlineStr">
@@ -45418,31 +45630,50 @@
       </c>
       <c r="E23" s="23" t="inlineStr">
         <is>
-          <t>Utmark omrekna til «fulldyrka» dekar (900 FEm/da) = Fôreiningar (FEm) henta frå utmark [C22] / 900</t>
+          <t>Overflatedyrka korrigert for maskinkostnader (delt på 2) = Overflatedyrka jord til eng og beite [C7] / 2</t>
         </is>
       </c>
       <c r="F23" s="24" t="inlineStr">
         <is>
-          <t>=C22/900</t>
+          <t>=C7/2</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>4. UTREKNING – «Kueiningar» og eigen grovfôrkostnad pr produksjon (berre produksjonar med i totalen)</t>
-        </is>
-      </c>
-      <c r="B24" s="19" t="n"/>
-      <c r="C24" s="19" t="n"/>
-      <c r="D24" s="19" t="n"/>
-      <c r="E24" s="19" t="n"/>
-      <c r="F24" s="19" t="n"/>
+      <c r="A24" s="20" t="inlineStr">
+        <is>
+          <t>Kulturbeite korrigert for maskinkostnader (delt på 10)</t>
+        </is>
+      </c>
+      <c r="B24" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C24" s="36">
+        <f>C19*0.1</f>
+        <v/>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>da</t>
+        </is>
+      </c>
+      <c r="E24" s="23" t="inlineStr">
+        <is>
+          <t>Kulturbeite korrigert for maskinkostnader (delt på 10) = Kulturbeite til eige bruk [C19] × 0,1</t>
+        </is>
+      </c>
+      <c r="F24" s="24" t="inlineStr">
+        <is>
+          <t>=C19*0.1</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="20" t="inlineStr">
         <is>
-          <t>Kueiningar – Mjølk</t>
+          <t>Dekar grovfôr – maskinkostnadsgrunnlag (overflate/2 + fulldyrka + kulturbeite×10 %)</t>
         </is>
       </c>
       <c r="B25" s="21" t="inlineStr">
@@ -45450,30 +45681,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C25" s="38">
-        <f>'Mjølk'!C59*IF(Oversikt!$B$16="J",1,0)</f>
+      <c r="C25" s="36">
+        <f>C23+C18+C24</f>
         <v/>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>stk</t>
+          <t>da</t>
         </is>
       </c>
       <c r="E25" s="23" t="inlineStr">
         <is>
-          <t>Kueiningar – Mjølk = «Kueiningar» [Mjølk!C59] × Med i totalen Mjølk [Oversikt!B16 → 1/0]</t>
+          <t>Dekar grovfôr – maskinkostnadsgrunnlag (overflate/2 + fulldyrka + kulturbeite×10 %) = Overflatedyrka korrigert for maskinkostnader (delt på 2) [C23] + Fulldyrka til eigen grovfôrbasert husdyrproduksjon [C18] + Kulturbeite korrigert for maskinkostnader (delt på 10) [C24]</t>
         </is>
       </c>
       <c r="F25" s="24" t="inlineStr">
         <is>
-          <t>='Mjølk'!C59*IF(Oversikt!$B$16="J",1,0)</t>
+          <t>=C23+C18+C24</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="20" t="inlineStr">
         <is>
-          <t>Kueiningar – Oksar</t>
+          <t>Småfe på utmarksbeite</t>
         </is>
       </c>
       <c r="B26" s="21" t="inlineStr">
@@ -45481,8 +45712,8 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C26" s="38">
-        <f>Oksar!C56*IF(Oversikt!$B$17="J",1,0)</f>
+      <c r="C26" s="22">
+        <f>C12+C13</f>
         <v/>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -45492,19 +45723,19 @@
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
-          <t>Kueiningar – Oksar = «Kueiningar» [Oksar!C56] × Med i totalen Oksar [Oversikt!B17 → 1/0]</t>
+          <t>Småfe på utmarksbeite = Sau på utmarksbeite (1,05 FEm/dag, 95 dagar) [C12] + Lam på utmarksbeite (1 FEm/dag, 90 dagar) [C13]</t>
         </is>
       </c>
       <c r="F26" s="24" t="inlineStr">
         <is>
-          <t>=Oksar!C56*IF(Oversikt!$B$17="J",1,0)</t>
+          <t>=C12+C13</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="20" t="inlineStr">
         <is>
-          <t>Kueiningar – Mellomkalv</t>
+          <t>Storfe på utmarksbeite</t>
         </is>
       </c>
       <c r="B27" s="21" t="inlineStr">
@@ -45512,8 +45743,8 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C27" s="38">
-        <f>Mellomkalv!C56*IF(Oversikt!$B$18="J",1,0)</f>
+      <c r="C27" s="22">
+        <f>C14+C15</f>
         <v/>
       </c>
       <c r="D27" s="12" t="inlineStr">
@@ -45523,19 +45754,19 @@
       </c>
       <c r="E27" s="23" t="inlineStr">
         <is>
-          <t>Kueiningar – Mellomkalv = «Kueiningar» [Mellomkalv!C56] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0]</t>
+          <t>Storfe på utmarksbeite = Kyr på utmarksbeite (7,2 FEm/dag, 92 dagar) [C14] + Ungdyr på utmarksbeite (4,8 FEm/dag, 92 dagar) [C15]</t>
         </is>
       </c>
       <c r="F27" s="24" t="inlineStr">
         <is>
-          <t>=Mellomkalv!C56*IF(Oversikt!$B$18="J",1,0)</t>
+          <t>=C14+C15</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>Kueiningar – Ammekyr</t>
+          <t>Fôreiningar (FEm) henta frå utmark</t>
         </is>
       </c>
       <c r="B28" s="21" t="inlineStr">
@@ -45543,30 +45774,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C28" s="38">
-        <f>Ammekyr!C61*IF(Oversikt!$B$19="J",1,0)</f>
+      <c r="C28" s="22">
+        <f>C12*1.05*95+C13*1*90+C14*7.2*92+C15*4.8*92</f>
         <v/>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>stk</t>
+          <t>FEm</t>
         </is>
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
-          <t>Kueiningar – Ammekyr = «Kueiningar» [Ammekyr!C61] × Med i totalen Ammekyr [Oversikt!B19 → 1/0]</t>
+          <t>Fôreiningar (FEm) henta frå utmark = Sau på utmarksbeite (1,05 FEm/dag, 95 dagar) [C12] × 1,05 × 95 + Lam på utmarksbeite (1 FEm/dag, 90 dagar) [C13] × 1 × 90 + Kyr på utmarksbeite (7,2 FEm/dag, 92 dagar) [C14] × 7,2 × 92 + Ungdyr på utmarksbeite (4,8 FEm/dag, 92 dagar) [C15] × 4,8 × 92</t>
         </is>
       </c>
       <c r="F28" s="24" t="inlineStr">
         <is>
-          <t>=Ammekyr!C61*IF(Oversikt!$B$19="J",1,0)</t>
+          <t>=C12*1.05*95+C13*1*90+C14*7.2*92+C15*4.8*92</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>Kueiningar – Sau</t>
+          <t>Utmark omrekna til «fulldyrka» dekar (900 FEm/da)</t>
         </is>
       </c>
       <c r="B29" s="21" t="inlineStr">
@@ -45574,92 +45805,73 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C29" s="38">
-        <f>Sau!C67*IF(Oversikt!$B$23="J",1,0)</f>
+      <c r="C29" s="36">
+        <f>C28/900</f>
         <v/>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
+          <t>da</t>
+        </is>
+      </c>
+      <c r="E29" s="23" t="inlineStr">
+        <is>
+          <t>Utmark omrekna til «fulldyrka» dekar (900 FEm/da) = Fôreiningar (FEm) henta frå utmark [C28] / 900</t>
+        </is>
+      </c>
+      <c r="F29" s="24" t="inlineStr">
+        <is>
+          <t>=C28/900</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="18" t="inlineStr">
+        <is>
+          <t>4. UTREKNING – «Kueiningar» og eigen grovfôrkostnad pr produksjon (berre produksjonar med i totalen)</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="n"/>
+      <c r="C30" s="19" t="n"/>
+      <c r="D30" s="19" t="n"/>
+      <c r="E30" s="19" t="n"/>
+      <c r="F30" s="19" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t>Kueiningar – Mjølk</t>
+        </is>
+      </c>
+      <c r="B31" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C31" s="38">
+        <f>'Mjølk'!C59*IF(Oversikt!$B$16="J",1,0)</f>
+        <v/>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
           <t>stk</t>
         </is>
       </c>
-      <c r="E29" s="23" t="inlineStr">
-        <is>
-          <t>Kueiningar – Sau = «Kueiningar» [Sau!C67] × Med i totalen Sau [Oversikt!B23 → 1/0]</t>
-        </is>
-      </c>
-      <c r="F29" s="24" t="inlineStr">
-        <is>
-          <t>=Sau!C67*IF(Oversikt!$B$23="J",1,0)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="20" t="inlineStr">
-        <is>
-          <t>Kueiningar – Geit</t>
-        </is>
-      </c>
-      <c r="B30" s="21" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C30" s="38">
-        <f>Geit!C55*IF(Oversikt!$B$24="J",1,0)</f>
-        <v/>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
-        <is>
-          <t>stk</t>
-        </is>
-      </c>
-      <c r="E30" s="23" t="inlineStr">
-        <is>
-          <t>Kueiningar – Geit = «Kueiningar» [Geit!C55] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
-        </is>
-      </c>
-      <c r="F30" s="24" t="inlineStr">
-        <is>
-          <t>=Geit!C55*IF(Oversikt!$B$24="J",1,0)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="25" t="inlineStr">
-        <is>
-          <t>Sum «kueiningar»</t>
-        </is>
-      </c>
-      <c r="B31" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C31" s="39">
-        <f>C25+C26+C27+C28+C29+C30</f>
-        <v/>
-      </c>
-      <c r="D31" s="28" t="inlineStr">
-        <is>
-          <t>stk</t>
-        </is>
-      </c>
-      <c r="E31" s="29" t="inlineStr">
-        <is>
-          <t>Sum «kueiningar» = Kueiningar – Mjølk [C25] + Kueiningar – Oksar [C26] + Kueiningar – Mellomkalv [C27] + Kueiningar – Ammekyr [C28] + Kueiningar – Sau [C29] + Kueiningar – Geit [C30]</t>
-        </is>
-      </c>
-      <c r="F31" s="30" t="inlineStr">
-        <is>
-          <t>=C25+C26+C27+C28+C29+C30</t>
+      <c r="E31" s="23" t="inlineStr">
+        <is>
+          <t>Kueiningar – Mjølk = «Kueiningar» [Mjølk!C59] × Med i totalen Mjølk [Oversikt!B16 → 1/0]</t>
+        </is>
+      </c>
+      <c r="F31" s="24" t="inlineStr">
+        <is>
+          <t>='Mjølk'!C59*IF(Oversikt!$B$16="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Mjølk</t>
+          <t>Kueiningar – Oksar</t>
         </is>
       </c>
       <c r="B32" s="21" t="inlineStr">
@@ -45667,30 +45879,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C32" s="22">
-        <f>'Mjølk'!C53*IF(Oversikt!$B$16="J",1,0)</f>
+      <c r="C32" s="38">
+        <f>Oksar!C56*IF(Oversikt!$B$17="J",1,0)</f>
         <v/>
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>stk</t>
         </is>
       </c>
       <c r="E32" s="23" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Mjølk = Sum eigen grovfôrproduksjon (utan lagerendring) [Mjølk!C53] × Med i totalen Mjølk [Oversikt!B16 → 1/0]</t>
+          <t>Kueiningar – Oksar = «Kueiningar» [Oksar!C56] × Med i totalen Oksar [Oversikt!B17 → 1/0]</t>
         </is>
       </c>
       <c r="F32" s="24" t="inlineStr">
         <is>
-          <t>='Mjølk'!C53*IF(Oversikt!$B$16="J",1,0)</t>
+          <t>=Oksar!C56*IF(Oversikt!$B$17="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Oksar</t>
+          <t>Kueiningar – Mellomkalv</t>
         </is>
       </c>
       <c r="B33" s="21" t="inlineStr">
@@ -45698,30 +45910,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C33" s="22">
-        <f>Oksar!C50*IF(Oversikt!$B$17="J",1,0)</f>
+      <c r="C33" s="38">
+        <f>Mellomkalv!C56*IF(Oversikt!$B$18="J",1,0)</f>
         <v/>
       </c>
       <c r="D33" s="12" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>stk</t>
         </is>
       </c>
       <c r="E33" s="23" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Oksar = Sum eigen grovfôrproduksjon (utan lagerendring) [Oksar!C50] × Med i totalen Oksar [Oversikt!B17 → 1/0]</t>
+          <t>Kueiningar – Mellomkalv = «Kueiningar» [Mellomkalv!C56] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0]</t>
         </is>
       </c>
       <c r="F33" s="24" t="inlineStr">
         <is>
-          <t>=Oksar!C50*IF(Oversikt!$B$17="J",1,0)</t>
+          <t>=Mellomkalv!C56*IF(Oversikt!$B$18="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Mellomkalv</t>
+          <t>Kueiningar – Ammekyr</t>
         </is>
       </c>
       <c r="B34" s="21" t="inlineStr">
@@ -45729,30 +45941,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C34" s="22">
-        <f>Mellomkalv!C50*IF(Oversikt!$B$18="J",1,0)</f>
+      <c r="C34" s="38">
+        <f>Ammekyr!C61*IF(Oversikt!$B$19="J",1,0)</f>
         <v/>
       </c>
       <c r="D34" s="12" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>stk</t>
         </is>
       </c>
       <c r="E34" s="23" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Mellomkalv = Sum eigen grovfôrproduksjon (utan lagerendring) [Mellomkalv!C50] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0]</t>
+          <t>Kueiningar – Ammekyr = «Kueiningar» [Ammekyr!C61] × Med i totalen Ammekyr [Oversikt!B19 → 1/0]</t>
         </is>
       </c>
       <c r="F34" s="24" t="inlineStr">
         <is>
-          <t>=Mellomkalv!C50*IF(Oversikt!$B$18="J",1,0)</t>
+          <t>=Ammekyr!C61*IF(Oversikt!$B$19="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Ammekyr</t>
+          <t>Kueiningar – Sau</t>
         </is>
       </c>
       <c r="B35" s="21" t="inlineStr">
@@ -45760,30 +45972,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C35" s="22">
-        <f>Ammekyr!C55*IF(Oversikt!$B$19="J",1,0)</f>
+      <c r="C35" s="38">
+        <f>Sau!C67*IF(Oversikt!$B$23="J",1,0)</f>
         <v/>
       </c>
       <c r="D35" s="12" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>stk</t>
         </is>
       </c>
       <c r="E35" s="23" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Ammekyr = Sum eigen grovfôrproduksjon (utan lagerendring) [Ammekyr!C55] × Med i totalen Ammekyr [Oversikt!B19 → 1/0]</t>
+          <t>Kueiningar – Sau = «Kueiningar» [Sau!C67] × Med i totalen Sau [Oversikt!B23 → 1/0]</t>
         </is>
       </c>
       <c r="F35" s="24" t="inlineStr">
         <is>
-          <t>=Ammekyr!C55*IF(Oversikt!$B$19="J",1,0)</t>
+          <t>=Sau!C67*IF(Oversikt!$B$23="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Sau</t>
+          <t>Kueiningar – Geit</t>
         </is>
       </c>
       <c r="B36" s="21" t="inlineStr">
@@ -45791,30 +46003,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C36" s="22">
-        <f>Sau!C61*IF(Oversikt!$B$23="J",1,0)</f>
+      <c r="C36" s="38">
+        <f>Geit!C55*IF(Oversikt!$B$24="J",1,0)</f>
         <v/>
       </c>
       <c r="D36" s="12" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>stk</t>
         </is>
       </c>
       <c r="E36" s="23" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Sau = Sum eigen grovfôrproduksjon (utan lagerendring) [Sau!C61] × Med i totalen Sau [Oversikt!B23 → 1/0]</t>
+          <t>Kueiningar – Geit = «Kueiningar» [Geit!C55] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
         </is>
       </c>
       <c r="F36" s="24" t="inlineStr">
         <is>
-          <t>=Sau!C61*IF(Oversikt!$B$23="J",1,0)</t>
+          <t>=Geit!C55*IF(Oversikt!$B$24="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Geit</t>
+          <t>Kueiningar – storfe</t>
         </is>
       </c>
       <c r="B37" s="21" t="inlineStr">
@@ -45822,30 +46034,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C37" s="22">
-        <f>Geit!C49*IF(Oversikt!$B$24="J",1,0)</f>
+      <c r="C37" s="38">
+        <f>C31+C32+C33+C34</f>
         <v/>
       </c>
       <c r="D37" s="12" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>stk</t>
         </is>
       </c>
       <c r="E37" s="23" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Geit = Sum eigen grovfôrproduksjon (utan lagerendring) [Geit!C49] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
+          <t>Kueiningar – storfe = Kueiningar – Mjølk [C31] + Kueiningar – Oksar [C32] + Kueiningar – Mellomkalv [C33] + Kueiningar – Ammekyr [C34]</t>
         </is>
       </c>
       <c r="F37" s="24" t="inlineStr">
         <is>
-          <t>=Geit!C49*IF(Oversikt!$B$24="J",1,0)</t>
+          <t>=C31+C32+C33+C34</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>Sum eigen grovfôrkostnad (fordelingsnøkkel areal)</t>
+          <t>Kueiningar – småfe</t>
         </is>
       </c>
       <c r="B38" s="21" t="inlineStr">
@@ -45853,61 +46065,61 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C38" s="22">
-        <f>C32+C33+C34+C35+C36+C37</f>
+      <c r="C38" s="38">
+        <f>C35+C36</f>
         <v/>
       </c>
       <c r="D38" s="12" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>stk</t>
         </is>
       </c>
       <c r="E38" s="23" t="inlineStr">
         <is>
-          <t>Sum eigen grovfôrkostnad (fordelingsnøkkel areal) = Eigen grovfôrkostnad – Mjølk [C32] + Eigen grovfôrkostnad – Oksar [C33] + Eigen grovfôrkostnad – Mellomkalv [C34] + Eigen grovfôrkostnad – Ammekyr [C35] + Eigen grovfôrkostnad – Sau [C36] + Eigen grovfôrkostnad – Geit [C37]</t>
+          <t>Kueiningar – småfe = Kueiningar – Sau [C35] + Kueiningar – Geit [C36]</t>
         </is>
       </c>
       <c r="F38" s="24" t="inlineStr">
         <is>
-          <t>=C32+C33+C34+C35+C36+C37</t>
+          <t>=C35+C36</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="20" t="inlineStr">
-        <is>
-          <t>Sum variabel grovfôrkostnad (utan plast)</t>
-        </is>
-      </c>
-      <c r="B39" s="21" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C39" s="22">
-        <f>'Mjølk'!C52*IF(Oversikt!$B$16="J",1,0)+Oksar!C49*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C49*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C54*IF(Oversikt!$B$19="J",1,0)+Sau!C60*IF(Oversikt!$B$23="J",1,0)+Geit!C48*IF(Oversikt!$B$24="J",1,0)</f>
-        <v/>
-      </c>
-      <c r="D39" s="12" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E39" s="23" t="inlineStr">
-        <is>
-          <t>Sum variabel grovfôrkostnad (utan plast) = Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Mjølk!C52] × Med i totalen Mjølk [Oversikt!B16 → 1/0] + Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Oksar!C49] × Med i totalen Oksar [Oversikt!B17 → 1/0] + Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Mellomkalv!C49] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0] + Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Ammekyr!C54] × Med i totalen Ammekyr [Oversikt!B19 → 1/0] + Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Sau!C60] × Med i totalen Sau [Oversikt!B23 → 1/0] + Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Geit!C48] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
-        </is>
-      </c>
-      <c r="F39" s="24" t="inlineStr">
-        <is>
-          <t>='Mjølk'!C52*IF(Oversikt!$B$16="J",1,0)+Oksar!C49*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C49*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C54*IF(Oversikt!$B$19="J",1,0)+Sau!C60*IF(Oversikt!$B$23="J",1,0)+Geit!C48*IF(Oversikt!$B$24="J",1,0)</t>
+      <c r="A39" s="25" t="inlineStr">
+        <is>
+          <t>Sum «kueiningar»</t>
+        </is>
+      </c>
+      <c r="B39" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C39" s="39">
+        <f>C37+C38</f>
+        <v/>
+      </c>
+      <c r="D39" s="28" t="inlineStr">
+        <is>
+          <t>stk</t>
+        </is>
+      </c>
+      <c r="E39" s="29" t="inlineStr">
+        <is>
+          <t>Sum «kueiningar» = Kueiningar – storfe [C37] + Kueiningar – småfe [C38]</t>
+        </is>
+      </c>
+      <c r="F39" s="30" t="inlineStr">
+        <is>
+          <t>=C37+C38</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>Maskinkostnader i grovfôrproduksjonane</t>
+          <t>Eigen grovfôrkostnad – Mjølk</t>
         </is>
       </c>
       <c r="B40" s="21" t="inlineStr">
@@ -45916,7 +46128,7 @@
         </is>
       </c>
       <c r="C40" s="22">
-        <f>'Faste kostnader'!C46*IF(Oversikt!$B$16="J",1,0)+'Faste kostnader'!C47*IF(Oversikt!$B$17="J",1,0)+'Faste kostnader'!C48*IF(Oversikt!$B$18="J",1,0)+'Faste kostnader'!C49*IF(Oversikt!$B$19="J",1,0)+'Faste kostnader'!C53*IF(Oversikt!$B$23="J",1,0)+'Faste kostnader'!C54*IF(Oversikt!$B$24="J",1,0)</f>
+        <f>'Mjølk'!C53*IF(Oversikt!$B$16="J",1,0)</f>
         <v/>
       </c>
       <c r="D40" s="12" t="inlineStr">
@@ -45926,19 +46138,19 @@
       </c>
       <c r="E40" s="23" t="inlineStr">
         <is>
-          <t>Maskinkostnader i grovfôrproduksjonane = Maskinkostnader – Mjølk [Faste kostnader!C46] × Med i totalen Mjølk [Oversikt!B16 → 1/0] + Maskinkostnader – Oksar [Faste kostnader!C47] × Med i totalen Oksar [Oversikt!B17 → 1/0] + Maskinkostnader – Mellomkalv [Faste kostnader!C48] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0] + Maskinkostnader – Ammekyr [Faste kostnader!C49] × Med i totalen Ammekyr [Oversikt!B19 → 1/0] + Maskinkostnader – Sau [Faste kostnader!C53] × Med i totalen Sau [Oversikt!B23 → 1/0] + Maskinkostnader – Geit [Faste kostnader!C54] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
+          <t>Eigen grovfôrkostnad – Mjølk = Sum eigen grovfôrproduksjon (utan lagerendring) [Mjølk!C53] × Med i totalen Mjølk [Oversikt!B16 → 1/0]</t>
         </is>
       </c>
       <c r="F40" s="24" t="inlineStr">
         <is>
-          <t>='Faste kostnader'!C46*IF(Oversikt!$B$16="J",1,0)+'Faste kostnader'!C47*IF(Oversikt!$B$17="J",1,0)+'Faste kostnader'!C48*IF(Oversikt!$B$18="J",1,0)+'Faste kostnader'!C49*IF(Oversikt!$B$19="J",1,0)+'Faste kostnader'!C53*IF(Oversikt!$B$23="J",1,0)+'Faste kostnader'!C54*IF(Oversikt!$B$24="J",1,0)</t>
+          <t>='Mjølk'!C53*IF(Oversikt!$B$16="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>DB grovfôrbaserte husdyr u/tilskot</t>
+          <t>Eigen grovfôrkostnad – Oksar</t>
         </is>
       </c>
       <c r="B41" s="21" t="inlineStr">
@@ -45947,7 +46159,7 @@
         </is>
       </c>
       <c r="C41" s="22">
-        <f>'Mjølk'!C56*IF(Oversikt!$B$16="J",1,0)+Oksar!C53*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C53*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C58*IF(Oversikt!$B$19="J",1,0)+Sau!C64*IF(Oversikt!$B$23="J",1,0)+Geit!C52*IF(Oversikt!$B$24="J",1,0)</f>
+        <f>Oksar!C50*IF(Oversikt!$B$17="J",1,0)</f>
         <v/>
       </c>
       <c r="D41" s="12" t="inlineStr">
@@ -45957,19 +46169,19 @@
       </c>
       <c r="E41" s="23" t="inlineStr">
         <is>
-          <t>DB grovfôrbaserte husdyr u/tilskot = Dekningsbidrag (DB) utan tilskot [Mjølk!C56] × Med i totalen Mjølk [Oversikt!B16 → 1/0] + Dekningsbidrag (DB) utan tilskot [Oksar!C53] × Med i totalen Oksar [Oversikt!B17 → 1/0] + Dekningsbidrag (DB) utan tilskot [Mellomkalv!C53] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0] + Dekningsbidrag (DB) utan tilskot [Ammekyr!C58] × Med i totalen Ammekyr [Oversikt!B19 → 1/0] + Dekningsbidrag (DB) utan tilskot [Sau!C64] × Med i totalen Sau [Oversikt!B23 → 1/0] + Dekningsbidrag (DB) utan tilskot [Geit!C52] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
+          <t>Eigen grovfôrkostnad – Oksar = Sum eigen grovfôrproduksjon (utan lagerendring) [Oksar!C50] × Med i totalen Oksar [Oversikt!B17 → 1/0]</t>
         </is>
       </c>
       <c r="F41" s="24" t="inlineStr">
         <is>
-          <t>='Mjølk'!C56*IF(Oversikt!$B$16="J",1,0)+Oksar!C53*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C53*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C58*IF(Oversikt!$B$19="J",1,0)+Sau!C64*IF(Oversikt!$B$23="J",1,0)+Geit!C52*IF(Oversikt!$B$24="J",1,0)</t>
+          <t>=Oksar!C50*IF(Oversikt!$B$17="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>DB grovfôrbaserte husdyr m/tilskot</t>
+          <t>Eigen grovfôrkostnad – Mellomkalv</t>
         </is>
       </c>
       <c r="B42" s="21" t="inlineStr">
@@ -45978,7 +46190,7 @@
         </is>
       </c>
       <c r="C42" s="22">
-        <f>'Mjølk'!C57*IF(Oversikt!$B$16="J",1,0)+Oksar!C54*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C54*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C59*IF(Oversikt!$B$19="J",1,0)+Sau!C65*IF(Oversikt!$B$23="J",1,0)+Geit!C53*IF(Oversikt!$B$24="J",1,0)</f>
+        <f>Mellomkalv!C50*IF(Oversikt!$B$18="J",1,0)</f>
         <v/>
       </c>
       <c r="D42" s="12" t="inlineStr">
@@ -45988,31 +46200,50 @@
       </c>
       <c r="E42" s="23" t="inlineStr">
         <is>
-          <t>DB grovfôrbaserte husdyr m/tilskot = Dekningsbidrag (DB) med tilskot [Mjølk!C57] × Med i totalen Mjølk [Oversikt!B16 → 1/0] + Dekningsbidrag (DB) med tilskot [Oksar!C54] × Med i totalen Oksar [Oversikt!B17 → 1/0] + Dekningsbidrag (DB) med tilskot [Mellomkalv!C54] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0] + Dekningsbidrag (DB) med tilskot [Ammekyr!C59] × Med i totalen Ammekyr [Oversikt!B19 → 1/0] + Dekningsbidrag (DB) med tilskot [Sau!C65] × Med i totalen Sau [Oversikt!B23 → 1/0] + Dekningsbidrag (DB) med tilskot [Geit!C53] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
+          <t>Eigen grovfôrkostnad – Mellomkalv = Sum eigen grovfôrproduksjon (utan lagerendring) [Mellomkalv!C50] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0]</t>
         </is>
       </c>
       <c r="F42" s="24" t="inlineStr">
         <is>
-          <t>='Mjølk'!C57*IF(Oversikt!$B$16="J",1,0)+Oksar!C54*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C54*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C59*IF(Oversikt!$B$19="J",1,0)+Sau!C65*IF(Oversikt!$B$23="J",1,0)+Geit!C53*IF(Oversikt!$B$24="J",1,0)</t>
+          <t>=Mellomkalv!C50*IF(Oversikt!$B$18="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="18" t="inlineStr">
-        <is>
-          <t>4b. UTREKNING – Arealbehov etter fôrnorm (kontroll av grovfôrbalansen)</t>
-        </is>
-      </c>
-      <c r="B43" s="19" t="n"/>
-      <c r="C43" s="19" t="n"/>
-      <c r="D43" s="19" t="n"/>
-      <c r="E43" s="19" t="n"/>
-      <c r="F43" s="19" t="n"/>
+      <c r="A43" s="20" t="inlineStr">
+        <is>
+          <t>Eigen grovfôrkostnad – Ammekyr</t>
+        </is>
+      </c>
+      <c r="B43" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C43" s="22">
+        <f>Ammekyr!C55*IF(Oversikt!$B$19="J",1,0)</f>
+        <v/>
+      </c>
+      <c r="D43" s="12" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E43" s="23" t="inlineStr">
+        <is>
+          <t>Eigen grovfôrkostnad – Ammekyr = Sum eigen grovfôrproduksjon (utan lagerendring) [Ammekyr!C55] × Med i totalen Ammekyr [Oversikt!B19 → 1/0]</t>
+        </is>
+      </c>
+      <c r="F43" s="24" t="inlineStr">
+        <is>
+          <t>=Ammekyr!C55*IF(Oversikt!$B$19="J",1,0)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Mjølk</t>
+          <t>Eigen grovfôrkostnad – Sau</t>
         </is>
       </c>
       <c r="B44" s="21" t="inlineStr">
@@ -46020,30 +46251,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C44" s="36">
-        <f>'Mjølk'!C7*('Mjølk'!C17/625+'Mjølk'!C18/650)*IF(Oversikt!$B$16="J",1,0)</f>
+      <c r="C44" s="22">
+        <f>Sau!C61*IF(Oversikt!$B$23="J",1,0)</f>
         <v/>
       </c>
       <c r="D44" s="12" t="inlineStr">
         <is>
-          <t>da</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E44" s="23" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Mjølk = Tal årskyr [Mjølk!C7] × (Fôrnorm beite (FEm) [Mjølk!C17] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Mjølk!C18] / 650) × Med i totalen Mjølk [Oversikt!B16 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
+          <t>Eigen grovfôrkostnad – Sau = Sum eigen grovfôrproduksjon (utan lagerendring) [Sau!C61] × Med i totalen Sau [Oversikt!B23 → 1/0]</t>
         </is>
       </c>
       <c r="F44" s="24" t="inlineStr">
         <is>
-          <t>='Mjølk'!C7*('Mjølk'!C17/625+'Mjølk'!C18/650)*IF(Oversikt!$B$16="J",1,0)</t>
+          <t>=Sau!C61*IF(Oversikt!$B$23="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Oksar</t>
+          <t>Eigen grovfôrkostnad – Geit</t>
         </is>
       </c>
       <c r="B45" s="21" t="inlineStr">
@@ -46051,30 +46282,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C45" s="36">
-        <f>Oksar!C7*(Oksar!C16/625+Oksar!C17/650)*IF(Oversikt!$B$17="J",1,0)</f>
+      <c r="C45" s="22">
+        <f>Geit!C49*IF(Oversikt!$B$24="J",1,0)</f>
         <v/>
       </c>
       <c r="D45" s="12" t="inlineStr">
         <is>
-          <t>da</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E45" s="23" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Oksar = Tal produserte oksar [Oksar!C7] × (Fôrnorm beite (FEm) [Oksar!C16] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Oksar!C17] / 650) × Med i totalen Oksar [Oversikt!B17 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
+          <t>Eigen grovfôrkostnad – Geit = Sum eigen grovfôrproduksjon (utan lagerendring) [Geit!C49] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
         </is>
       </c>
       <c r="F45" s="24" t="inlineStr">
         <is>
-          <t>=Oksar!C7*(Oksar!C16/625+Oksar!C17/650)*IF(Oversikt!$B$17="J",1,0)</t>
+          <t>=Geit!C49*IF(Oversikt!$B$24="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Mellomkalv</t>
+          <t>Sum eigen grovfôrkostnad (fordelingsnøkkel areal)</t>
         </is>
       </c>
       <c r="B46" s="21" t="inlineStr">
@@ -46082,30 +46313,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C46" s="36">
-        <f>Mellomkalv!C7*(Mellomkalv!C16/625+Mellomkalv!C17/650)*IF(Oversikt!$B$18="J",1,0)</f>
+      <c r="C46" s="22">
+        <f>C40+C41+C42+C43+C44+C45</f>
         <v/>
       </c>
       <c r="D46" s="12" t="inlineStr">
         <is>
-          <t>da</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E46" s="23" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Mellomkalv = Tal produserte kalvar [Mellomkalv!C7] × (Fôrnorm beite (FEm) [Mellomkalv!C16] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Mellomkalv!C17] / 650) × Med i totalen Mellomkalv [Oversikt!B18 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
+          <t>Sum eigen grovfôrkostnad (fordelingsnøkkel areal) = Eigen grovfôrkostnad – Mjølk [C40] + Eigen grovfôrkostnad – Oksar [C41] + Eigen grovfôrkostnad – Mellomkalv [C42] + Eigen grovfôrkostnad – Ammekyr [C43] + Eigen grovfôrkostnad – Sau [C44] + Eigen grovfôrkostnad – Geit [C45]</t>
         </is>
       </c>
       <c r="F46" s="24" t="inlineStr">
         <is>
-          <t>=Mellomkalv!C7*(Mellomkalv!C16/625+Mellomkalv!C17/650)*IF(Oversikt!$B$18="J",1,0)</t>
+          <t>=C40+C41+C42+C43+C44+C45</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Ammekyr</t>
+          <t>Sum variabel grovfôrkostnad (utan plast)</t>
         </is>
       </c>
       <c r="B47" s="21" t="inlineStr">
@@ -46113,30 +46344,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C47" s="36">
-        <f>Ammekyr!C7*(Ammekyr!C21/625+Ammekyr!C22/650)*IF(Oversikt!$B$19="J",1,0)</f>
+      <c r="C47" s="22">
+        <f>'Mjølk'!C52*IF(Oversikt!$B$16="J",1,0)+Oksar!C49*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C49*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C54*IF(Oversikt!$B$19="J",1,0)+Sau!C60*IF(Oversikt!$B$23="J",1,0)+Geit!C48*IF(Oversikt!$B$24="J",1,0)</f>
         <v/>
       </c>
       <c r="D47" s="12" t="inlineStr">
         <is>
-          <t>da</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E47" s="23" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Ammekyr = Tal ammekyr [Ammekyr!C7] × (Fôrnorm beite (FEm) [Ammekyr!C21] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Ammekyr!C22] / 650) × Med i totalen Ammekyr [Oversikt!B19 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
+          <t>Sum variabel grovfôrkostnad (utan plast) = Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Mjølk!C52] × Med i totalen Mjølk [Oversikt!B16 → 1/0] + Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Oksar!C49] × Med i totalen Oksar [Oversikt!B17 → 1/0] + Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Mellomkalv!C49] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0] + Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Ammekyr!C54] × Med i totalen Ammekyr [Oversikt!B19 → 1/0] + Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Sau!C60] × Med i totalen Sau [Oversikt!B23 → 1/0] + Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Geit!C48] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
         </is>
       </c>
       <c r="F47" s="24" t="inlineStr">
         <is>
-          <t>=Ammekyr!C7*(Ammekyr!C21/625+Ammekyr!C22/650)*IF(Oversikt!$B$19="J",1,0)</t>
+          <t>='Mjølk'!C52*IF(Oversikt!$B$16="J",1,0)+Oksar!C49*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C49*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C54*IF(Oversikt!$B$19="J",1,0)+Sau!C60*IF(Oversikt!$B$23="J",1,0)+Geit!C48*IF(Oversikt!$B$24="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Sau</t>
+          <t>Maskinkostnader i grovfôrproduksjonane</t>
         </is>
       </c>
       <c r="B48" s="21" t="inlineStr">
@@ -46144,30 +46375,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C48" s="36">
-        <f>Sau!C7*(Sau!C25/625+Sau!C26/650)*IF(Oversikt!$B$23="J",1,0)</f>
+      <c r="C48" s="22">
+        <f>'Faste kostnader'!C46*IF(Oversikt!$B$16="J",1,0)+'Faste kostnader'!C47*IF(Oversikt!$B$17="J",1,0)+'Faste kostnader'!C48*IF(Oversikt!$B$18="J",1,0)+'Faste kostnader'!C49*IF(Oversikt!$B$19="J",1,0)+'Faste kostnader'!C53*IF(Oversikt!$B$23="J",1,0)+'Faste kostnader'!C54*IF(Oversikt!$B$24="J",1,0)</f>
         <v/>
       </c>
       <c r="D48" s="12" t="inlineStr">
         <is>
-          <t>da</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E48" s="23" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Sau = Tal vinterfôra sau [Sau!C7] × (Fôrnorm beite (FEm) [Sau!C25] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Sau!C26] / 650) × Med i totalen Sau [Oversikt!B23 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
+          <t>Maskinkostnader i grovfôrproduksjonane = Maskinkostnader – Mjølk [Faste kostnader!C46] × Med i totalen Mjølk [Oversikt!B16 → 1/0] + Maskinkostnader – Oksar [Faste kostnader!C47] × Med i totalen Oksar [Oversikt!B17 → 1/0] + Maskinkostnader – Mellomkalv [Faste kostnader!C48] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0] + Maskinkostnader – Ammekyr [Faste kostnader!C49] × Med i totalen Ammekyr [Oversikt!B19 → 1/0] + Maskinkostnader – Sau [Faste kostnader!C53] × Med i totalen Sau [Oversikt!B23 → 1/0] + Maskinkostnader – Geit [Faste kostnader!C54] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
         </is>
       </c>
       <c r="F48" s="24" t="inlineStr">
         <is>
-          <t>=Sau!C7*(Sau!C25/625+Sau!C26/650)*IF(Oversikt!$B$23="J",1,0)</t>
+          <t>='Faste kostnader'!C46*IF(Oversikt!$B$16="J",1,0)+'Faste kostnader'!C47*IF(Oversikt!$B$17="J",1,0)+'Faste kostnader'!C48*IF(Oversikt!$B$18="J",1,0)+'Faste kostnader'!C49*IF(Oversikt!$B$19="J",1,0)+'Faste kostnader'!C53*IF(Oversikt!$B$23="J",1,0)+'Faste kostnader'!C54*IF(Oversikt!$B$24="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="20" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Geit</t>
+          <t>DB grovfôrbaserte husdyr u/tilskot</t>
         </is>
       </c>
       <c r="B49" s="21" t="inlineStr">
@@ -46175,30 +46406,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C49" s="36">
-        <f>Geit!C7*(Geit!C14/625+Geit!C15/650)*IF(Oversikt!$B$24="J",1,0)</f>
+      <c r="C49" s="22">
+        <f>'Mjølk'!C56*IF(Oversikt!$B$16="J",1,0)+Oksar!C53*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C53*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C58*IF(Oversikt!$B$19="J",1,0)+Sau!C64*IF(Oversikt!$B$23="J",1,0)+Geit!C52*IF(Oversikt!$B$24="J",1,0)</f>
         <v/>
       </c>
       <c r="D49" s="12" t="inlineStr">
         <is>
-          <t>da</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E49" s="23" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Geit = Tal årsgeiter [Geit!C7] × (Fôrnorm beite (FEm) [Geit!C14] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Geit!C15] / 650) × Med i totalen Geit [Oversikt!B24 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
+          <t>DB grovfôrbaserte husdyr u/tilskot = Dekningsbidrag (DB) utan tilskot [Mjølk!C56] × Med i totalen Mjølk [Oversikt!B16 → 1/0] + Dekningsbidrag (DB) utan tilskot [Oksar!C53] × Med i totalen Oksar [Oversikt!B17 → 1/0] + Dekningsbidrag (DB) utan tilskot [Mellomkalv!C53] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0] + Dekningsbidrag (DB) utan tilskot [Ammekyr!C58] × Med i totalen Ammekyr [Oversikt!B19 → 1/0] + Dekningsbidrag (DB) utan tilskot [Sau!C64] × Med i totalen Sau [Oversikt!B23 → 1/0] + Dekningsbidrag (DB) utan tilskot [Geit!C52] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
         </is>
       </c>
       <c r="F49" s="24" t="inlineStr">
         <is>
-          <t>=Geit!C7*(Geit!C14/625+Geit!C15/650)*IF(Oversikt!$B$24="J",1,0)</t>
+          <t>='Mjølk'!C56*IF(Oversikt!$B$16="J",1,0)+Oksar!C53*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C53*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C58*IF(Oversikt!$B$19="J",1,0)+Sau!C64*IF(Oversikt!$B$23="J",1,0)+Geit!C52*IF(Oversikt!$B$24="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="20" t="inlineStr">
         <is>
-          <t>Sum arealbehov etter fôrnorm</t>
+          <t>DB grovfôrbaserte husdyr m/tilskot</t>
         </is>
       </c>
       <c r="B50" s="21" t="inlineStr">
@@ -46206,30 +46437,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C50" s="36">
-        <f>C44+C45+C46+C47+C48+C49</f>
+      <c r="C50" s="22">
+        <f>'Mjølk'!C57*IF(Oversikt!$B$16="J",1,0)+Oksar!C54*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C54*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C59*IF(Oversikt!$B$19="J",1,0)+Sau!C65*IF(Oversikt!$B$23="J",1,0)+Geit!C53*IF(Oversikt!$B$24="J",1,0)</f>
         <v/>
       </c>
       <c r="D50" s="12" t="inlineStr">
         <is>
-          <t>da</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E50" s="23" t="inlineStr">
         <is>
-          <t>Sum arealbehov etter fôrnorm = Arealbehov etter fôrnorm – Mjølk [C44] + Arealbehov etter fôrnorm – Oksar [C45] + Arealbehov etter fôrnorm – Mellomkalv [C46] + Arealbehov etter fôrnorm – Ammekyr [C47] + Arealbehov etter fôrnorm – Sau [C48] + Arealbehov etter fôrnorm – Geit [C49]</t>
+          <t>DB grovfôrbaserte husdyr m/tilskot = Dekningsbidrag (DB) med tilskot [Mjølk!C57] × Med i totalen Mjølk [Oversikt!B16 → 1/0] + Dekningsbidrag (DB) med tilskot [Oksar!C54] × Med i totalen Oksar [Oversikt!B17 → 1/0] + Dekningsbidrag (DB) med tilskot [Mellomkalv!C54] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0] + Dekningsbidrag (DB) med tilskot [Ammekyr!C59] × Med i totalen Ammekyr [Oversikt!B19 → 1/0] + Dekningsbidrag (DB) med tilskot [Sau!C65] × Med i totalen Sau [Oversikt!B23 → 1/0] + Dekningsbidrag (DB) med tilskot [Geit!C53] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
         </is>
       </c>
       <c r="F50" s="24" t="inlineStr">
         <is>
-          <t>=C44+C45+C46+C47+C48+C49</t>
+          <t>='Mjølk'!C57*IF(Oversikt!$B$16="J",1,0)+Oksar!C54*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C54*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C59*IF(Oversikt!$B$19="J",1,0)+Sau!C65*IF(Oversikt!$B$23="J",1,0)+Geit!C53*IF(Oversikt!$B$24="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="18" t="inlineStr">
         <is>
-          <t>5. OUTPUT – Nøkkeltal grovfôr</t>
+          <t>4b. UTREKNING – Arealbehov etter fôrnorm (kontroll av grovfôrbalansen)</t>
         </is>
       </c>
       <c r="B51" s="19" t="n"/>
@@ -46239,281 +46470,510 @@
       <c r="F51" s="19" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="25" t="inlineStr">
-        <is>
-          <t>Variabel grovfôrkostnad pr korrigert dekar</t>
-        </is>
-      </c>
-      <c r="B52" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C52" s="39">
-        <f>IF((C21)=0,0,(C39)/(C21))</f>
-        <v/>
-      </c>
-      <c r="D52" s="28" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E52" s="29" t="inlineStr">
-        <is>
-          <t>Variabel grovfôrkostnad pr korrigert dekar = Sum variabel grovfôrkostnad (utan plast) [C39] ÷ Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C21]</t>
-        </is>
-      </c>
-      <c r="F52" s="30" t="inlineStr">
-        <is>
-          <t>=IF((C21)=0,0,(C39)/(C21))</t>
+      <c r="A52" s="20" t="inlineStr">
+        <is>
+          <t>Arealbehov etter fôrnorm – Mjølk</t>
+        </is>
+      </c>
+      <c r="B52" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C52" s="36">
+        <f>'Mjølk'!C7*('Mjølk'!C17/625+'Mjølk'!C18/650)*IF(Oversikt!$B$16="J",1,0)</f>
+        <v/>
+      </c>
+      <c r="D52" s="12" t="inlineStr">
+        <is>
+          <t>da</t>
+        </is>
+      </c>
+      <c r="E52" s="23" t="inlineStr">
+        <is>
+          <t>Arealbehov etter fôrnorm – Mjølk = Tal årskyr [Mjølk!C7] × (Fôrnorm beite (FEm) [Mjølk!C17] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Mjølk!C18] / 650) × Med i totalen Mjølk [Oversikt!B16 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
+        </is>
+      </c>
+      <c r="F52" s="24" t="inlineStr">
+        <is>
+          <t>='Mjølk'!C7*('Mjølk'!C17/625+'Mjølk'!C18/650)*IF(Oversikt!$B$16="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="25" t="inlineStr">
-        <is>
-          <t>Maskinkostnader pr dekar grovfôr</t>
-        </is>
-      </c>
-      <c r="B53" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C53" s="39">
-        <f>IF((C20)=0,0,(C40)/(C20))</f>
-        <v/>
-      </c>
-      <c r="D53" s="28" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E53" s="29" t="inlineStr">
-        <is>
-          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader i grovfôrproduksjonane [C40] ÷ Dekar grovfôr – maskinkostnadsgrunnlag (overflate/2 + fulldyrka + kulturbeite×10 %) [C20]</t>
-        </is>
-      </c>
-      <c r="F53" s="30" t="inlineStr">
-        <is>
-          <t>=IF((C20)=0,0,(C40)/(C20))</t>
+      <c r="A53" s="20" t="inlineStr">
+        <is>
+          <t>Arealbehov etter fôrnorm – Oksar</t>
+        </is>
+      </c>
+      <c r="B53" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C53" s="36">
+        <f>Oksar!C7*(Oksar!C16/625+Oksar!C17/650)*IF(Oversikt!$B$17="J",1,0)</f>
+        <v/>
+      </c>
+      <c r="D53" s="12" t="inlineStr">
+        <is>
+          <t>da</t>
+        </is>
+      </c>
+      <c r="E53" s="23" t="inlineStr">
+        <is>
+          <t>Arealbehov etter fôrnorm – Oksar = Tal produserte oksar [Oksar!C7] × (Fôrnorm beite (FEm) [Oksar!C16] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Oksar!C17] / 650) × Med i totalen Oksar [Oversikt!B17 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
+        </is>
+      </c>
+      <c r="F53" s="24" t="inlineStr">
+        <is>
+          <t>=Oksar!C7*(Oksar!C16/625+Oksar!C17/650)*IF(Oversikt!$B$17="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="25" t="inlineStr">
-        <is>
-          <t>Korrigerte dekar pr «kueining»</t>
-        </is>
-      </c>
-      <c r="B54" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C54" s="39">
-        <f>IF((C31)=0,0,(C21)/(C31))</f>
-        <v/>
-      </c>
-      <c r="D54" s="28" t="inlineStr">
+      <c r="A54" s="20" t="inlineStr">
+        <is>
+          <t>Arealbehov etter fôrnorm – Mellomkalv</t>
+        </is>
+      </c>
+      <c r="B54" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C54" s="36">
+        <f>Mellomkalv!C7*(Mellomkalv!C16/625+Mellomkalv!C17/650)*IF(Oversikt!$B$18="J",1,0)</f>
+        <v/>
+      </c>
+      <c r="D54" s="12" t="inlineStr">
         <is>
           <t>da</t>
         </is>
       </c>
-      <c r="E54" s="29" t="inlineStr">
-        <is>
-          <t>Korrigerte dekar pr «kueining» = Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C21] ÷ Sum «kueiningar» [C31]</t>
-        </is>
-      </c>
-      <c r="F54" s="30" t="inlineStr">
-        <is>
-          <t>=IF((C31)=0,0,(C21)/(C31))</t>
+      <c r="E54" s="23" t="inlineStr">
+        <is>
+          <t>Arealbehov etter fôrnorm – Mellomkalv = Tal produserte kalvar [Mellomkalv!C7] × (Fôrnorm beite (FEm) [Mellomkalv!C16] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Mellomkalv!C17] / 650) × Med i totalen Mellomkalv [Oversikt!B18 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
+        </is>
+      </c>
+      <c r="F54" s="24" t="inlineStr">
+        <is>
+          <t>=Mellomkalv!C7*(Mellomkalv!C16/625+Mellomkalv!C17/650)*IF(Oversikt!$B$18="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="25" t="inlineStr">
-        <is>
-          <t>Dekar fulldyrka pr «kueining»</t>
-        </is>
-      </c>
-      <c r="B55" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C55" s="39">
-        <f>IF((C31)=0,0,(C18)/(C31))</f>
-        <v/>
-      </c>
-      <c r="D55" s="28" t="inlineStr">
+      <c r="A55" s="20" t="inlineStr">
+        <is>
+          <t>Arealbehov etter fôrnorm – Ammekyr</t>
+        </is>
+      </c>
+      <c r="B55" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C55" s="36">
+        <f>Ammekyr!C7*(Ammekyr!C21/625+Ammekyr!C22/650)*IF(Oversikt!$B$19="J",1,0)</f>
+        <v/>
+      </c>
+      <c r="D55" s="12" t="inlineStr">
         <is>
           <t>da</t>
         </is>
       </c>
-      <c r="E55" s="29" t="inlineStr">
-        <is>
-          <t>Dekar fulldyrka pr «kueining» = Fulldyrka til eigen grovfôrbasert husdyrproduksjon [C18] ÷ Sum «kueiningar» [C31]</t>
-        </is>
-      </c>
-      <c r="F55" s="30" t="inlineStr">
-        <is>
-          <t>=IF((C31)=0,0,(C18)/(C31))</t>
+      <c r="E55" s="23" t="inlineStr">
+        <is>
+          <t>Arealbehov etter fôrnorm – Ammekyr = Tal ammekyr [Ammekyr!C7] × (Fôrnorm beite (FEm) [Ammekyr!C21] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Ammekyr!C22] / 650) × Med i totalen Ammekyr [Oversikt!B19 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
+        </is>
+      </c>
+      <c r="F55" s="24" t="inlineStr">
+        <is>
+          <t>=Ammekyr!C7*(Ammekyr!C21/625+Ammekyr!C22/650)*IF(Oversikt!$B$19="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="25" t="inlineStr">
-        <is>
-          <t>Dekar kulturbeite pr «kueining»</t>
-        </is>
-      </c>
-      <c r="B56" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C56" s="39">
-        <f>IF((C31)=0,0,(C19)/(C31))</f>
-        <v/>
-      </c>
-      <c r="D56" s="28" t="inlineStr">
+      <c r="A56" s="20" t="inlineStr">
+        <is>
+          <t>Arealbehov etter fôrnorm – Sau</t>
+        </is>
+      </c>
+      <c r="B56" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C56" s="36">
+        <f>Sau!C7*(Sau!C25/625+Sau!C26/650)*IF(Oversikt!$B$23="J",1,0)</f>
+        <v/>
+      </c>
+      <c r="D56" s="12" t="inlineStr">
         <is>
           <t>da</t>
         </is>
       </c>
-      <c r="E56" s="29" t="inlineStr">
-        <is>
-          <t>Dekar kulturbeite pr «kueining» = Kulturbeite til eige bruk [C19] ÷ Sum «kueiningar» [C31]</t>
-        </is>
-      </c>
-      <c r="F56" s="30" t="inlineStr">
-        <is>
-          <t>=IF((C31)=0,0,(C19)/(C31))</t>
+      <c r="E56" s="23" t="inlineStr">
+        <is>
+          <t>Arealbehov etter fôrnorm – Sau = Tal vinterfôra sau [Sau!C7] × (Fôrnorm beite (FEm) [Sau!C25] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Sau!C26] / 650) × Med i totalen Sau [Oversikt!B23 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
+        </is>
+      </c>
+      <c r="F56" s="24" t="inlineStr">
+        <is>
+          <t>=Sau!C7*(Sau!C25/625+Sau!C26/650)*IF(Oversikt!$B$23="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="25" t="inlineStr">
-        <is>
-          <t>FEm frå utmark pr «kueining»</t>
-        </is>
-      </c>
-      <c r="B57" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C57" s="27">
-        <f>IF((C31)=0,0,(C22)/(C31))</f>
-        <v/>
-      </c>
-      <c r="D57" s="28" t="inlineStr">
-        <is>
-          <t>FEm</t>
-        </is>
-      </c>
-      <c r="E57" s="29" t="inlineStr">
-        <is>
-          <t>FEm frå utmark pr «kueining» = Fôreiningar (FEm) henta frå utmark [C22] ÷ Sum «kueiningar» [C31]</t>
-        </is>
-      </c>
-      <c r="F57" s="30" t="inlineStr">
-        <is>
-          <t>=IF((C31)=0,0,(C22)/(C31))</t>
+      <c r="A57" s="20" t="inlineStr">
+        <is>
+          <t>Arealbehov etter fôrnorm – Geit</t>
+        </is>
+      </c>
+      <c r="B57" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C57" s="36">
+        <f>Geit!C7*(Geit!C14/625+Geit!C15/650)*IF(Oversikt!$B$24="J",1,0)</f>
+        <v/>
+      </c>
+      <c r="D57" s="12" t="inlineStr">
+        <is>
+          <t>da</t>
+        </is>
+      </c>
+      <c r="E57" s="23" t="inlineStr">
+        <is>
+          <t>Arealbehov etter fôrnorm – Geit = Tal årsgeiter [Geit!C7] × (Fôrnorm beite (FEm) [Geit!C14] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Geit!C15] / 650) × Med i totalen Geit [Oversikt!B24 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
+        </is>
+      </c>
+      <c r="F57" s="24" t="inlineStr">
+        <is>
+          <t>=Geit!C7*(Geit!C14/625+Geit!C15/650)*IF(Oversikt!$B$24="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="25" t="inlineStr">
-        <is>
-          <t>DB grovfôrbaserte husdyr u/tilskot pr korrigert dekar</t>
-        </is>
-      </c>
-      <c r="B58" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C58" s="39">
-        <f>IF((C21)=0,0,(C41)/(C21))</f>
-        <v/>
-      </c>
-      <c r="D58" s="28" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E58" s="29" t="inlineStr">
-        <is>
-          <t>DB grovfôrbaserte husdyr u/tilskot pr korrigert dekar = DB grovfôrbaserte husdyr u/tilskot [C41] ÷ Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C21]</t>
-        </is>
-      </c>
-      <c r="F58" s="30" t="inlineStr">
-        <is>
-          <t>=IF((C21)=0,0,(C41)/(C21))</t>
+      <c r="A58" s="20" t="inlineStr">
+        <is>
+          <t>Sum arealbehov etter fôrnorm</t>
+        </is>
+      </c>
+      <c r="B58" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C58" s="36">
+        <f>C52+C53+C54+C55+C56+C57</f>
+        <v/>
+      </c>
+      <c r="D58" s="12" t="inlineStr">
+        <is>
+          <t>da</t>
+        </is>
+      </c>
+      <c r="E58" s="23" t="inlineStr">
+        <is>
+          <t>Sum arealbehov etter fôrnorm = Arealbehov etter fôrnorm – Mjølk [C52] + Arealbehov etter fôrnorm – Oksar [C53] + Arealbehov etter fôrnorm – Mellomkalv [C54] + Arealbehov etter fôrnorm – Ammekyr [C55] + Arealbehov etter fôrnorm – Sau [C56] + Arealbehov etter fôrnorm – Geit [C57]</t>
+        </is>
+      </c>
+      <c r="F58" s="24" t="inlineStr">
+        <is>
+          <t>=C52+C53+C54+C55+C56+C57</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="25" t="inlineStr">
-        <is>
-          <t>DB grovfôrbaserte husdyr m/tilskot pr korrigert dekar</t>
-        </is>
-      </c>
-      <c r="B59" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C59" s="39">
-        <f>IF((C21)=0,0,(C42)/(C21))</f>
-        <v/>
-      </c>
-      <c r="D59" s="28" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E59" s="29" t="inlineStr">
-        <is>
-          <t>DB grovfôrbaserte husdyr m/tilskot pr korrigert dekar = DB grovfôrbaserte husdyr m/tilskot [C42] ÷ Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C21]</t>
-        </is>
-      </c>
-      <c r="F59" s="30" t="inlineStr">
-        <is>
-          <t>=IF((C21)=0,0,(C42)/(C21))</t>
-        </is>
-      </c>
+      <c r="A59" s="18" t="inlineStr">
+        <is>
+          <t>5. OUTPUT – Nøkkeltal grovfôr</t>
+        </is>
+      </c>
+      <c r="B59" s="19" t="n"/>
+      <c r="C59" s="19" t="n"/>
+      <c r="D59" s="19" t="n"/>
+      <c r="E59" s="19" t="n"/>
+      <c r="F59" s="19" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="25" t="inlineStr">
         <is>
+          <t>Variabel grovfôrkostnad pr korrigert dekar</t>
+        </is>
+      </c>
+      <c r="B60" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C60" s="39">
+        <f>IF((C22)=0,0,(C47)/(C22))</f>
+        <v/>
+      </c>
+      <c r="D60" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E60" s="29" t="inlineStr">
+        <is>
+          <t>Variabel grovfôrkostnad pr korrigert dekar = Sum variabel grovfôrkostnad (utan plast) [C47] ÷ Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C22]</t>
+        </is>
+      </c>
+      <c r="F60" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C22)=0,0,(C47)/(C22))</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="25" t="inlineStr">
+        <is>
+          <t>Maskinkostnader pr dekar grovfôr</t>
+        </is>
+      </c>
+      <c r="B61" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C61" s="39">
+        <f>IF((C25)=0,0,(C48)/(C25))</f>
+        <v/>
+      </c>
+      <c r="D61" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E61" s="29" t="inlineStr">
+        <is>
+          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader i grovfôrproduksjonane [C48] ÷ Dekar grovfôr – maskinkostnadsgrunnlag (overflate/2 + fulldyrka + kulturbeite×10 %) [C25]</t>
+        </is>
+      </c>
+      <c r="F61" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C25)=0,0,(C48)/(C25))</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="25" t="inlineStr">
+        <is>
+          <t>Korrigerte dekar pr «kueining»</t>
+        </is>
+      </c>
+      <c r="B62" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C62" s="39">
+        <f>IF((C39)=0,0,(C22)/(C39))</f>
+        <v/>
+      </c>
+      <c r="D62" s="28" t="inlineStr">
+        <is>
+          <t>da</t>
+        </is>
+      </c>
+      <c r="E62" s="29" t="inlineStr">
+        <is>
+          <t>Korrigerte dekar pr «kueining» = Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C22] ÷ Sum «kueiningar» [C39]</t>
+        </is>
+      </c>
+      <c r="F62" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C39)=0,0,(C22)/(C39))</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="25" t="inlineStr">
+        <is>
+          <t>Dekar fulldyrka pr «kueining»</t>
+        </is>
+      </c>
+      <c r="B63" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C63" s="39">
+        <f>IF((C39)=0,0,(C18)/(C39))</f>
+        <v/>
+      </c>
+      <c r="D63" s="28" t="inlineStr">
+        <is>
+          <t>da</t>
+        </is>
+      </c>
+      <c r="E63" s="29" t="inlineStr">
+        <is>
+          <t>Dekar fulldyrka pr «kueining» = Fulldyrka til eigen grovfôrbasert husdyrproduksjon [C18] ÷ Sum «kueiningar» [C39]</t>
+        </is>
+      </c>
+      <c r="F63" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C39)=0,0,(C18)/(C39))</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="25" t="inlineStr">
+        <is>
+          <t>Dekar kulturbeite pr «kueining»</t>
+        </is>
+      </c>
+      <c r="B64" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C64" s="39">
+        <f>IF((C39)=0,0,(C19)/(C39))</f>
+        <v/>
+      </c>
+      <c r="D64" s="28" t="inlineStr">
+        <is>
+          <t>da</t>
+        </is>
+      </c>
+      <c r="E64" s="29" t="inlineStr">
+        <is>
+          <t>Dekar kulturbeite pr «kueining» = Kulturbeite til eige bruk [C19] ÷ Sum «kueiningar» [C39]</t>
+        </is>
+      </c>
+      <c r="F64" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C39)=0,0,(C19)/(C39))</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="25" t="inlineStr">
+        <is>
+          <t>FEm frå utmark pr «kueining»</t>
+        </is>
+      </c>
+      <c r="B65" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C65" s="27">
+        <f>IF((C39)=0,0,(C28)/(C39))</f>
+        <v/>
+      </c>
+      <c r="D65" s="28" t="inlineStr">
+        <is>
+          <t>FEm</t>
+        </is>
+      </c>
+      <c r="E65" s="29" t="inlineStr">
+        <is>
+          <t>FEm frå utmark pr «kueining» = Fôreiningar (FEm) henta frå utmark [C28] ÷ Sum «kueiningar» [C39]</t>
+        </is>
+      </c>
+      <c r="F65" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C39)=0,0,(C28)/(C39))</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="25" t="inlineStr">
+        <is>
+          <t>DB grovfôrbaserte husdyr u/tilskot pr korrigert dekar</t>
+        </is>
+      </c>
+      <c r="B66" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C66" s="39">
+        <f>IF((C22)=0,0,(C49)/(C22))</f>
+        <v/>
+      </c>
+      <c r="D66" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E66" s="29" t="inlineStr">
+        <is>
+          <t>DB grovfôrbaserte husdyr u/tilskot pr korrigert dekar = DB grovfôrbaserte husdyr u/tilskot [C49] ÷ Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C22]</t>
+        </is>
+      </c>
+      <c r="F66" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C22)=0,0,(C49)/(C22))</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="25" t="inlineStr">
+        <is>
+          <t>DB grovfôrbaserte husdyr m/tilskot pr korrigert dekar</t>
+        </is>
+      </c>
+      <c r="B67" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C67" s="39">
+        <f>IF((C22)=0,0,(C50)/(C22))</f>
+        <v/>
+      </c>
+      <c r="D67" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E67" s="29" t="inlineStr">
+        <is>
+          <t>DB grovfôrbaserte husdyr m/tilskot pr korrigert dekar = DB grovfôrbaserte husdyr m/tilskot [C50] ÷ Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C22]</t>
+        </is>
+      </c>
+      <c r="F67" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C22)=0,0,(C50)/(C22))</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="25" t="inlineStr">
+        <is>
           <t>Korrigert grovfôrareal i % av arealbehov etter fôrnorm</t>
         </is>
       </c>
-      <c r="B60" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C60" s="33">
-        <f>IF((C50)=0,0,(C21)/(C50))</f>
-        <v/>
-      </c>
-      <c r="D60" s="28" t="inlineStr">
+      <c r="B68" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C68" s="33">
+        <f>IF((C58)=0,0,(C22)/(C58))</f>
+        <v/>
+      </c>
+      <c r="D68" s="28" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E60" s="29" t="inlineStr">
-        <is>
-          <t>Korrigert grovfôrareal i % av arealbehov etter fôrnorm = Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C21] ÷ Sum arealbehov etter fôrnorm [C50]   (Under 100 % tyder på kjøpt fôr eller høge avlingar, over 100 % på overskot av areal)</t>
-        </is>
-      </c>
-      <c r="F60" s="30" t="inlineStr">
-        <is>
-          <t>=IF((C50)=0,0,(C21)/(C50))</t>
+      <c r="E68" s="29" t="inlineStr">
+        <is>
+          <t>Korrigert grovfôrareal i % av arealbehov etter fôrnorm = Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C22] ÷ Sum arealbehov etter fôrnorm [C58]   (Under 100 % tyder på kjøpt fôr eller høge avlingar, over 100 % på overskot av areal)</t>
+        </is>
+      </c>
+      <c r="F68" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C58)=0,0,(C22)/(C58))</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Nøkkeltall fra Agro-malen: solgt avling per dekar, sum planteareal, korrigerte dekar per kueining for storfe
Kg slakt i melkeproduksjonen hentes nå for alle storfe-suffikser (511–515),
slik at kjøttprisen har samme omfang i teller og nevner.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HrtCx2hBap2TXaC318T6kC
</commit_message>
<xml_diff>
--- a/excel/Analyse_jordbruk_produksjonar.xlsx
+++ b/excel/Analyse_jordbruk_produksjonar.xlsx
@@ -1081,7 +1081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -2412,7 +2412,7 @@
     <row r="55">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr m²</t>
+          <t>Seld avling pr m² (kg)</t>
         </is>
       </c>
       <c r="B55" s="26" t="inlineStr">
@@ -2420,52 +2420,83 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C55" s="39">
-        <f>IF((C7)=0,0,(C23)/(C7))</f>
+      <c r="C55" s="37">
+        <f>IF((C7)=0,0,(C9)/(C7))</f>
         <v/>
       </c>
       <c r="D55" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E55" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr m² = Maskinkostnader fordelt [C23] ÷ Tal m² [C7]</t>
+          <t>Seld avling pr m² (kg) = Seld mengd [C9] ÷ Tal m² [C7]</t>
         </is>
       </c>
       <c r="F55" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C23)/(C7))</t>
+          <t>=IF((C7)=0,0,(C9)/(C7))</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="25" t="inlineStr">
         <is>
+          <t>Maskinkostnader pr m²</t>
+        </is>
+      </c>
+      <c r="B56" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C56" s="39">
+        <f>IF((C7)=0,0,(C23)/(C7))</f>
+        <v/>
+      </c>
+      <c r="D56" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E56" s="29" t="inlineStr">
+        <is>
+          <t>Maskinkostnader pr m² = Maskinkostnader fordelt [C23] ÷ Tal m² [C7]</t>
+        </is>
+      </c>
+      <c r="F56" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C7)=0,0,(C23)/(C7))</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="25" t="inlineStr">
+        <is>
           <t>DB etter maskinkostnader pr m²</t>
         </is>
       </c>
-      <c r="B56" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C56" s="39">
+      <c r="B57" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C57" s="39">
         <f>IF((C7)=0,0,(C29)/(C7))</f>
         <v/>
       </c>
-      <c r="D56" s="28" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E56" s="29" t="inlineStr">
+      <c r="D57" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E57" s="29" t="inlineStr">
         <is>
           <t>DB etter maskinkostnader pr m² = DB m/tilskot etter maskinkostnader [C29] ÷ Tal m² [C7]</t>
         </is>
       </c>
-      <c r="F56" s="30" t="inlineStr">
+      <c r="F57" s="30" t="inlineStr">
         <is>
           <t>=IF((C7)=0,0,(C29)/(C7))</t>
         </is>
@@ -2483,7 +2514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -3814,7 +3845,7 @@
     <row r="55">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr m²</t>
+          <t>Seld avling pr m² (kg)</t>
         </is>
       </c>
       <c r="B55" s="26" t="inlineStr">
@@ -3822,52 +3853,83 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C55" s="39">
-        <f>IF((C7)=0,0,(C23)/(C7))</f>
+      <c r="C55" s="37">
+        <f>IF((C7)=0,0,(C9)/(C7))</f>
         <v/>
       </c>
       <c r="D55" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E55" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr m² = Maskinkostnader fordelt [C23] ÷ Tal m² [C7]</t>
+          <t>Seld avling pr m² (kg) = Seld mengd [C9] ÷ Tal m² [C7]</t>
         </is>
       </c>
       <c r="F55" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C23)/(C7))</t>
+          <t>=IF((C7)=0,0,(C9)/(C7))</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="25" t="inlineStr">
         <is>
+          <t>Maskinkostnader pr m²</t>
+        </is>
+      </c>
+      <c r="B56" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C56" s="39">
+        <f>IF((C7)=0,0,(C23)/(C7))</f>
+        <v/>
+      </c>
+      <c r="D56" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E56" s="29" t="inlineStr">
+        <is>
+          <t>Maskinkostnader pr m² = Maskinkostnader fordelt [C23] ÷ Tal m² [C7]</t>
+        </is>
+      </c>
+      <c r="F56" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C7)=0,0,(C23)/(C7))</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="25" t="inlineStr">
+        <is>
           <t>DB etter maskinkostnader pr m²</t>
         </is>
       </c>
-      <c r="B56" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C56" s="39">
+      <c r="B57" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C57" s="39">
         <f>IF((C7)=0,0,(C29)/(C7))</f>
         <v/>
       </c>
-      <c r="D56" s="28" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E56" s="29" t="inlineStr">
+      <c r="D57" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E57" s="29" t="inlineStr">
         <is>
           <t>DB etter maskinkostnader pr m² = DB m/tilskot etter maskinkostnader [C29] ÷ Tal m² [C7]</t>
         </is>
       </c>
-      <c r="F56" s="30" t="inlineStr">
+      <c r="F57" s="30" t="inlineStr">
         <is>
           <t>=IF((C7)=0,0,(C29)/(C7))</t>
         </is>
@@ -3885,7 +3947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -5159,7 +5221,7 @@
     <row r="53">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar</t>
+          <t>Seld avling pr dekar (kg)</t>
         </is>
       </c>
       <c r="B53" s="26" t="inlineStr">
@@ -5167,52 +5229,83 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C53" s="39">
-        <f>IF((C7)=0,0,(C22)/(C7))</f>
+      <c r="C53" s="37">
+        <f>IF((C7)=0,0,(C9)/(C7))</f>
         <v/>
       </c>
       <c r="D53" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E53" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar = Maskinkostnader fordelt [C22] ÷ Tal dekar [C7]</t>
+          <t>Seld avling pr dekar (kg) = Seld mengd [C9] ÷ Tal dekar [C7]</t>
         </is>
       </c>
       <c r="F53" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C22)/(C7))</t>
+          <t>=IF((C7)=0,0,(C9)/(C7))</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="25" t="inlineStr">
         <is>
+          <t>Maskinkostnader pr dekar</t>
+        </is>
+      </c>
+      <c r="B54" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C54" s="39">
+        <f>IF((C7)=0,0,(C22)/(C7))</f>
+        <v/>
+      </c>
+      <c r="D54" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E54" s="29" t="inlineStr">
+        <is>
+          <t>Maskinkostnader pr dekar = Maskinkostnader fordelt [C22] ÷ Tal dekar [C7]</t>
+        </is>
+      </c>
+      <c r="F54" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C7)=0,0,(C22)/(C7))</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="25" t="inlineStr">
+        <is>
           <t>DB etter maskinkostnader pr dekar</t>
         </is>
       </c>
-      <c r="B54" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C54" s="39">
+      <c r="B55" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C55" s="39">
         <f>IF((C7)=0,0,(C28)/(C7))</f>
         <v/>
       </c>
-      <c r="D54" s="28" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E54" s="29" t="inlineStr">
+      <c r="D55" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E55" s="29" t="inlineStr">
         <is>
           <t>DB etter maskinkostnader pr dekar = DB m/tilskot etter maskinkostnader [C28] ÷ Tal dekar [C7]</t>
         </is>
       </c>
-      <c r="F54" s="30" t="inlineStr">
+      <c r="F55" s="30" t="inlineStr">
         <is>
           <t>=IF((C7)=0,0,(C28)/(C7))</t>
         </is>
@@ -5230,7 +5323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -6504,7 +6597,7 @@
     <row r="53">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar</t>
+          <t>Seld avling pr dekar (kg)</t>
         </is>
       </c>
       <c r="B53" s="26" t="inlineStr">
@@ -6512,52 +6605,83 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C53" s="39">
-        <f>IF((C7)=0,0,(C22)/(C7))</f>
+      <c r="C53" s="37">
+        <f>IF((C7)=0,0,(C9)/(C7))</f>
         <v/>
       </c>
       <c r="D53" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E53" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar = Maskinkostnader fordelt [C22] ÷ Tal dekar [C7]</t>
+          <t>Seld avling pr dekar (kg) = Seld mengd [C9] ÷ Tal dekar [C7]</t>
         </is>
       </c>
       <c r="F53" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C22)/(C7))</t>
+          <t>=IF((C7)=0,0,(C9)/(C7))</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="25" t="inlineStr">
         <is>
+          <t>Maskinkostnader pr dekar</t>
+        </is>
+      </c>
+      <c r="B54" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C54" s="39">
+        <f>IF((C7)=0,0,(C22)/(C7))</f>
+        <v/>
+      </c>
+      <c r="D54" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E54" s="29" t="inlineStr">
+        <is>
+          <t>Maskinkostnader pr dekar = Maskinkostnader fordelt [C22] ÷ Tal dekar [C7]</t>
+        </is>
+      </c>
+      <c r="F54" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C7)=0,0,(C22)/(C7))</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="25" t="inlineStr">
+        <is>
           <t>DB etter maskinkostnader pr dekar</t>
         </is>
       </c>
-      <c r="B54" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C54" s="39">
+      <c r="B55" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C55" s="39">
         <f>IF((C7)=0,0,(C28)/(C7))</f>
         <v/>
       </c>
-      <c r="D54" s="28" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E54" s="29" t="inlineStr">
+      <c r="D55" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E55" s="29" t="inlineStr">
         <is>
           <t>DB etter maskinkostnader pr dekar = DB m/tilskot etter maskinkostnader [C28] ÷ Tal dekar [C7]</t>
         </is>
       </c>
-      <c r="F54" s="30" t="inlineStr">
+      <c r="F55" s="30" t="inlineStr">
         <is>
           <t>=IF((C7)=0,0,(C28)/(C7))</t>
         </is>
@@ -6575,7 +6699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -7849,7 +7973,7 @@
     <row r="53">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar</t>
+          <t>Seld avling pr dekar (kg)</t>
         </is>
       </c>
       <c r="B53" s="26" t="inlineStr">
@@ -7857,52 +7981,83 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C53" s="39">
-        <f>IF((C7)=0,0,(C22)/(C7))</f>
+      <c r="C53" s="37">
+        <f>IF((C7)=0,0,(C9)/(C7))</f>
         <v/>
       </c>
       <c r="D53" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E53" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar = Maskinkostnader fordelt [C22] ÷ Tal dekar [C7]</t>
+          <t>Seld avling pr dekar (kg) = Seld mengd [C9] ÷ Tal dekar [C7]</t>
         </is>
       </c>
       <c r="F53" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C22)/(C7))</t>
+          <t>=IF((C7)=0,0,(C9)/(C7))</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="25" t="inlineStr">
         <is>
+          <t>Maskinkostnader pr dekar</t>
+        </is>
+      </c>
+      <c r="B54" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C54" s="39">
+        <f>IF((C7)=0,0,(C22)/(C7))</f>
+        <v/>
+      </c>
+      <c r="D54" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E54" s="29" t="inlineStr">
+        <is>
+          <t>Maskinkostnader pr dekar = Maskinkostnader fordelt [C22] ÷ Tal dekar [C7]</t>
+        </is>
+      </c>
+      <c r="F54" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C7)=0,0,(C22)/(C7))</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="25" t="inlineStr">
+        <is>
           <t>DB etter maskinkostnader pr dekar</t>
         </is>
       </c>
-      <c r="B54" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C54" s="39">
+      <c r="B55" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C55" s="39">
         <f>IF((C7)=0,0,(C28)/(C7))</f>
         <v/>
       </c>
-      <c r="D54" s="28" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E54" s="29" t="inlineStr">
+      <c r="D55" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E55" s="29" t="inlineStr">
         <is>
           <t>DB etter maskinkostnader pr dekar = DB m/tilskot etter maskinkostnader [C28] ÷ Tal dekar [C7]</t>
         </is>
       </c>
-      <c r="F54" s="30" t="inlineStr">
+      <c r="F55" s="30" t="inlineStr">
         <is>
           <t>=IF((C7)=0,0,(C28)/(C7))</t>
         </is>
@@ -7920,7 +8075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F104"/>
+  <dimension ref="A1:F105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -10211,7 +10366,7 @@
         </is>
       </c>
       <c r="C90" s="39">
-        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C53)/('Grovfôr'!C46)))=0,0,(C56)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C53)/('Grovfôr'!C46))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C53)/('Grovfôr'!C49)))=0,0,(C56)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C53)/('Grovfôr'!C49))))</f>
         <v/>
       </c>
       <c r="D90" s="28" t="inlineStr">
@@ -10221,12 +10376,12 @@
       </c>
       <c r="E90" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C56] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C53] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
+          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C56] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C53] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C49])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
         </is>
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C53)/('Grovfôr'!C46)))=0,0,(C56)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C53)/('Grovfôr'!C46))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C53)/('Grovfôr'!C49)))=0,0,(C56)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C53)/('Grovfôr'!C49))))</t>
         </is>
       </c>
     </row>
@@ -10242,7 +10397,7 @@
         </is>
       </c>
       <c r="C91" s="39">
-        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C53)/('Grovfôr'!C46)))=0,0,(C57)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C53)/('Grovfôr'!C46))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C53)/('Grovfôr'!C49)))=0,0,(C57)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C53)/('Grovfôr'!C49))))</f>
         <v/>
       </c>
       <c r="D91" s="28" t="inlineStr">
@@ -10252,12 +10407,12 @@
       </c>
       <c r="E91" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C57] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C53] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])</t>
+          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C57] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C53] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C49])</t>
         </is>
       </c>
       <c r="F91" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C53)/('Grovfôr'!C46)))=0,0,(C57)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C53)/('Grovfôr'!C46))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C53)/('Grovfôr'!C49)))=0,0,(C57)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C53)/('Grovfôr'!C49))))</t>
         </is>
       </c>
     </row>
@@ -10273,7 +10428,7 @@
         </is>
       </c>
       <c r="C92" s="40">
-        <f>'Grovfôr'!C60</f>
+        <f>'Grovfôr'!C63</f>
         <v/>
       </c>
       <c r="D92" s="28" t="inlineStr">
@@ -10283,12 +10438,12 @@
       </c>
       <c r="E92" s="29" t="inlineStr">
         <is>
-          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C60]</t>
+          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C63]</t>
         </is>
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C60</t>
+          <t>='Grovfôr'!C63</t>
         </is>
       </c>
     </row>
@@ -10304,7 +10459,7 @@
         </is>
       </c>
       <c r="C93" s="40">
-        <f>'Grovfôr'!C61</f>
+        <f>'Grovfôr'!C64</f>
         <v/>
       </c>
       <c r="D93" s="28" t="inlineStr">
@@ -10314,12 +10469,12 @@
       </c>
       <c r="E93" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C61]</t>
+          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C64]</t>
         </is>
       </c>
       <c r="F93" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C61</t>
+          <t>='Grovfôr'!C64</t>
         </is>
       </c>
     </row>
@@ -10335,7 +10490,7 @@
         </is>
       </c>
       <c r="C94" s="40">
-        <f>'Grovfôr'!C62</f>
+        <f>'Grovfôr'!C65</f>
         <v/>
       </c>
       <c r="D94" s="28" t="inlineStr">
@@ -10345,12 +10500,12 @@
       </c>
       <c r="E94" s="29" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining» (heile garden) = Korrigerte dekar pr «kueining» [Grovfôr!C62]</t>
+          <t>Korrigerte dekar pr «kueining» (heile garden) = Korrigerte dekar pr «kueining» [Grovfôr!C65]</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C62</t>
+          <t>='Grovfôr'!C65</t>
         </is>
       </c>
     </row>
@@ -10366,7 +10521,7 @@
         </is>
       </c>
       <c r="C95" s="39">
-        <f>IF((C59)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C53)/('Grovfôr'!C46)))/(C59))</f>
+        <f>IF((C59)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C53)/('Grovfôr'!C49)))/(C59))</f>
         <v/>
       </c>
       <c r="D95" s="28" t="inlineStr">
@@ -10376,50 +10531,50 @@
       </c>
       <c r="E95" s="29" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining» i produksjonen = (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C53] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46]) ÷ «Kueiningar» [C59]   (Grovfôrarealet produksjonen får (etter eigen grovfôrkostnad) delt på kueiningane i produksjonen)</t>
+          <t>Korrigerte dekar pr «kueining» i produksjonen = (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C53] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C49]) ÷ «Kueiningar» [C59]   (Grovfôrarealet produksjonen får (etter eigen grovfôrkostnad) delt på kueiningane i produksjonen)</t>
         </is>
       </c>
       <c r="F95" s="30" t="inlineStr">
         <is>
-          <t>=IF((C59)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C53)/('Grovfôr'!C46)))/(C59))</t>
+          <t>=IF((C59)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C53)/('Grovfôr'!C49)))/(C59))</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="25" t="inlineStr">
         <is>
-          <t>Oppnådd mjølkepris pr liter (u/distriktstilskot)</t>
+          <t>Korrigerte dekar pr «kueining» – storfe samla</t>
         </is>
       </c>
       <c r="B96" s="26" t="inlineStr">
         <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C96" s="39">
-        <f>IF((C8)=0,0,(C22-C27)/(C8))</f>
+          <t>Lenkje frå anna ark</t>
+        </is>
+      </c>
+      <c r="C96" s="40">
+        <f>'Grovfôr'!C42</f>
         <v/>
       </c>
       <c r="D96" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>da</t>
         </is>
       </c>
       <c r="E96" s="29" t="inlineStr">
         <is>
-          <t>Oppnådd mjølkepris pr liter (u/distriktstilskot) = (Mjølk [C22] − Herav distriktstilskot mjølk [C27]) ÷ Levert mjølk [C8]</t>
+          <t>Korrigerte dekar pr «kueining» – storfe samla = Korrigerte dekar pr «kueining» – storfe [Grovfôr!C42]   (Som i Agro: grovfôrarealet til alle storfeproduksjonane delt på storfe-kueiningane)</t>
         </is>
       </c>
       <c r="F96" s="30" t="inlineStr">
         <is>
-          <t>=IF((C8)=0,0,(C22-C27)/(C8))</t>
+          <t>='Grovfôr'!C42</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="25" t="inlineStr">
         <is>
-          <t>Oppnådd slaktepris pr kg (u/distriktstilskot)</t>
+          <t>Oppnådd mjølkepris pr liter (u/distriktstilskot)</t>
         </is>
       </c>
       <c r="B97" s="26" t="inlineStr">
@@ -10428,7 +10583,7 @@
         </is>
       </c>
       <c r="C97" s="39">
-        <f>IF((C10)=0,0,(C23-C28)/(C10))</f>
+        <f>IF((C8)=0,0,(C22-C27)/(C8))</f>
         <v/>
       </c>
       <c r="D97" s="28" t="inlineStr">
@@ -10438,19 +10593,19 @@
       </c>
       <c r="E97" s="29" t="inlineStr">
         <is>
-          <t>Oppnådd slaktepris pr kg (u/distriktstilskot) = (Slakt [C23] − Herav distriktstilskot kjøt [C28]) ÷ Kg slakt storfe (mjølkeproduksjonen) [C10]</t>
+          <t>Oppnådd mjølkepris pr liter (u/distriktstilskot) = (Mjølk [C22] − Herav distriktstilskot mjølk [C27]) ÷ Levert mjølk [C8]</t>
         </is>
       </c>
       <c r="F97" s="30" t="inlineStr">
         <is>
-          <t>=IF((C10)=0,0,(C23-C28)/(C10))</t>
+          <t>=IF((C8)=0,0,(C22-C27)/(C8))</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="25" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr liter</t>
+          <t>Oppnådd slaktepris pr kg (u/distriktstilskot)</t>
         </is>
       </c>
       <c r="B98" s="26" t="inlineStr">
@@ -10459,7 +10614,7 @@
         </is>
       </c>
       <c r="C98" s="39">
-        <f>IF((C8)=0,0,(C47)/(C8))</f>
+        <f>IF((C10)=0,0,(C23-C28)/(C10))</f>
         <v/>
       </c>
       <c r="D98" s="28" t="inlineStr">
@@ -10469,19 +10624,19 @@
       </c>
       <c r="E98" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr liter = Maskinkostnader fordelt [C47] ÷ Levert mjølk [C8]</t>
+          <t>Oppnådd slaktepris pr kg (u/distriktstilskot) = (Slakt [C23] − Herav distriktstilskot kjøt [C28]) ÷ Kg slakt storfe (mjølkeproduksjonen) [C10]</t>
         </is>
       </c>
       <c r="F98" s="30" t="inlineStr">
         <is>
-          <t>=IF((C8)=0,0,(C47)/(C8))</t>
+          <t>=IF((C10)=0,0,(C23-C28)/(C10))</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="25" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr liter</t>
+          <t>Maskinkostnader pr liter</t>
         </is>
       </c>
       <c r="B99" s="26" t="inlineStr">
@@ -10490,7 +10645,7 @@
         </is>
       </c>
       <c r="C99" s="39">
-        <f>IF((C8)=0,0,(C48)/(C8))</f>
+        <f>IF((C8)=0,0,(C47)/(C8))</f>
         <v/>
       </c>
       <c r="D99" s="28" t="inlineStr">
@@ -10500,19 +10655,19 @@
       </c>
       <c r="E99" s="29" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr liter = Innandørsmekanisering fordelt [C48] ÷ Levert mjølk [C8]</t>
+          <t>Maskinkostnader pr liter = Maskinkostnader fordelt [C47] ÷ Levert mjølk [C8]</t>
         </is>
       </c>
       <c r="F99" s="30" t="inlineStr">
         <is>
-          <t>=IF((C8)=0,0,(C48)/(C8))</t>
+          <t>=IF((C8)=0,0,(C47)/(C8))</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="25" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr årsku</t>
+          <t>Innandørsmekanisering pr liter</t>
         </is>
       </c>
       <c r="B100" s="26" t="inlineStr">
@@ -10521,7 +10676,7 @@
         </is>
       </c>
       <c r="C100" s="39">
-        <f>IF((C7)=0,0,(C48)/(C7))</f>
+        <f>IF((C8)=0,0,(C48)/(C8))</f>
         <v/>
       </c>
       <c r="D100" s="28" t="inlineStr">
@@ -10531,19 +10686,19 @@
       </c>
       <c r="E100" s="29" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr årsku = Innandørsmekanisering fordelt [C48] ÷ Tal årskyr [C7]</t>
+          <t>Innandørsmekanisering pr liter = Innandørsmekanisering fordelt [C48] ÷ Levert mjølk [C8]</t>
         </is>
       </c>
       <c r="F100" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C48)/(C7))</t>
+          <t>=IF((C8)=0,0,(C48)/(C8))</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="25" t="inlineStr">
         <is>
-          <t>Levert mjølk pr årsku (liter)</t>
+          <t>Innandørsmekanisering pr årsku</t>
         </is>
       </c>
       <c r="B101" s="26" t="inlineStr">
@@ -10551,30 +10706,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C101" s="27">
-        <f>IF((C7)=0,0,(C8)/(C7))</f>
+      <c r="C101" s="39">
+        <f>IF((C7)=0,0,(C48)/(C7))</f>
         <v/>
       </c>
       <c r="D101" s="28" t="inlineStr">
         <is>
-          <t>liter</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E101" s="29" t="inlineStr">
         <is>
-          <t>Levert mjølk pr årsku (liter) = Levert mjølk [C8] ÷ Tal årskyr [C7]</t>
+          <t>Innandørsmekanisering pr årsku = Innandørsmekanisering fordelt [C48] ÷ Tal årskyr [C7]</t>
         </is>
       </c>
       <c r="F101" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C8)/(C7))</t>
+          <t>=IF((C7)=0,0,(C48)/(C7))</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="25" t="inlineStr">
         <is>
-          <t>Påsettprosent</t>
+          <t>Levert mjølk pr årsku (liter)</t>
         </is>
       </c>
       <c r="B102" s="26" t="inlineStr">
@@ -10582,30 +10737,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C102" s="33">
-        <f>C60</f>
+      <c r="C102" s="27">
+        <f>IF((C7)=0,0,(C8)/(C7))</f>
         <v/>
       </c>
       <c r="D102" s="28" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>liter</t>
         </is>
       </c>
       <c r="E102" s="29" t="inlineStr">
         <is>
-          <t>Påsettprosent = Påsettprosent [C60]</t>
+          <t>Levert mjølk pr årsku (liter) = Levert mjølk [C8] ÷ Tal årskyr [C7]</t>
         </is>
       </c>
       <c r="F102" s="30" t="inlineStr">
         <is>
-          <t>=C60</t>
+          <t>=IF((C7)=0,0,(C8)/(C7))</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="25" t="inlineStr">
         <is>
-          <t>Kvoteoppfylling</t>
+          <t>Påsettprosent</t>
         </is>
       </c>
       <c r="B103" s="26" t="inlineStr">
@@ -10614,7 +10769,7 @@
         </is>
       </c>
       <c r="C103" s="33">
-        <f>IF((C9)=0,0,(C8)/(C9))</f>
+        <f>C60</f>
         <v/>
       </c>
       <c r="D103" s="28" t="inlineStr">
@@ -10624,41 +10779,72 @@
       </c>
       <c r="E103" s="29" t="inlineStr">
         <is>
-          <t>Kvoteoppfylling = Levert mjølk [C8] ÷ Disponibel mjølkekvote [C9]</t>
+          <t>Påsettprosent = Påsettprosent [C60]</t>
         </is>
       </c>
       <c r="F103" s="30" t="inlineStr">
         <is>
-          <t>=IF((C9)=0,0,(C8)/(C9))</t>
+          <t>=C60</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="25" t="inlineStr">
         <is>
+          <t>Kvoteoppfylling</t>
+        </is>
+      </c>
+      <c r="B104" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C104" s="33">
+        <f>IF((C9)=0,0,(C8)/(C9))</f>
+        <v/>
+      </c>
+      <c r="D104" s="28" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E104" s="29" t="inlineStr">
+        <is>
+          <t>Kvoteoppfylling = Levert mjølk [C8] ÷ Disponibel mjølkekvote [C9]</t>
+        </is>
+      </c>
+      <c r="F104" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C9)=0,0,(C8)/(C9))</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="25" t="inlineStr">
+        <is>
           <t>Analysegruppe (påsett)</t>
         </is>
       </c>
-      <c r="B104" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C104" s="41">
+      <c r="B105" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C105" s="41">
         <f>IF(C60&lt;=0.8,"Påsett &lt; 80 %",IF(C60&lt;1.2,"Påsett 80–120 %","Påsett &gt; 120 %"))</f>
         <v/>
       </c>
-      <c r="D104" s="28" t="inlineStr">
+      <c r="D105" s="28" t="inlineStr">
         <is>
           <t>tekst</t>
         </is>
       </c>
-      <c r="E104" s="29" t="inlineStr">
+      <c r="E105" s="29" t="inlineStr">
         <is>
           <t>Analysegruppe (påsett) = HVIS(Påsettprosent [C60]&lt;=0,8; "Påsett &lt; 80 %"; HVIS(Påsettprosent [C60]&lt;1,2; "Påsett 80–120 %"; "Påsett &gt; 120 %"))   (Tilsvarar arka «Mjølk &lt;80%», «Mjølk 80-120%» og «Mjølk &gt;120%» i eksempelanalysen)</t>
         </is>
       </c>
-      <c r="F104" s="30" t="inlineStr">
+      <c r="F105" s="30" t="inlineStr">
         <is>
           <t>=IF(C60&lt;=0.8,"Påsett &lt; 80 %",IF(C60&lt;1.2,"Påsett 80–120 %","Påsett &gt; 120 %"))</t>
         </is>
@@ -10676,7 +10862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F96"/>
+  <dimension ref="A1:F97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -12796,7 +12982,7 @@
         </is>
       </c>
       <c r="C84" s="39">
-        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))=0,0,(C53)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C50)/('Grovfôr'!C49)))=0,0,(C53)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C50)/('Grovfôr'!C49))))</f>
         <v/>
       </c>
       <c r="D84" s="28" t="inlineStr">
@@ -12806,12 +12992,12 @@
       </c>
       <c r="E84" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C53] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
+          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C53] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C49])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
         </is>
       </c>
       <c r="F84" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))=0,0,(C53)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C50)/('Grovfôr'!C49)))=0,0,(C53)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C50)/('Grovfôr'!C49))))</t>
         </is>
       </c>
     </row>
@@ -12827,7 +13013,7 @@
         </is>
       </c>
       <c r="C85" s="39">
-        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))=0,0,(C54)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C50)/('Grovfôr'!C49)))=0,0,(C54)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C50)/('Grovfôr'!C49))))</f>
         <v/>
       </c>
       <c r="D85" s="28" t="inlineStr">
@@ -12837,12 +13023,12 @@
       </c>
       <c r="E85" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C54] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])</t>
+          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C54] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C49])</t>
         </is>
       </c>
       <c r="F85" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))=0,0,(C54)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C50)/('Grovfôr'!C49)))=0,0,(C54)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C50)/('Grovfôr'!C49))))</t>
         </is>
       </c>
     </row>
@@ -12858,7 +13044,7 @@
         </is>
       </c>
       <c r="C86" s="40">
-        <f>'Grovfôr'!C60</f>
+        <f>'Grovfôr'!C63</f>
         <v/>
       </c>
       <c r="D86" s="28" t="inlineStr">
@@ -12868,12 +13054,12 @@
       </c>
       <c r="E86" s="29" t="inlineStr">
         <is>
-          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C60]</t>
+          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C63]</t>
         </is>
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C60</t>
+          <t>='Grovfôr'!C63</t>
         </is>
       </c>
     </row>
@@ -12889,7 +13075,7 @@
         </is>
       </c>
       <c r="C87" s="40">
-        <f>'Grovfôr'!C61</f>
+        <f>'Grovfôr'!C64</f>
         <v/>
       </c>
       <c r="D87" s="28" t="inlineStr">
@@ -12899,12 +13085,12 @@
       </c>
       <c r="E87" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C61]</t>
+          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C64]</t>
         </is>
       </c>
       <c r="F87" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C61</t>
+          <t>='Grovfôr'!C64</t>
         </is>
       </c>
     </row>
@@ -12920,7 +13106,7 @@
         </is>
       </c>
       <c r="C88" s="40">
-        <f>'Grovfôr'!C62</f>
+        <f>'Grovfôr'!C65</f>
         <v/>
       </c>
       <c r="D88" s="28" t="inlineStr">
@@ -12930,12 +13116,12 @@
       </c>
       <c r="E88" s="29" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining» (heile garden) = Korrigerte dekar pr «kueining» [Grovfôr!C62]</t>
+          <t>Korrigerte dekar pr «kueining» (heile garden) = Korrigerte dekar pr «kueining» [Grovfôr!C65]</t>
         </is>
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C62</t>
+          <t>='Grovfôr'!C65</t>
         </is>
       </c>
     </row>
@@ -12951,7 +13137,7 @@
         </is>
       </c>
       <c r="C89" s="39">
-        <f>IF((C56)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))/(C56))</f>
+        <f>IF((C56)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C50)/('Grovfôr'!C49)))/(C56))</f>
         <v/>
       </c>
       <c r="D89" s="28" t="inlineStr">
@@ -12961,50 +13147,50 @@
       </c>
       <c r="E89" s="29" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining» i produksjonen = (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46]) ÷ «Kueiningar» [C56]   (Grovfôrarealet produksjonen får (etter eigen grovfôrkostnad) delt på kueiningane i produksjonen)</t>
+          <t>Korrigerte dekar pr «kueining» i produksjonen = (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C49]) ÷ «Kueiningar» [C56]   (Grovfôrarealet produksjonen får (etter eigen grovfôrkostnad) delt på kueiningane i produksjonen)</t>
         </is>
       </c>
       <c r="F89" s="30" t="inlineStr">
         <is>
-          <t>=IF((C56)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))/(C56))</t>
+          <t>=IF((C56)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C50)/('Grovfôr'!C49)))/(C56))</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="25" t="inlineStr">
         <is>
-          <t>Snitt slaktepris pr okse</t>
+          <t>Korrigerte dekar pr «kueining» – storfe samla</t>
         </is>
       </c>
       <c r="B90" s="26" t="inlineStr">
         <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C90" s="39">
-        <f>IF((C9)=0,0,(C21)/(C9))</f>
+          <t>Lenkje frå anna ark</t>
+        </is>
+      </c>
+      <c r="C90" s="40">
+        <f>'Grovfôr'!C42</f>
         <v/>
       </c>
       <c r="D90" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>da</t>
         </is>
       </c>
       <c r="E90" s="29" t="inlineStr">
         <is>
-          <t>Snitt slaktepris pr okse = Slakt [C21] ÷ Tal slakta oksar [C9]</t>
+          <t>Korrigerte dekar pr «kueining» – storfe samla = Korrigerte dekar pr «kueining» – storfe [Grovfôr!C42]   (Som i Agro: grovfôrarealet til alle storfeproduksjonane delt på storfe-kueiningane)</t>
         </is>
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>=IF((C9)=0,0,(C21)/(C9))</t>
+          <t>='Grovfôr'!C42</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="25" t="inlineStr">
         <is>
-          <t>Snitt kjøpspris pr kalv</t>
+          <t>Snitt slaktepris pr okse</t>
         </is>
       </c>
       <c r="B91" s="26" t="inlineStr">
@@ -13013,7 +13199,7 @@
         </is>
       </c>
       <c r="C91" s="39">
-        <f>IF((C11)=0,0,(C41)/(C11))</f>
+        <f>IF((C9)=0,0,(C21)/(C9))</f>
         <v/>
       </c>
       <c r="D91" s="28" t="inlineStr">
@@ -13023,19 +13209,19 @@
       </c>
       <c r="E91" s="29" t="inlineStr">
         <is>
-          <t>Snitt kjøpspris pr kalv = Innkjøp dyr [C41] ÷ Tal kjøpte kalvar [C11]</t>
+          <t>Snitt slaktepris pr okse = Slakt [C21] ÷ Tal slakta oksar [C9]</t>
         </is>
       </c>
       <c r="F91" s="30" t="inlineStr">
         <is>
-          <t>=IF((C11)=0,0,(C41)/(C11))</t>
+          <t>=IF((C9)=0,0,(C21)/(C9))</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="25" t="inlineStr">
         <is>
-          <t>Slaktepris – kjøpspris pr okse</t>
+          <t>Snitt kjøpspris pr kalv</t>
         </is>
       </c>
       <c r="B92" s="26" t="inlineStr">
@@ -13044,7 +13230,7 @@
         </is>
       </c>
       <c r="C92" s="39">
-        <f>IF((C9)=0,0,(C21)/(C9))-IF((C11)=0,0,(C41)/(C11))</f>
+        <f>IF((C11)=0,0,(C41)/(C11))</f>
         <v/>
       </c>
       <c r="D92" s="28" t="inlineStr">
@@ -13054,19 +13240,19 @@
       </c>
       <c r="E92" s="29" t="inlineStr">
         <is>
-          <t>Slaktepris – kjøpspris pr okse = Slakt [C21] ÷ Tal slakta oksar [C9] − Innkjøp dyr [C41] ÷ Tal kjøpte kalvar [C11]</t>
+          <t>Snitt kjøpspris pr kalv = Innkjøp dyr [C41] ÷ Tal kjøpte kalvar [C11]</t>
         </is>
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>=IF((C9)=0,0,(C21)/(C9))-IF((C11)=0,0,(C41)/(C11))</t>
+          <t>=IF((C11)=0,0,(C41)/(C11))</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="25" t="inlineStr">
         <is>
-          <t>Oppnådd pris pr kg slakt (u/distriktstilskot)</t>
+          <t>Slaktepris – kjøpspris pr okse</t>
         </is>
       </c>
       <c r="B93" s="26" t="inlineStr">
@@ -13075,7 +13261,7 @@
         </is>
       </c>
       <c r="C93" s="39">
-        <f>IF((C8)=0,0,(C21-C25)/(C8))</f>
+        <f>IF((C9)=0,0,(C21)/(C9))-IF((C11)=0,0,(C41)/(C11))</f>
         <v/>
       </c>
       <c r="D93" s="28" t="inlineStr">
@@ -13085,19 +13271,19 @@
       </c>
       <c r="E93" s="29" t="inlineStr">
         <is>
-          <t>Oppnådd pris pr kg slakt (u/distriktstilskot) = (Slakt [C21] − Herav distriktstilskot kjøt [C25]) ÷ Kg slakt [C8]</t>
+          <t>Slaktepris – kjøpspris pr okse = Slakt [C21] ÷ Tal slakta oksar [C9] − Innkjøp dyr [C41] ÷ Tal kjøpte kalvar [C11]</t>
         </is>
       </c>
       <c r="F93" s="30" t="inlineStr">
         <is>
-          <t>=IF((C8)=0,0,(C21-C25)/(C8))</t>
+          <t>=IF((C9)=0,0,(C21)/(C9))-IF((C11)=0,0,(C41)/(C11))</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="25" t="inlineStr">
         <is>
-          <t>Slaktevekt pr okse (kg)</t>
+          <t>Oppnådd pris pr kg slakt (u/distriktstilskot)</t>
         </is>
       </c>
       <c r="B94" s="26" t="inlineStr">
@@ -13105,30 +13291,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C94" s="37">
-        <f>IF((C9)=0,0,(C8)/(C9))</f>
+      <c r="C94" s="39">
+        <f>IF((C8)=0,0,(C21-C25)/(C8))</f>
         <v/>
       </c>
       <c r="D94" s="28" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E94" s="29" t="inlineStr">
         <is>
-          <t>Slaktevekt pr okse (kg) = Kg slakt [C8] ÷ Tal slakta oksar [C9]</t>
+          <t>Oppnådd pris pr kg slakt (u/distriktstilskot) = (Slakt [C21] − Herav distriktstilskot kjøt [C25]) ÷ Kg slakt [C8]</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>=IF((C9)=0,0,(C8)/(C9))</t>
+          <t>=IF((C8)=0,0,(C21-C25)/(C8))</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="25" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr okse</t>
+          <t>Slaktevekt pr okse (kg)</t>
         </is>
       </c>
       <c r="B95" s="26" t="inlineStr">
@@ -13136,52 +13322,83 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C95" s="39">
-        <f>IF((C7)=0,0,(C45)/(C7))</f>
+      <c r="C95" s="37">
+        <f>IF((C9)=0,0,(C8)/(C9))</f>
         <v/>
       </c>
       <c r="D95" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E95" s="29" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr okse = Innandørsmekanisering fordelt [C45] ÷ Tal produserte oksar [C7]</t>
+          <t>Slaktevekt pr okse (kg) = Kg slakt [C8] ÷ Tal slakta oksar [C9]</t>
         </is>
       </c>
       <c r="F95" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C45)/(C7))</t>
+          <t>=IF((C9)=0,0,(C8)/(C9))</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="25" t="inlineStr">
         <is>
+          <t>Innandørsmekanisering pr okse</t>
+        </is>
+      </c>
+      <c r="B96" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C96" s="39">
+        <f>IF((C7)=0,0,(C45)/(C7))</f>
+        <v/>
+      </c>
+      <c r="D96" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E96" s="29" t="inlineStr">
+        <is>
+          <t>Innandørsmekanisering pr okse = Innandørsmekanisering fordelt [C45] ÷ Tal produserte oksar [C7]</t>
+        </is>
+      </c>
+      <c r="F96" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C7)=0,0,(C45)/(C7))</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="25" t="inlineStr">
+        <is>
           <t>Tapsprosent</t>
         </is>
       </c>
-      <c r="B96" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C96" s="33">
+      <c r="B97" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C97" s="33">
         <f>MAX(0,IF((C12+C14+C11)=0,0,((C12+C14+C11)-(C13+C15+C9+C10))/(C12+C14+C11)))</f>
         <v/>
       </c>
-      <c r="D96" s="28" t="inlineStr">
+      <c r="D97" s="28" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E96" s="29" t="inlineStr">
+      <c r="E97" s="29" t="inlineStr">
         <is>
           <t>Tapsprosent = MAKS(0; ((Oksar over 12 md pr 1.1. [C12] + Oksar/kalvar under 12 md pr 1.1. [C14] + Tal kjøpte kalvar [C11]) − (Oksar over 12 md pr 31.12. [C13] + Oksar/kalvar under 12 md pr 31.12. [C15] + Tal slakta oksar [C9] + Tal storfe selt til liv [C10])) ÷ (Oksar over 12 md pr 1.1. [C12] + Oksar/kalvar under 12 md pr 1.1. [C14] + Tal kjøpte kalvar [C11]))   ((Inngåande dyr + kjøpte) – (utgåande dyr + slakta + selde), delt på inngåande + kjøpte)</t>
         </is>
       </c>
-      <c r="F96" s="30" t="inlineStr">
+      <c r="F97" s="30" t="inlineStr">
         <is>
           <t>=MAX(0,IF((C12+C14+C11)=0,0,((C12+C14+C11)-(C13+C15+C9+C10))/(C12+C14+C11)))</t>
         </is>
@@ -13199,7 +13416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F96"/>
+  <dimension ref="A1:F97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -15319,7 +15536,7 @@
         </is>
       </c>
       <c r="C84" s="39">
-        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))=0,0,(C53)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C50)/('Grovfôr'!C49)))=0,0,(C53)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C50)/('Grovfôr'!C49))))</f>
         <v/>
       </c>
       <c r="D84" s="28" t="inlineStr">
@@ -15329,12 +15546,12 @@
       </c>
       <c r="E84" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C53] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
+          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C53] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C49])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
         </is>
       </c>
       <c r="F84" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))=0,0,(C53)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C50)/('Grovfôr'!C49)))=0,0,(C53)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C50)/('Grovfôr'!C49))))</t>
         </is>
       </c>
     </row>
@@ -15350,7 +15567,7 @@
         </is>
       </c>
       <c r="C85" s="39">
-        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))=0,0,(C54)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C50)/('Grovfôr'!C49)))=0,0,(C54)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C50)/('Grovfôr'!C49))))</f>
         <v/>
       </c>
       <c r="D85" s="28" t="inlineStr">
@@ -15360,12 +15577,12 @@
       </c>
       <c r="E85" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C54] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])</t>
+          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C54] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C49])</t>
         </is>
       </c>
       <c r="F85" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))=0,0,(C54)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C50)/('Grovfôr'!C49)))=0,0,(C54)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C50)/('Grovfôr'!C49))))</t>
         </is>
       </c>
     </row>
@@ -15381,7 +15598,7 @@
         </is>
       </c>
       <c r="C86" s="40">
-        <f>'Grovfôr'!C60</f>
+        <f>'Grovfôr'!C63</f>
         <v/>
       </c>
       <c r="D86" s="28" t="inlineStr">
@@ -15391,12 +15608,12 @@
       </c>
       <c r="E86" s="29" t="inlineStr">
         <is>
-          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C60]</t>
+          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C63]</t>
         </is>
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C60</t>
+          <t>='Grovfôr'!C63</t>
         </is>
       </c>
     </row>
@@ -15412,7 +15629,7 @@
         </is>
       </c>
       <c r="C87" s="40">
-        <f>'Grovfôr'!C61</f>
+        <f>'Grovfôr'!C64</f>
         <v/>
       </c>
       <c r="D87" s="28" t="inlineStr">
@@ -15422,12 +15639,12 @@
       </c>
       <c r="E87" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C61]</t>
+          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C64]</t>
         </is>
       </c>
       <c r="F87" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C61</t>
+          <t>='Grovfôr'!C64</t>
         </is>
       </c>
     </row>
@@ -15443,7 +15660,7 @@
         </is>
       </c>
       <c r="C88" s="40">
-        <f>'Grovfôr'!C62</f>
+        <f>'Grovfôr'!C65</f>
         <v/>
       </c>
       <c r="D88" s="28" t="inlineStr">
@@ -15453,12 +15670,12 @@
       </c>
       <c r="E88" s="29" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining» (heile garden) = Korrigerte dekar pr «kueining» [Grovfôr!C62]</t>
+          <t>Korrigerte dekar pr «kueining» (heile garden) = Korrigerte dekar pr «kueining» [Grovfôr!C65]</t>
         </is>
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C62</t>
+          <t>='Grovfôr'!C65</t>
         </is>
       </c>
     </row>
@@ -15474,7 +15691,7 @@
         </is>
       </c>
       <c r="C89" s="39">
-        <f>IF((C56)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))/(C56))</f>
+        <f>IF((C56)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C50)/('Grovfôr'!C49)))/(C56))</f>
         <v/>
       </c>
       <c r="D89" s="28" t="inlineStr">
@@ -15484,50 +15701,50 @@
       </c>
       <c r="E89" s="29" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining» i produksjonen = (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46]) ÷ «Kueiningar» [C56]   (Grovfôrarealet produksjonen får (etter eigen grovfôrkostnad) delt på kueiningane i produksjonen)</t>
+          <t>Korrigerte dekar pr «kueining» i produksjonen = (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C50] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C49]) ÷ «Kueiningar» [C56]   (Grovfôrarealet produksjonen får (etter eigen grovfôrkostnad) delt på kueiningane i produksjonen)</t>
         </is>
       </c>
       <c r="F89" s="30" t="inlineStr">
         <is>
-          <t>=IF((C56)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C50)/('Grovfôr'!C46)))/(C56))</t>
+          <t>=IF((C56)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C50)/('Grovfôr'!C49)))/(C56))</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="25" t="inlineStr">
         <is>
-          <t>Snitt slaktepris pr kalv (u/distriktstilskot)</t>
+          <t>Korrigerte dekar pr «kueining» – storfe samla</t>
         </is>
       </c>
       <c r="B90" s="26" t="inlineStr">
         <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C90" s="39">
-        <f>IF((C9)=0,0,(C21-C25)/(C9))</f>
+          <t>Lenkje frå anna ark</t>
+        </is>
+      </c>
+      <c r="C90" s="40">
+        <f>'Grovfôr'!C42</f>
         <v/>
       </c>
       <c r="D90" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>da</t>
         </is>
       </c>
       <c r="E90" s="29" t="inlineStr">
         <is>
-          <t>Snitt slaktepris pr kalv (u/distriktstilskot) = (Slakt [C21] − Herav distriktstilskot kjøt [C25]) ÷ Tal slakta kalvar [C9]</t>
+          <t>Korrigerte dekar pr «kueining» – storfe samla = Korrigerte dekar pr «kueining» – storfe [Grovfôr!C42]   (Som i Agro: grovfôrarealet til alle storfeproduksjonane delt på storfe-kueiningane)</t>
         </is>
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>=IF((C9)=0,0,(C21-C25)/(C9))</t>
+          <t>='Grovfôr'!C42</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="25" t="inlineStr">
         <is>
-          <t>Snitt kjøpspris pr kalv</t>
+          <t>Snitt slaktepris pr kalv (u/distriktstilskot)</t>
         </is>
       </c>
       <c r="B91" s="26" t="inlineStr">
@@ -15536,7 +15753,7 @@
         </is>
       </c>
       <c r="C91" s="39">
-        <f>IF((C11)=0,0,(C41)/(C11))</f>
+        <f>IF((C9)=0,0,(C21-C25)/(C9))</f>
         <v/>
       </c>
       <c r="D91" s="28" t="inlineStr">
@@ -15546,19 +15763,19 @@
       </c>
       <c r="E91" s="29" t="inlineStr">
         <is>
-          <t>Snitt kjøpspris pr kalv = Innkjøp dyr [C41] ÷ Tal kjøpte kalvar [C11]</t>
+          <t>Snitt slaktepris pr kalv (u/distriktstilskot) = (Slakt [C21] − Herav distriktstilskot kjøt [C25]) ÷ Tal slakta kalvar [C9]</t>
         </is>
       </c>
       <c r="F91" s="30" t="inlineStr">
         <is>
-          <t>=IF((C11)=0,0,(C41)/(C11))</t>
+          <t>=IF((C9)=0,0,(C21-C25)/(C9))</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="25" t="inlineStr">
         <is>
-          <t>Slaktepris – kjøpspris pr kalv</t>
+          <t>Snitt kjøpspris pr kalv</t>
         </is>
       </c>
       <c r="B92" s="26" t="inlineStr">
@@ -15567,7 +15784,7 @@
         </is>
       </c>
       <c r="C92" s="39">
-        <f>IF((C9)=0,0,(C21)/(C9))-IF((C11)=0,0,(C41)/(C11))</f>
+        <f>IF((C11)=0,0,(C41)/(C11))</f>
         <v/>
       </c>
       <c r="D92" s="28" t="inlineStr">
@@ -15577,19 +15794,19 @@
       </c>
       <c r="E92" s="29" t="inlineStr">
         <is>
-          <t>Slaktepris – kjøpspris pr kalv = Slakt [C21] ÷ Tal slakta kalvar [C9] − Innkjøp dyr [C41] ÷ Tal kjøpte kalvar [C11]</t>
+          <t>Snitt kjøpspris pr kalv = Innkjøp dyr [C41] ÷ Tal kjøpte kalvar [C11]</t>
         </is>
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>=IF((C9)=0,0,(C21)/(C9))-IF((C11)=0,0,(C41)/(C11))</t>
+          <t>=IF((C11)=0,0,(C41)/(C11))</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="25" t="inlineStr">
         <is>
-          <t>Oppnådd pris pr kg slakt (u/distriktstilskot)</t>
+          <t>Slaktepris – kjøpspris pr kalv</t>
         </is>
       </c>
       <c r="B93" s="26" t="inlineStr">
@@ -15598,7 +15815,7 @@
         </is>
       </c>
       <c r="C93" s="39">
-        <f>IF((C8)=0,0,(C21-C25)/(C8))</f>
+        <f>IF((C9)=0,0,(C21)/(C9))-IF((C11)=0,0,(C41)/(C11))</f>
         <v/>
       </c>
       <c r="D93" s="28" t="inlineStr">
@@ -15608,19 +15825,19 @@
       </c>
       <c r="E93" s="29" t="inlineStr">
         <is>
-          <t>Oppnådd pris pr kg slakt (u/distriktstilskot) = (Slakt [C21] − Herav distriktstilskot kjøt [C25]) ÷ Kg slakt [C8]</t>
+          <t>Slaktepris – kjøpspris pr kalv = Slakt [C21] ÷ Tal slakta kalvar [C9] − Innkjøp dyr [C41] ÷ Tal kjøpte kalvar [C11]</t>
         </is>
       </c>
       <c r="F93" s="30" t="inlineStr">
         <is>
-          <t>=IF((C8)=0,0,(C21-C25)/(C8))</t>
+          <t>=IF((C9)=0,0,(C21)/(C9))-IF((C11)=0,0,(C41)/(C11))</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="25" t="inlineStr">
         <is>
-          <t>Slaktevekt pr kalv (kg)</t>
+          <t>Oppnådd pris pr kg slakt (u/distriktstilskot)</t>
         </is>
       </c>
       <c r="B94" s="26" t="inlineStr">
@@ -15628,30 +15845,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C94" s="37">
-        <f>IF((C9)=0,0,(C8)/(C9))</f>
+      <c r="C94" s="39">
+        <f>IF((C8)=0,0,(C21-C25)/(C8))</f>
         <v/>
       </c>
       <c r="D94" s="28" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E94" s="29" t="inlineStr">
         <is>
-          <t>Slaktevekt pr kalv (kg) = Kg slakt [C8] ÷ Tal slakta kalvar [C9]</t>
+          <t>Oppnådd pris pr kg slakt (u/distriktstilskot) = (Slakt [C21] − Herav distriktstilskot kjøt [C25]) ÷ Kg slakt [C8]</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>=IF((C9)=0,0,(C8)/(C9))</t>
+          <t>=IF((C8)=0,0,(C21-C25)/(C8))</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="25" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr kalv</t>
+          <t>Slaktevekt pr kalv (kg)</t>
         </is>
       </c>
       <c r="B95" s="26" t="inlineStr">
@@ -15659,52 +15876,83 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C95" s="39">
-        <f>IF((C7)=0,0,(C45)/(C7))</f>
+      <c r="C95" s="37">
+        <f>IF((C9)=0,0,(C8)/(C9))</f>
         <v/>
       </c>
       <c r="D95" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E95" s="29" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr kalv = Innandørsmekanisering fordelt [C45] ÷ Tal produserte kalvar [C7]</t>
+          <t>Slaktevekt pr kalv (kg) = Kg slakt [C8] ÷ Tal slakta kalvar [C9]</t>
         </is>
       </c>
       <c r="F95" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C45)/(C7))</t>
+          <t>=IF((C9)=0,0,(C8)/(C9))</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="25" t="inlineStr">
         <is>
+          <t>Innandørsmekanisering pr kalv</t>
+        </is>
+      </c>
+      <c r="B96" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C96" s="39">
+        <f>IF((C7)=0,0,(C45)/(C7))</f>
+        <v/>
+      </c>
+      <c r="D96" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E96" s="29" t="inlineStr">
+        <is>
+          <t>Innandørsmekanisering pr kalv = Innandørsmekanisering fordelt [C45] ÷ Tal produserte kalvar [C7]</t>
+        </is>
+      </c>
+      <c r="F96" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C7)=0,0,(C45)/(C7))</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="25" t="inlineStr">
+        <is>
           <t>Tapsprosent</t>
         </is>
       </c>
-      <c r="B96" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C96" s="33">
+      <c r="B97" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C97" s="33">
         <f>MAX(0,IF((C12+C14+C11)=0,0,((C12+C14+C11)-(C13+C15+C9+C10))/(C12+C14+C11)))</f>
         <v/>
       </c>
-      <c r="D96" s="28" t="inlineStr">
+      <c r="D97" s="28" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E96" s="29" t="inlineStr">
+      <c r="E97" s="29" t="inlineStr">
         <is>
           <t>Tapsprosent = MAKS(0; ((Ungdyr over 12 md pr 1.1. [C12] + Kalvar under 12 md pr 1.1. [C14] + Tal kjøpte kalvar [C11]) − (Ungdyr over 12 md pr 31.12. [C13] + Kalvar under 12 md pr 31.12. [C15] + Tal slakta kalvar [C9] + Tal selt til liv [C10])) ÷ (Ungdyr over 12 md pr 1.1. [C12] + Kalvar under 12 md pr 1.1. [C14] + Tal kjøpte kalvar [C11]))</t>
         </is>
       </c>
-      <c r="F96" s="30" t="inlineStr">
+      <c r="F97" s="30" t="inlineStr">
         <is>
           <t>=MAX(0,IF((C12+C14+C11)=0,0,((C12+C14+C11)-(C13+C15+C9+C10))/(C12+C14+C11)))</t>
         </is>
@@ -15722,7 +15970,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:F102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -18003,7 +18251,7 @@
         </is>
       </c>
       <c r="C90" s="39">
-        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C55)/('Grovfôr'!C46)))=0,0,(C58)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C55)/('Grovfôr'!C46))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C55)/('Grovfôr'!C49)))=0,0,(C58)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C55)/('Grovfôr'!C49))))</f>
         <v/>
       </c>
       <c r="D90" s="28" t="inlineStr">
@@ -18013,12 +18261,12 @@
       </c>
       <c r="E90" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C58] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C55] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
+          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C58] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C55] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C49])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
         </is>
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C55)/('Grovfôr'!C46)))=0,0,(C58)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C55)/('Grovfôr'!C46))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C55)/('Grovfôr'!C49)))=0,0,(C58)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C55)/('Grovfôr'!C49))))</t>
         </is>
       </c>
     </row>
@@ -18034,7 +18282,7 @@
         </is>
       </c>
       <c r="C91" s="39">
-        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C55)/('Grovfôr'!C46)))=0,0,(C59)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C55)/('Grovfôr'!C46))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C55)/('Grovfôr'!C49)))=0,0,(C59)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C55)/('Grovfôr'!C49))))</f>
         <v/>
       </c>
       <c r="D91" s="28" t="inlineStr">
@@ -18044,12 +18292,12 @@
       </c>
       <c r="E91" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C59] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C55] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])</t>
+          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C59] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C55] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C49])</t>
         </is>
       </c>
       <c r="F91" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C55)/('Grovfôr'!C46)))=0,0,(C59)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C55)/('Grovfôr'!C46))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C55)/('Grovfôr'!C49)))=0,0,(C59)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C55)/('Grovfôr'!C49))))</t>
         </is>
       </c>
     </row>
@@ -18065,7 +18313,7 @@
         </is>
       </c>
       <c r="C92" s="40">
-        <f>'Grovfôr'!C60</f>
+        <f>'Grovfôr'!C63</f>
         <v/>
       </c>
       <c r="D92" s="28" t="inlineStr">
@@ -18075,12 +18323,12 @@
       </c>
       <c r="E92" s="29" t="inlineStr">
         <is>
-          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C60]</t>
+          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C63]</t>
         </is>
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C60</t>
+          <t>='Grovfôr'!C63</t>
         </is>
       </c>
     </row>
@@ -18096,7 +18344,7 @@
         </is>
       </c>
       <c r="C93" s="40">
-        <f>'Grovfôr'!C61</f>
+        <f>'Grovfôr'!C64</f>
         <v/>
       </c>
       <c r="D93" s="28" t="inlineStr">
@@ -18106,12 +18354,12 @@
       </c>
       <c r="E93" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C61]</t>
+          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C64]</t>
         </is>
       </c>
       <c r="F93" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C61</t>
+          <t>='Grovfôr'!C64</t>
         </is>
       </c>
     </row>
@@ -18127,7 +18375,7 @@
         </is>
       </c>
       <c r="C94" s="40">
-        <f>'Grovfôr'!C62</f>
+        <f>'Grovfôr'!C65</f>
         <v/>
       </c>
       <c r="D94" s="28" t="inlineStr">
@@ -18137,12 +18385,12 @@
       </c>
       <c r="E94" s="29" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining» (heile garden) = Korrigerte dekar pr «kueining» [Grovfôr!C62]</t>
+          <t>Korrigerte dekar pr «kueining» (heile garden) = Korrigerte dekar pr «kueining» [Grovfôr!C65]</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C62</t>
+          <t>='Grovfôr'!C65</t>
         </is>
       </c>
     </row>
@@ -18158,7 +18406,7 @@
         </is>
       </c>
       <c r="C95" s="39">
-        <f>IF((C61)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C55)/('Grovfôr'!C46)))/(C61))</f>
+        <f>IF((C61)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C55)/('Grovfôr'!C49)))/(C61))</f>
         <v/>
       </c>
       <c r="D95" s="28" t="inlineStr">
@@ -18168,50 +18416,50 @@
       </c>
       <c r="E95" s="29" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining» i produksjonen = (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C55] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46]) ÷ «Kueiningar» [C61]   (Grovfôrarealet produksjonen får (etter eigen grovfôrkostnad) delt på kueiningane i produksjonen)</t>
+          <t>Korrigerte dekar pr «kueining» i produksjonen = (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C55] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C49]) ÷ «Kueiningar» [C61]   (Grovfôrarealet produksjonen får (etter eigen grovfôrkostnad) delt på kueiningane i produksjonen)</t>
         </is>
       </c>
       <c r="F95" s="30" t="inlineStr">
         <is>
-          <t>=IF((C61)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C55)/('Grovfôr'!C46)))/(C61))</t>
+          <t>=IF((C61)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C55)/('Grovfôr'!C49)))/(C61))</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="25" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr ammeku</t>
+          <t>Korrigerte dekar pr «kueining» – storfe samla</t>
         </is>
       </c>
       <c r="B96" s="26" t="inlineStr">
         <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C96" s="39">
-        <f>IF((C7)=0,0,(C50)/(C7))</f>
+          <t>Lenkje frå anna ark</t>
+        </is>
+      </c>
+      <c r="C96" s="40">
+        <f>'Grovfôr'!C42</f>
         <v/>
       </c>
       <c r="D96" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>da</t>
         </is>
       </c>
       <c r="E96" s="29" t="inlineStr">
         <is>
-          <t>Innandørsmekanisering pr ammeku = Innandørsmekanisering fordelt [C50] ÷ Tal ammekyr [C7]</t>
+          <t>Korrigerte dekar pr «kueining» – storfe samla = Korrigerte dekar pr «kueining» – storfe [Grovfôr!C42]   (Som i Agro: grovfôrarealet til alle storfeproduksjonane delt på storfe-kueiningane)</t>
         </is>
       </c>
       <c r="F96" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C50)/(C7))</t>
+          <t>='Grovfôr'!C42</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="25" t="inlineStr">
         <is>
-          <t>Påsettprosent</t>
+          <t>Innandørsmekanisering pr ammeku</t>
         </is>
       </c>
       <c r="B97" s="26" t="inlineStr">
@@ -18219,30 +18467,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C97" s="33">
-        <f>C62</f>
+      <c r="C97" s="39">
+        <f>IF((C7)=0,0,(C50)/(C7))</f>
         <v/>
       </c>
       <c r="D97" s="28" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E97" s="29" t="inlineStr">
         <is>
-          <t>Påsettprosent = Påsettprosent [C62]</t>
+          <t>Innandørsmekanisering pr ammeku = Innandørsmekanisering fordelt [C50] ÷ Tal ammekyr [C7]</t>
         </is>
       </c>
       <c r="F97" s="30" t="inlineStr">
         <is>
-          <t>=C62</t>
+          <t>=IF((C7)=0,0,(C50)/(C7))</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="25" t="inlineStr">
         <is>
-          <t>Snitt slaktevekt kyr (kg)</t>
+          <t>Påsettprosent</t>
         </is>
       </c>
       <c r="B98" s="26" t="inlineStr">
@@ -18250,30 +18498,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C98" s="37">
-        <f>IF((C17)=0,0,(C16)/(C17))</f>
+      <c r="C98" s="33">
+        <f>C62</f>
         <v/>
       </c>
       <c r="D98" s="28" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E98" s="29" t="inlineStr">
         <is>
-          <t>Snitt slaktevekt kyr (kg) = Kg slakt kyr [C16] ÷ Tal slakta kyr [C17]</t>
+          <t>Påsettprosent = Påsettprosent [C62]</t>
         </is>
       </c>
       <c r="F98" s="30" t="inlineStr">
         <is>
-          <t>=IF((C17)=0,0,(C16)/(C17))</t>
+          <t>=C62</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="25" t="inlineStr">
         <is>
-          <t>Nyttbar kalv pr ku</t>
+          <t>Snitt slaktevekt kyr (kg)</t>
         </is>
       </c>
       <c r="B99" s="26" t="inlineStr">
@@ -18281,30 +18529,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C99" s="39">
-        <f>IF((C7)=0,0,((C9+C11+C13+C15)+C19-C20-(C8+C10+C12+C14))/(C7))</f>
+      <c r="C99" s="37">
+        <f>IF((C17)=0,0,(C16)/(C17))</f>
         <v/>
       </c>
       <c r="D99" s="28" t="inlineStr">
         <is>
-          <t>stk</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E99" s="29" t="inlineStr">
         <is>
-          <t>Nyttbar kalv pr ku = ((Ammekyr pr 31.12. [C9] + Avlsokse pr 31.12. [C11] + Ungdyr over 12 md pr 31.12. [C13] + Kalvar/ungdyr under 12 md pr 31.12. [C15]) + Tal dyr slakta / selt til liv [C19] − Tal kjøpte dyr [C20] − (Ammekyr pr 1.1. [C8] + Avlsokse pr 1.1. [C10] + Ungdyr over 12 md pr 1.1. [C12] + Kalvar/ungdyr under 12 md pr 1.1. [C14])) ÷ Tal ammekyr [C7]   ((Dyr 31.12. + slakta/selde – kjøpte – dyr 1.1.) delt på tal ammekyr)</t>
+          <t>Snitt slaktevekt kyr (kg) = Kg slakt kyr [C16] ÷ Tal slakta kyr [C17]</t>
         </is>
       </c>
       <c r="F99" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,((C9+C11+C13+C15)+C19-C20-(C8+C10+C12+C14))/(C7))</t>
+          <t>=IF((C17)=0,0,(C16)/(C17))</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="25" t="inlineStr">
         <is>
-          <t>Oppnådd pris pr kg slakt (u/distriktstilskot)</t>
+          <t>Nyttbar kalv pr ku</t>
         </is>
       </c>
       <c r="B100" s="26" t="inlineStr">
@@ -18313,51 +18561,82 @@
         </is>
       </c>
       <c r="C100" s="39">
-        <f>IF((C18)=0,0,(C27-C30)/(C18))</f>
+        <f>IF((C7)=0,0,((C9+C11+C13+C15)+C19-C20-(C8+C10+C12+C14))/(C7))</f>
         <v/>
       </c>
       <c r="D100" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>stk</t>
         </is>
       </c>
       <c r="E100" s="29" t="inlineStr">
         <is>
-          <t>Oppnådd pris pr kg slakt (u/distriktstilskot) = (Slakt [C27] − Herav distriktstilskot kjøt [C30]) ÷ Kg slakt totalt [C18]</t>
+          <t>Nyttbar kalv pr ku = ((Ammekyr pr 31.12. [C9] + Avlsokse pr 31.12. [C11] + Ungdyr over 12 md pr 31.12. [C13] + Kalvar/ungdyr under 12 md pr 31.12. [C15]) + Tal dyr slakta / selt til liv [C19] − Tal kjøpte dyr [C20] − (Ammekyr pr 1.1. [C8] + Avlsokse pr 1.1. [C10] + Ungdyr over 12 md pr 1.1. [C12] + Kalvar/ungdyr under 12 md pr 1.1. [C14])) ÷ Tal ammekyr [C7]   ((Dyr 31.12. + slakta/selde – kjøpte – dyr 1.1.) delt på tal ammekyr)</t>
         </is>
       </c>
       <c r="F100" s="30" t="inlineStr">
         <is>
-          <t>=IF((C18)=0,0,(C27-C30)/(C18))</t>
+          <t>=IF((C7)=0,0,((C9+C11+C13+C15)+C19-C20-(C8+C10+C12+C14))/(C7))</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="25" t="inlineStr">
         <is>
+          <t>Oppnådd pris pr kg slakt (u/distriktstilskot)</t>
+        </is>
+      </c>
+      <c r="B101" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C101" s="39">
+        <f>IF((C18)=0,0,(C27-C30)/(C18))</f>
+        <v/>
+      </c>
+      <c r="D101" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E101" s="29" t="inlineStr">
+        <is>
+          <t>Oppnådd pris pr kg slakt (u/distriktstilskot) = (Slakt [C27] − Herav distriktstilskot kjøt [C30]) ÷ Kg slakt totalt [C18]</t>
+        </is>
+      </c>
+      <c r="F101" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C18)=0,0,(C27-C30)/(C18))</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="25" t="inlineStr">
+        <is>
           <t>Analysegruppe (påsett)</t>
         </is>
       </c>
-      <c r="B101" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C101" s="41">
+      <c r="B102" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C102" s="41">
         <f>IF(C62&gt;0.5,"Påsett &gt; 50 %","Påsett &lt; 50 %")</f>
         <v/>
       </c>
-      <c r="D101" s="28" t="inlineStr">
+      <c r="D102" s="28" t="inlineStr">
         <is>
           <t>tekst</t>
         </is>
       </c>
-      <c r="E101" s="29" t="inlineStr">
+      <c r="E102" s="29" t="inlineStr">
         <is>
           <t>Analysegruppe (påsett) = HVIS(Påsettprosent [C62]&gt;0,5; "Påsett &gt; 50 %"; "Påsett &lt; 50 %")   (Tilsvarar arka «Ammekyr &lt;50%» og «Ammekyr &gt;50%» i eksempelanalysen)</t>
         </is>
       </c>
-      <c r="F101" s="30" t="inlineStr">
+      <c r="F102" s="30" t="inlineStr">
         <is>
           <t>=IF(C62&gt;0.5,"Påsett &gt; 50 %","Påsett &lt; 50 %")</t>
         </is>
@@ -27771,7 +28050,7 @@
         </is>
       </c>
       <c r="C100" s="39">
-        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C61)/('Grovfôr'!C46)))=0,0,(C64)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C61)/('Grovfôr'!C46))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C61)/('Grovfôr'!C49)))=0,0,(C64)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C61)/('Grovfôr'!C49))))</f>
         <v/>
       </c>
       <c r="D100" s="28" t="inlineStr">
@@ -27781,12 +28060,12 @@
       </c>
       <c r="E100" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C64] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C61] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
+          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C64] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C61] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C49])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
         </is>
       </c>
       <c r="F100" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C61)/('Grovfôr'!C46)))=0,0,(C64)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C61)/('Grovfôr'!C46))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C61)/('Grovfôr'!C49)))=0,0,(C64)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C61)/('Grovfôr'!C49))))</t>
         </is>
       </c>
     </row>
@@ -27802,7 +28081,7 @@
         </is>
       </c>
       <c r="C101" s="39">
-        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C61)/('Grovfôr'!C46)))=0,0,(C65)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C61)/('Grovfôr'!C46))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C61)/('Grovfôr'!C49)))=0,0,(C65)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C61)/('Grovfôr'!C49))))</f>
         <v/>
       </c>
       <c r="D101" s="28" t="inlineStr">
@@ -27812,12 +28091,12 @@
       </c>
       <c r="E101" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C65] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C61] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])</t>
+          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C65] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C61] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C49])</t>
         </is>
       </c>
       <c r="F101" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C61)/('Grovfôr'!C46)))=0,0,(C65)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C61)/('Grovfôr'!C46))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C61)/('Grovfôr'!C49)))=0,0,(C65)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C61)/('Grovfôr'!C49))))</t>
         </is>
       </c>
     </row>
@@ -27833,7 +28112,7 @@
         </is>
       </c>
       <c r="C102" s="40">
-        <f>'Grovfôr'!C60</f>
+        <f>'Grovfôr'!C63</f>
         <v/>
       </c>
       <c r="D102" s="28" t="inlineStr">
@@ -27843,12 +28122,12 @@
       </c>
       <c r="E102" s="29" t="inlineStr">
         <is>
-          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C60]</t>
+          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C63]</t>
         </is>
       </c>
       <c r="F102" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C60</t>
+          <t>='Grovfôr'!C63</t>
         </is>
       </c>
     </row>
@@ -27864,7 +28143,7 @@
         </is>
       </c>
       <c r="C103" s="40">
-        <f>'Grovfôr'!C61</f>
+        <f>'Grovfôr'!C64</f>
         <v/>
       </c>
       <c r="D103" s="28" t="inlineStr">
@@ -27874,12 +28153,12 @@
       </c>
       <c r="E103" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C61]</t>
+          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C64]</t>
         </is>
       </c>
       <c r="F103" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C61</t>
+          <t>='Grovfôr'!C64</t>
         </is>
       </c>
     </row>
@@ -27895,7 +28174,7 @@
         </is>
       </c>
       <c r="C104" s="40">
-        <f>'Grovfôr'!C62</f>
+        <f>'Grovfôr'!C65</f>
         <v/>
       </c>
       <c r="D104" s="28" t="inlineStr">
@@ -27905,12 +28184,12 @@
       </c>
       <c r="E104" s="29" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining» (heile garden) = Korrigerte dekar pr «kueining» [Grovfôr!C62]</t>
+          <t>Korrigerte dekar pr «kueining» (heile garden) = Korrigerte dekar pr «kueining» [Grovfôr!C65]</t>
         </is>
       </c>
       <c r="F104" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C62</t>
+          <t>='Grovfôr'!C65</t>
         </is>
       </c>
     </row>
@@ -27926,7 +28205,7 @@
         </is>
       </c>
       <c r="C105" s="39">
-        <f>IF((C67)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C61)/('Grovfôr'!C46)))/(C67))</f>
+        <f>IF((C67)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C61)/('Grovfôr'!C49)))/(C67))</f>
         <v/>
       </c>
       <c r="D105" s="28" t="inlineStr">
@@ -27936,12 +28215,12 @@
       </c>
       <c r="E105" s="29" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining» i produksjonen = (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C61] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46]) ÷ «Kueiningar» [C67]   (Grovfôrarealet produksjonen får (etter eigen grovfôrkostnad) delt på kueiningane i produksjonen)</t>
+          <t>Korrigerte dekar pr «kueining» i produksjonen = (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C61] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C49]) ÷ «Kueiningar» [C67]   (Grovfôrarealet produksjonen får (etter eigen grovfôrkostnad) delt på kueiningane i produksjonen)</t>
         </is>
       </c>
       <c r="F105" s="30" t="inlineStr">
         <is>
-          <t>=IF((C67)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C61)/('Grovfôr'!C46)))/(C67))</t>
+          <t>=IF((C67)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C61)/('Grovfôr'!C49)))/(C67))</t>
         </is>
       </c>
     </row>
@@ -30299,7 +30578,7 @@
         </is>
       </c>
       <c r="C85" s="39">
-        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C49)/('Grovfôr'!C46)))=0,0,(C52)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C49)/('Grovfôr'!C46))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C49)/('Grovfôr'!C49)))=0,0,(C52)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C49)/('Grovfôr'!C49))))</f>
         <v/>
       </c>
       <c r="D85" s="28" t="inlineStr">
@@ -30309,12 +30588,12 @@
       </c>
       <c r="E85" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C52] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C49] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
+          <t>DB pr dekar grovfôr u/tilskot = Dekningsbidrag (DB) utan tilskot [C52] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C49] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C49])   (Grovfôrarealet blir fordelt etter produksjonen sin del av eigen grovfôrkostnad)</t>
         </is>
       </c>
       <c r="F85" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C49)/('Grovfôr'!C46)))=0,0,(C52)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C49)/('Grovfôr'!C46))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C49)/('Grovfôr'!C49)))=0,0,(C52)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C49)/('Grovfôr'!C49))))</t>
         </is>
       </c>
     </row>
@@ -30330,7 +30609,7 @@
         </is>
       </c>
       <c r="C86" s="39">
-        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C49)/('Grovfôr'!C46)))=0,0,(C53)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C49)/('Grovfôr'!C46))))</f>
+        <f>IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C49)/('Grovfôr'!C49)))=0,0,(C53)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C49)/('Grovfôr'!C49))))</f>
         <v/>
       </c>
       <c r="D86" s="28" t="inlineStr">
@@ -30340,12 +30619,12 @@
       </c>
       <c r="E86" s="29" t="inlineStr">
         <is>
-          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C53] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C49] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46])</t>
+          <t>DB pr dekar grovfôr m/tilskot = Dekningsbidrag (DB) med tilskot [C53] ÷ (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C49] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C49])</t>
         </is>
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C49)/('Grovfôr'!C46)))=0,0,(C53)/('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C49)/('Grovfôr'!C46))))</t>
+          <t>=IF(('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C49)/('Grovfôr'!C49)))=0,0,(C53)/('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C49)/('Grovfôr'!C49))))</t>
         </is>
       </c>
     </row>
@@ -30361,7 +30640,7 @@
         </is>
       </c>
       <c r="C87" s="40">
-        <f>'Grovfôr'!C60</f>
+        <f>'Grovfôr'!C63</f>
         <v/>
       </c>
       <c r="D87" s="28" t="inlineStr">
@@ -30371,12 +30650,12 @@
       </c>
       <c r="E87" s="29" t="inlineStr">
         <is>
-          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C60]</t>
+          <t>Variabel grovfôrkostnad pr dekar = Variabel grovfôrkostnad pr korrigert dekar [Grovfôr!C63]</t>
         </is>
       </c>
       <c r="F87" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C60</t>
+          <t>='Grovfôr'!C63</t>
         </is>
       </c>
     </row>
@@ -30392,7 +30671,7 @@
         </is>
       </c>
       <c r="C88" s="40">
-        <f>'Grovfôr'!C61</f>
+        <f>'Grovfôr'!C64</f>
         <v/>
       </c>
       <c r="D88" s="28" t="inlineStr">
@@ -30402,12 +30681,12 @@
       </c>
       <c r="E88" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C61]</t>
+          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader pr dekar grovfôr [Grovfôr!C64]</t>
         </is>
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C61</t>
+          <t>='Grovfôr'!C64</t>
         </is>
       </c>
     </row>
@@ -30423,7 +30702,7 @@
         </is>
       </c>
       <c r="C89" s="40">
-        <f>'Grovfôr'!C62</f>
+        <f>'Grovfôr'!C65</f>
         <v/>
       </c>
       <c r="D89" s="28" t="inlineStr">
@@ -30433,12 +30712,12 @@
       </c>
       <c r="E89" s="29" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining» (heile garden) = Korrigerte dekar pr «kueining» [Grovfôr!C62]</t>
+          <t>Korrigerte dekar pr «kueining» (heile garden) = Korrigerte dekar pr «kueining» [Grovfôr!C65]</t>
         </is>
       </c>
       <c r="F89" s="30" t="inlineStr">
         <is>
-          <t>='Grovfôr'!C62</t>
+          <t>='Grovfôr'!C65</t>
         </is>
       </c>
     </row>
@@ -30454,7 +30733,7 @@
         </is>
       </c>
       <c r="C90" s="39">
-        <f>IF((C55)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C49)/('Grovfôr'!C46)))/(C55))</f>
+        <f>IF((C55)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C49)/('Grovfôr'!C49)))/(C55))</f>
         <v/>
       </c>
       <c r="D90" s="28" t="inlineStr">
@@ -30464,12 +30743,12 @@
       </c>
       <c r="E90" s="29" t="inlineStr">
         <is>
-          <t>Korrigerte dekar pr «kueining» i produksjonen = (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C49] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C46]) ÷ «Kueiningar» [C55]   (Grovfôrarealet produksjonen får (etter eigen grovfôrkostnad) delt på kueiningane i produksjonen)</t>
+          <t>Korrigerte dekar pr «kueining» i produksjonen = (Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [Grovfôr!C22] × Sum eigen grovfôrproduksjon (utan lagerendring) [C49] ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [Grovfôr!C49]) ÷ «Kueiningar» [C55]   (Grovfôrarealet produksjonen får (etter eigen grovfôrkostnad) delt på kueiningane i produksjonen)</t>
         </is>
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>=IF((C55)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C46)=0,0,(C49)/('Grovfôr'!C46)))/(C55))</t>
+          <t>=IF((C55)=0,0,('Grovfôr'!C22*IF(('Grovfôr'!C49)=0,0,(C49)/('Grovfôr'!C49)))/(C55))</t>
         </is>
       </c>
     </row>
@@ -45114,7 +45393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -45766,7 +46045,7 @@
     <row r="28">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>Fôreiningar (FEm) henta frå utmark</t>
+          <t>Sum dekar planteproduksjon (korn, potet, grønsaker, gulrot, kålrot)</t>
         </is>
       </c>
       <c r="B28" s="21" t="inlineStr">
@@ -45774,104 +46053,104 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C28" s="22">
-        <f>C12*1.05*95+C13*1*90+C14*7.2*92+C15*4.8*92</f>
+      <c r="C28" s="36">
+        <f>Korn!C7*IF(Oversikt!$B$7="J",1,0)+Potet!C7*IF(Oversikt!$B$10="J",1,0)+'Frilandsgrønsak'!C7*IF(Oversikt!$B$13="J",1,0)+Gulrot!C7*IF(Oversikt!$B$14="J",1,0)+'Kålrot'!C7*IF(Oversikt!$B$15="J",1,0)</f>
         <v/>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>FEm</t>
+          <t>da</t>
         </is>
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
-          <t>Fôreiningar (FEm) henta frå utmark = Sau på utmarksbeite (1,05 FEm/dag, 95 dagar) [C12] × 1,05 × 95 + Lam på utmarksbeite (1 FEm/dag, 90 dagar) [C13] × 1 × 90 + Kyr på utmarksbeite (7,2 FEm/dag, 92 dagar) [C14] × 7,2 × 92 + Ungdyr på utmarksbeite (4,8 FEm/dag, 92 dagar) [C15] × 4,8 × 92</t>
+          <t>Sum dekar planteproduksjon (korn, potet, grønsaker, gulrot, kålrot) = Tal dekar [Korn!C7] × Med i totalen Korn [Oversikt!B7 → 1/0] + Tal dekar [Potet!C7] × Med i totalen Potet [Oversikt!B10 → 1/0] + Tal dekar [Frilandsgrønsak!C7] × Med i totalen Frilandsgrønsak [Oversikt!B13 → 1/0] + Tal dekar [Gulrot!C7] × Med i totalen Gulrot [Oversikt!B14 → 1/0] + Tal dekar [Kålrot!C7] × Med i totalen Kålrot [Oversikt!B15 → 1/0]</t>
         </is>
       </c>
       <c r="F28" s="24" t="inlineStr">
         <is>
-          <t>=C12*1.05*95+C13*1*90+C14*7.2*92+C15*4.8*92</t>
+          <t>=Korn!C7*IF(Oversikt!$B$7="J",1,0)+Potet!C7*IF(Oversikt!$B$10="J",1,0)+'Frilandsgrønsak'!C7*IF(Oversikt!$B$13="J",1,0)+Gulrot!C7*IF(Oversikt!$B$14="J",1,0)+'Kålrot'!C7*IF(Oversikt!$B$15="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="20" t="inlineStr">
         <is>
+          <t>Fôreiningar (FEm) henta frå utmark</t>
+        </is>
+      </c>
+      <c r="B29" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C29" s="22">
+        <f>C12*1.05*95+C13*1*90+C14*7.2*92+C15*4.8*92</f>
+        <v/>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>FEm</t>
+        </is>
+      </c>
+      <c r="E29" s="23" t="inlineStr">
+        <is>
+          <t>Fôreiningar (FEm) henta frå utmark = Sau på utmarksbeite (1,05 FEm/dag, 95 dagar) [C12] × 1,05 × 95 + Lam på utmarksbeite (1 FEm/dag, 90 dagar) [C13] × 1 × 90 + Kyr på utmarksbeite (7,2 FEm/dag, 92 dagar) [C14] × 7,2 × 92 + Ungdyr på utmarksbeite (4,8 FEm/dag, 92 dagar) [C15] × 4,8 × 92</t>
+        </is>
+      </c>
+      <c r="F29" s="24" t="inlineStr">
+        <is>
+          <t>=C12*1.05*95+C13*1*90+C14*7.2*92+C15*4.8*92</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
           <t>Utmark omrekna til «fulldyrka» dekar (900 FEm/da)</t>
         </is>
       </c>
-      <c r="B29" s="21" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C29" s="36">
-        <f>C28/900</f>
-        <v/>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
+      <c r="B30" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C30" s="36">
+        <f>C29/900</f>
+        <v/>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
         <is>
           <t>da</t>
         </is>
       </c>
-      <c r="E29" s="23" t="inlineStr">
-        <is>
-          <t>Utmark omrekna til «fulldyrka» dekar (900 FEm/da) = Fôreiningar (FEm) henta frå utmark [C28] / 900</t>
-        </is>
-      </c>
-      <c r="F29" s="24" t="inlineStr">
-        <is>
-          <t>=C28/900</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="18" t="inlineStr">
+      <c r="E30" s="23" t="inlineStr">
+        <is>
+          <t>Utmark omrekna til «fulldyrka» dekar (900 FEm/da) = Fôreiningar (FEm) henta frå utmark [C29] / 900</t>
+        </is>
+      </c>
+      <c r="F30" s="24" t="inlineStr">
+        <is>
+          <t>=C29/900</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="18" t="inlineStr">
         <is>
           <t>4. UTREKNING – «Kueiningar» og eigen grovfôrkostnad pr produksjon (berre produksjonar med i totalen)</t>
         </is>
       </c>
-      <c r="B30" s="19" t="n"/>
-      <c r="C30" s="19" t="n"/>
-      <c r="D30" s="19" t="n"/>
-      <c r="E30" s="19" t="n"/>
-      <c r="F30" s="19" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="20" t="inlineStr">
-        <is>
-          <t>Kueiningar – Mjølk</t>
-        </is>
-      </c>
-      <c r="B31" s="21" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C31" s="38">
-        <f>'Mjølk'!C59*IF(Oversikt!$B$16="J",1,0)</f>
-        <v/>
-      </c>
-      <c r="D31" s="12" t="inlineStr">
-        <is>
-          <t>stk</t>
-        </is>
-      </c>
-      <c r="E31" s="23" t="inlineStr">
-        <is>
-          <t>Kueiningar – Mjølk = «Kueiningar» [Mjølk!C59] × Med i totalen Mjølk [Oversikt!B16 → 1/0]</t>
-        </is>
-      </c>
-      <c r="F31" s="24" t="inlineStr">
-        <is>
-          <t>='Mjølk'!C59*IF(Oversikt!$B$16="J",1,0)</t>
-        </is>
-      </c>
+      <c r="B31" s="19" t="n"/>
+      <c r="C31" s="19" t="n"/>
+      <c r="D31" s="19" t="n"/>
+      <c r="E31" s="19" t="n"/>
+      <c r="F31" s="19" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>Kueiningar – Oksar</t>
+          <t>Kueiningar – Mjølk</t>
         </is>
       </c>
       <c r="B32" s="21" t="inlineStr">
@@ -45880,7 +46159,7 @@
         </is>
       </c>
       <c r="C32" s="38">
-        <f>Oksar!C56*IF(Oversikt!$B$17="J",1,0)</f>
+        <f>'Mjølk'!C59*IF(Oversikt!$B$16="J",1,0)</f>
         <v/>
       </c>
       <c r="D32" s="12" t="inlineStr">
@@ -45890,19 +46169,19 @@
       </c>
       <c r="E32" s="23" t="inlineStr">
         <is>
-          <t>Kueiningar – Oksar = «Kueiningar» [Oksar!C56] × Med i totalen Oksar [Oversikt!B17 → 1/0]</t>
+          <t>Kueiningar – Mjølk = «Kueiningar» [Mjølk!C59] × Med i totalen Mjølk [Oversikt!B16 → 1/0]</t>
         </is>
       </c>
       <c r="F32" s="24" t="inlineStr">
         <is>
-          <t>=Oksar!C56*IF(Oversikt!$B$17="J",1,0)</t>
+          <t>='Mjølk'!C59*IF(Oversikt!$B$16="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>Kueiningar – Mellomkalv</t>
+          <t>Kueiningar – Oksar</t>
         </is>
       </c>
       <c r="B33" s="21" t="inlineStr">
@@ -45911,7 +46190,7 @@
         </is>
       </c>
       <c r="C33" s="38">
-        <f>Mellomkalv!C56*IF(Oversikt!$B$18="J",1,0)</f>
+        <f>Oksar!C56*IF(Oversikt!$B$17="J",1,0)</f>
         <v/>
       </c>
       <c r="D33" s="12" t="inlineStr">
@@ -45921,19 +46200,19 @@
       </c>
       <c r="E33" s="23" t="inlineStr">
         <is>
-          <t>Kueiningar – Mellomkalv = «Kueiningar» [Mellomkalv!C56] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0]</t>
+          <t>Kueiningar – Oksar = «Kueiningar» [Oksar!C56] × Med i totalen Oksar [Oversikt!B17 → 1/0]</t>
         </is>
       </c>
       <c r="F33" s="24" t="inlineStr">
         <is>
-          <t>=Mellomkalv!C56*IF(Oversikt!$B$18="J",1,0)</t>
+          <t>=Oksar!C56*IF(Oversikt!$B$17="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>Kueiningar – Ammekyr</t>
+          <t>Kueiningar – Mellomkalv</t>
         </is>
       </c>
       <c r="B34" s="21" t="inlineStr">
@@ -45942,7 +46221,7 @@
         </is>
       </c>
       <c r="C34" s="38">
-        <f>Ammekyr!C61*IF(Oversikt!$B$19="J",1,0)</f>
+        <f>Mellomkalv!C56*IF(Oversikt!$B$18="J",1,0)</f>
         <v/>
       </c>
       <c r="D34" s="12" t="inlineStr">
@@ -45952,19 +46231,19 @@
       </c>
       <c r="E34" s="23" t="inlineStr">
         <is>
-          <t>Kueiningar – Ammekyr = «Kueiningar» [Ammekyr!C61] × Med i totalen Ammekyr [Oversikt!B19 → 1/0]</t>
+          <t>Kueiningar – Mellomkalv = «Kueiningar» [Mellomkalv!C56] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0]</t>
         </is>
       </c>
       <c r="F34" s="24" t="inlineStr">
         <is>
-          <t>=Ammekyr!C61*IF(Oversikt!$B$19="J",1,0)</t>
+          <t>=Mellomkalv!C56*IF(Oversikt!$B$18="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>Kueiningar – Sau</t>
+          <t>Kueiningar – Ammekyr</t>
         </is>
       </c>
       <c r="B35" s="21" t="inlineStr">
@@ -45973,7 +46252,7 @@
         </is>
       </c>
       <c r="C35" s="38">
-        <f>Sau!C67*IF(Oversikt!$B$23="J",1,0)</f>
+        <f>Ammekyr!C61*IF(Oversikt!$B$19="J",1,0)</f>
         <v/>
       </c>
       <c r="D35" s="12" t="inlineStr">
@@ -45983,19 +46262,19 @@
       </c>
       <c r="E35" s="23" t="inlineStr">
         <is>
-          <t>Kueiningar – Sau = «Kueiningar» [Sau!C67] × Med i totalen Sau [Oversikt!B23 → 1/0]</t>
+          <t>Kueiningar – Ammekyr = «Kueiningar» [Ammekyr!C61] × Med i totalen Ammekyr [Oversikt!B19 → 1/0]</t>
         </is>
       </c>
       <c r="F35" s="24" t="inlineStr">
         <is>
-          <t>=Sau!C67*IF(Oversikt!$B$23="J",1,0)</t>
+          <t>=Ammekyr!C61*IF(Oversikt!$B$19="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>Kueiningar – Geit</t>
+          <t>Kueiningar – Sau</t>
         </is>
       </c>
       <c r="B36" s="21" t="inlineStr">
@@ -46004,7 +46283,7 @@
         </is>
       </c>
       <c r="C36" s="38">
-        <f>Geit!C55*IF(Oversikt!$B$24="J",1,0)</f>
+        <f>Sau!C67*IF(Oversikt!$B$23="J",1,0)</f>
         <v/>
       </c>
       <c r="D36" s="12" t="inlineStr">
@@ -46014,19 +46293,19 @@
       </c>
       <c r="E36" s="23" t="inlineStr">
         <is>
-          <t>Kueiningar – Geit = «Kueiningar» [Geit!C55] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
+          <t>Kueiningar – Sau = «Kueiningar» [Sau!C67] × Med i totalen Sau [Oversikt!B23 → 1/0]</t>
         </is>
       </c>
       <c r="F36" s="24" t="inlineStr">
         <is>
-          <t>=Geit!C55*IF(Oversikt!$B$24="J",1,0)</t>
+          <t>=Sau!C67*IF(Oversikt!$B$23="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>Kueiningar – storfe</t>
+          <t>Kueiningar – Geit</t>
         </is>
       </c>
       <c r="B37" s="21" t="inlineStr">
@@ -46035,7 +46314,7 @@
         </is>
       </c>
       <c r="C37" s="38">
-        <f>C31+C32+C33+C34</f>
+        <f>Geit!C55*IF(Oversikt!$B$24="J",1,0)</f>
         <v/>
       </c>
       <c r="D37" s="12" t="inlineStr">
@@ -46045,112 +46324,112 @@
       </c>
       <c r="E37" s="23" t="inlineStr">
         <is>
-          <t>Kueiningar – storfe = Kueiningar – Mjølk [C31] + Kueiningar – Oksar [C32] + Kueiningar – Mellomkalv [C33] + Kueiningar – Ammekyr [C34]</t>
+          <t>Kueiningar – Geit = «Kueiningar» [Geit!C55] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
         </is>
       </c>
       <c r="F37" s="24" t="inlineStr">
         <is>
-          <t>=C31+C32+C33+C34</t>
+          <t>=Geit!C55*IF(Oversikt!$B$24="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="20" t="inlineStr">
         <is>
+          <t>Kueiningar – storfe</t>
+        </is>
+      </c>
+      <c r="B38" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C38" s="38">
+        <f>C32+C33+C34+C35</f>
+        <v/>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>stk</t>
+        </is>
+      </c>
+      <c r="E38" s="23" t="inlineStr">
+        <is>
+          <t>Kueiningar – storfe = Kueiningar – Mjølk [C32] + Kueiningar – Oksar [C33] + Kueiningar – Mellomkalv [C34] + Kueiningar – Ammekyr [C35]</t>
+        </is>
+      </c>
+      <c r="F38" s="24" t="inlineStr">
+        <is>
+          <t>=C32+C33+C34+C35</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="20" t="inlineStr">
+        <is>
           <t>Kueiningar – småfe</t>
         </is>
       </c>
-      <c r="B38" s="21" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C38" s="38">
-        <f>C35+C36</f>
-        <v/>
-      </c>
-      <c r="D38" s="12" t="inlineStr">
+      <c r="B39" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C39" s="38">
+        <f>C36+C37</f>
+        <v/>
+      </c>
+      <c r="D39" s="12" t="inlineStr">
         <is>
           <t>stk</t>
         </is>
       </c>
-      <c r="E38" s="23" t="inlineStr">
-        <is>
-          <t>Kueiningar – småfe = Kueiningar – Sau [C35] + Kueiningar – Geit [C36]</t>
-        </is>
-      </c>
-      <c r="F38" s="24" t="inlineStr">
-        <is>
-          <t>=C35+C36</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="25" t="inlineStr">
+      <c r="E39" s="23" t="inlineStr">
+        <is>
+          <t>Kueiningar – småfe = Kueiningar – Sau [C36] + Kueiningar – Geit [C37]</t>
+        </is>
+      </c>
+      <c r="F39" s="24" t="inlineStr">
+        <is>
+          <t>=C36+C37</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="25" t="inlineStr">
         <is>
           <t>Sum «kueiningar»</t>
         </is>
       </c>
-      <c r="B39" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C39" s="39">
-        <f>C37+C38</f>
-        <v/>
-      </c>
-      <c r="D39" s="28" t="inlineStr">
+      <c r="B40" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C40" s="39">
+        <f>C38+C39</f>
+        <v/>
+      </c>
+      <c r="D40" s="28" t="inlineStr">
         <is>
           <t>stk</t>
         </is>
       </c>
-      <c r="E39" s="29" t="inlineStr">
-        <is>
-          <t>Sum «kueiningar» = Kueiningar – storfe [C37] + Kueiningar – småfe [C38]</t>
-        </is>
-      </c>
-      <c r="F39" s="30" t="inlineStr">
-        <is>
-          <t>=C37+C38</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="20" t="inlineStr">
-        <is>
-          <t>Eigen grovfôrkostnad – Mjølk</t>
-        </is>
-      </c>
-      <c r="B40" s="21" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C40" s="22">
-        <f>'Mjølk'!C53*IF(Oversikt!$B$16="J",1,0)</f>
-        <v/>
-      </c>
-      <c r="D40" s="12" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E40" s="23" t="inlineStr">
-        <is>
-          <t>Eigen grovfôrkostnad – Mjølk = Sum eigen grovfôrproduksjon (utan lagerendring) [Mjølk!C53] × Med i totalen Mjølk [Oversikt!B16 → 1/0]</t>
-        </is>
-      </c>
-      <c r="F40" s="24" t="inlineStr">
-        <is>
-          <t>='Mjølk'!C53*IF(Oversikt!$B$16="J",1,0)</t>
+      <c r="E40" s="29" t="inlineStr">
+        <is>
+          <t>Sum «kueiningar» = Kueiningar – storfe [C38] + Kueiningar – småfe [C39]</t>
+        </is>
+      </c>
+      <c r="F40" s="30" t="inlineStr">
+        <is>
+          <t>=C38+C39</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Oksar</t>
+          <t>Korrigert grovfôrareal til storfe</t>
         </is>
       </c>
       <c r="B41" s="21" t="inlineStr">
@@ -46158,30 +46437,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C41" s="22">
-        <f>Oksar!C50*IF(Oversikt!$B$17="J",1,0)</f>
+      <c r="C41" s="36">
+        <f>C22*IF((C49)=0,0,('Mjølk'!C53*IF(Oversikt!$B$16="J",1,0)+Oksar!C50*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C50*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C55*IF(Oversikt!$B$19="J",1,0))/(C49))</f>
         <v/>
       </c>
       <c r="D41" s="12" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>da</t>
         </is>
       </c>
       <c r="E41" s="23" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Oksar = Sum eigen grovfôrproduksjon (utan lagerendring) [Oksar!C50] × Med i totalen Oksar [Oversikt!B17 → 1/0]</t>
+          <t>Korrigert grovfôrareal til storfe = Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C22] × (Sum eigen grovfôrproduksjon (utan lagerendring) [Mjølk!C53] × Med i totalen Mjølk [Oversikt!B16 → 1/0] + Sum eigen grovfôrproduksjon (utan lagerendring) [Oksar!C50] × Med i totalen Oksar [Oversikt!B17 → 1/0] + Sum eigen grovfôrproduksjon (utan lagerendring) [Mellomkalv!C50] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0] + Sum eigen grovfôrproduksjon (utan lagerendring) [Ammekyr!C55] × Med i totalen Ammekyr [Oversikt!B19 → 1/0]) ÷ Sum eigen grovfôrkostnad (fordelingsnøkkel areal) [C49]</t>
         </is>
       </c>
       <c r="F41" s="24" t="inlineStr">
         <is>
-          <t>=Oksar!C50*IF(Oversikt!$B$17="J",1,0)</t>
+          <t>=C22*IF((C49)=0,0,('Mjølk'!C53*IF(Oversikt!$B$16="J",1,0)+Oksar!C50*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C50*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C55*IF(Oversikt!$B$19="J",1,0))/(C49))</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Mellomkalv</t>
+          <t>Korrigerte dekar pr «kueining» – storfe</t>
         </is>
       </c>
       <c r="B42" s="21" t="inlineStr">
@@ -46189,30 +46468,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C42" s="22">
-        <f>Mellomkalv!C50*IF(Oversikt!$B$18="J",1,0)</f>
+      <c r="C42" s="38">
+        <f>IF((C38)=0,0,(C41)/(C38))</f>
         <v/>
       </c>
       <c r="D42" s="12" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>da</t>
         </is>
       </c>
       <c r="E42" s="23" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Mellomkalv = Sum eigen grovfôrproduksjon (utan lagerendring) [Mellomkalv!C50] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0]</t>
+          <t>Korrigerte dekar pr «kueining» – storfe = Korrigert grovfôrareal til storfe [C41] ÷ Kueiningar – storfe [C38]</t>
         </is>
       </c>
       <c r="F42" s="24" t="inlineStr">
         <is>
-          <t>=Mellomkalv!C50*IF(Oversikt!$B$18="J",1,0)</t>
+          <t>=IF((C38)=0,0,(C41)/(C38))</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Ammekyr</t>
+          <t>Eigen grovfôrkostnad – Mjølk</t>
         </is>
       </c>
       <c r="B43" s="21" t="inlineStr">
@@ -46221,7 +46500,7 @@
         </is>
       </c>
       <c r="C43" s="22">
-        <f>Ammekyr!C55*IF(Oversikt!$B$19="J",1,0)</f>
+        <f>'Mjølk'!C53*IF(Oversikt!$B$16="J",1,0)</f>
         <v/>
       </c>
       <c r="D43" s="12" t="inlineStr">
@@ -46231,19 +46510,19 @@
       </c>
       <c r="E43" s="23" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Ammekyr = Sum eigen grovfôrproduksjon (utan lagerendring) [Ammekyr!C55] × Med i totalen Ammekyr [Oversikt!B19 → 1/0]</t>
+          <t>Eigen grovfôrkostnad – Mjølk = Sum eigen grovfôrproduksjon (utan lagerendring) [Mjølk!C53] × Med i totalen Mjølk [Oversikt!B16 → 1/0]</t>
         </is>
       </c>
       <c r="F43" s="24" t="inlineStr">
         <is>
-          <t>=Ammekyr!C55*IF(Oversikt!$B$19="J",1,0)</t>
+          <t>='Mjølk'!C53*IF(Oversikt!$B$16="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Sau</t>
+          <t>Eigen grovfôrkostnad – Oksar</t>
         </is>
       </c>
       <c r="B44" s="21" t="inlineStr">
@@ -46252,7 +46531,7 @@
         </is>
       </c>
       <c r="C44" s="22">
-        <f>Sau!C61*IF(Oversikt!$B$23="J",1,0)</f>
+        <f>Oksar!C50*IF(Oversikt!$B$17="J",1,0)</f>
         <v/>
       </c>
       <c r="D44" s="12" t="inlineStr">
@@ -46262,19 +46541,19 @@
       </c>
       <c r="E44" s="23" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Sau = Sum eigen grovfôrproduksjon (utan lagerendring) [Sau!C61] × Med i totalen Sau [Oversikt!B23 → 1/0]</t>
+          <t>Eigen grovfôrkostnad – Oksar = Sum eigen grovfôrproduksjon (utan lagerendring) [Oksar!C50] × Med i totalen Oksar [Oversikt!B17 → 1/0]</t>
         </is>
       </c>
       <c r="F44" s="24" t="inlineStr">
         <is>
-          <t>=Sau!C61*IF(Oversikt!$B$23="J",1,0)</t>
+          <t>=Oksar!C50*IF(Oversikt!$B$17="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Geit</t>
+          <t>Eigen grovfôrkostnad – Mellomkalv</t>
         </is>
       </c>
       <c r="B45" s="21" t="inlineStr">
@@ -46283,7 +46562,7 @@
         </is>
       </c>
       <c r="C45" s="22">
-        <f>Geit!C49*IF(Oversikt!$B$24="J",1,0)</f>
+        <f>Mellomkalv!C50*IF(Oversikt!$B$18="J",1,0)</f>
         <v/>
       </c>
       <c r="D45" s="12" t="inlineStr">
@@ -46293,19 +46572,19 @@
       </c>
       <c r="E45" s="23" t="inlineStr">
         <is>
-          <t>Eigen grovfôrkostnad – Geit = Sum eigen grovfôrproduksjon (utan lagerendring) [Geit!C49] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
+          <t>Eigen grovfôrkostnad – Mellomkalv = Sum eigen grovfôrproduksjon (utan lagerendring) [Mellomkalv!C50] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0]</t>
         </is>
       </c>
       <c r="F45" s="24" t="inlineStr">
         <is>
-          <t>=Geit!C49*IF(Oversikt!$B$24="J",1,0)</t>
+          <t>=Mellomkalv!C50*IF(Oversikt!$B$18="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>Sum eigen grovfôrkostnad (fordelingsnøkkel areal)</t>
+          <t>Eigen grovfôrkostnad – Ammekyr</t>
         </is>
       </c>
       <c r="B46" s="21" t="inlineStr">
@@ -46314,7 +46593,7 @@
         </is>
       </c>
       <c r="C46" s="22">
-        <f>C40+C41+C42+C43+C44+C45</f>
+        <f>Ammekyr!C55*IF(Oversikt!$B$19="J",1,0)</f>
         <v/>
       </c>
       <c r="D46" s="12" t="inlineStr">
@@ -46324,19 +46603,19 @@
       </c>
       <c r="E46" s="23" t="inlineStr">
         <is>
-          <t>Sum eigen grovfôrkostnad (fordelingsnøkkel areal) = Eigen grovfôrkostnad – Mjølk [C40] + Eigen grovfôrkostnad – Oksar [C41] + Eigen grovfôrkostnad – Mellomkalv [C42] + Eigen grovfôrkostnad – Ammekyr [C43] + Eigen grovfôrkostnad – Sau [C44] + Eigen grovfôrkostnad – Geit [C45]</t>
+          <t>Eigen grovfôrkostnad – Ammekyr = Sum eigen grovfôrproduksjon (utan lagerendring) [Ammekyr!C55] × Med i totalen Ammekyr [Oversikt!B19 → 1/0]</t>
         </is>
       </c>
       <c r="F46" s="24" t="inlineStr">
         <is>
-          <t>=C40+C41+C42+C43+C44+C45</t>
+          <t>=Ammekyr!C55*IF(Oversikt!$B$19="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>Sum variabel grovfôrkostnad (utan plast)</t>
+          <t>Eigen grovfôrkostnad – Sau</t>
         </is>
       </c>
       <c r="B47" s="21" t="inlineStr">
@@ -46345,7 +46624,7 @@
         </is>
       </c>
       <c r="C47" s="22">
-        <f>'Mjølk'!C52*IF(Oversikt!$B$16="J",1,0)+Oksar!C49*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C49*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C54*IF(Oversikt!$B$19="J",1,0)+Sau!C60*IF(Oversikt!$B$23="J",1,0)+Geit!C48*IF(Oversikt!$B$24="J",1,0)</f>
+        <f>Sau!C61*IF(Oversikt!$B$23="J",1,0)</f>
         <v/>
       </c>
       <c r="D47" s="12" t="inlineStr">
@@ -46355,19 +46634,19 @@
       </c>
       <c r="E47" s="23" t="inlineStr">
         <is>
-          <t>Sum variabel grovfôrkostnad (utan plast) = Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Mjølk!C52] × Med i totalen Mjølk [Oversikt!B16 → 1/0] + Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Oksar!C49] × Med i totalen Oksar [Oversikt!B17 → 1/0] + Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Mellomkalv!C49] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0] + Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Ammekyr!C54] × Med i totalen Ammekyr [Oversikt!B19 → 1/0] + Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Sau!C60] × Med i totalen Sau [Oversikt!B23 → 1/0] + Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Geit!C48] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
+          <t>Eigen grovfôrkostnad – Sau = Sum eigen grovfôrproduksjon (utan lagerendring) [Sau!C61] × Med i totalen Sau [Oversikt!B23 → 1/0]</t>
         </is>
       </c>
       <c r="F47" s="24" t="inlineStr">
         <is>
-          <t>='Mjølk'!C52*IF(Oversikt!$B$16="J",1,0)+Oksar!C49*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C49*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C54*IF(Oversikt!$B$19="J",1,0)+Sau!C60*IF(Oversikt!$B$23="J",1,0)+Geit!C48*IF(Oversikt!$B$24="J",1,0)</t>
+          <t>=Sau!C61*IF(Oversikt!$B$23="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>Maskinkostnader i grovfôrproduksjonane</t>
+          <t>Eigen grovfôrkostnad – Geit</t>
         </is>
       </c>
       <c r="B48" s="21" t="inlineStr">
@@ -46376,7 +46655,7 @@
         </is>
       </c>
       <c r="C48" s="22">
-        <f>'Faste kostnader'!C46*IF(Oversikt!$B$16="J",1,0)+'Faste kostnader'!C47*IF(Oversikt!$B$17="J",1,0)+'Faste kostnader'!C48*IF(Oversikt!$B$18="J",1,0)+'Faste kostnader'!C49*IF(Oversikt!$B$19="J",1,0)+'Faste kostnader'!C53*IF(Oversikt!$B$23="J",1,0)+'Faste kostnader'!C54*IF(Oversikt!$B$24="J",1,0)</f>
+        <f>Geit!C49*IF(Oversikt!$B$24="J",1,0)</f>
         <v/>
       </c>
       <c r="D48" s="12" t="inlineStr">
@@ -46386,19 +46665,19 @@
       </c>
       <c r="E48" s="23" t="inlineStr">
         <is>
-          <t>Maskinkostnader i grovfôrproduksjonane = Maskinkostnader – Mjølk [Faste kostnader!C46] × Med i totalen Mjølk [Oversikt!B16 → 1/0] + Maskinkostnader – Oksar [Faste kostnader!C47] × Med i totalen Oksar [Oversikt!B17 → 1/0] + Maskinkostnader – Mellomkalv [Faste kostnader!C48] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0] + Maskinkostnader – Ammekyr [Faste kostnader!C49] × Med i totalen Ammekyr [Oversikt!B19 → 1/0] + Maskinkostnader – Sau [Faste kostnader!C53] × Med i totalen Sau [Oversikt!B23 → 1/0] + Maskinkostnader – Geit [Faste kostnader!C54] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
+          <t>Eigen grovfôrkostnad – Geit = Sum eigen grovfôrproduksjon (utan lagerendring) [Geit!C49] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
         </is>
       </c>
       <c r="F48" s="24" t="inlineStr">
         <is>
-          <t>='Faste kostnader'!C46*IF(Oversikt!$B$16="J",1,0)+'Faste kostnader'!C47*IF(Oversikt!$B$17="J",1,0)+'Faste kostnader'!C48*IF(Oversikt!$B$18="J",1,0)+'Faste kostnader'!C49*IF(Oversikt!$B$19="J",1,0)+'Faste kostnader'!C53*IF(Oversikt!$B$23="J",1,0)+'Faste kostnader'!C54*IF(Oversikt!$B$24="J",1,0)</t>
+          <t>=Geit!C49*IF(Oversikt!$B$24="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="20" t="inlineStr">
         <is>
-          <t>DB grovfôrbaserte husdyr u/tilskot</t>
+          <t>Sum eigen grovfôrkostnad (fordelingsnøkkel areal)</t>
         </is>
       </c>
       <c r="B49" s="21" t="inlineStr">
@@ -46407,7 +46686,7 @@
         </is>
       </c>
       <c r="C49" s="22">
-        <f>'Mjølk'!C56*IF(Oversikt!$B$16="J",1,0)+Oksar!C53*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C53*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C58*IF(Oversikt!$B$19="J",1,0)+Sau!C64*IF(Oversikt!$B$23="J",1,0)+Geit!C52*IF(Oversikt!$B$24="J",1,0)</f>
+        <f>C43+C44+C45+C46+C47+C48</f>
         <v/>
       </c>
       <c r="D49" s="12" t="inlineStr">
@@ -46417,19 +46696,19 @@
       </c>
       <c r="E49" s="23" t="inlineStr">
         <is>
-          <t>DB grovfôrbaserte husdyr u/tilskot = Dekningsbidrag (DB) utan tilskot [Mjølk!C56] × Med i totalen Mjølk [Oversikt!B16 → 1/0] + Dekningsbidrag (DB) utan tilskot [Oksar!C53] × Med i totalen Oksar [Oversikt!B17 → 1/0] + Dekningsbidrag (DB) utan tilskot [Mellomkalv!C53] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0] + Dekningsbidrag (DB) utan tilskot [Ammekyr!C58] × Med i totalen Ammekyr [Oversikt!B19 → 1/0] + Dekningsbidrag (DB) utan tilskot [Sau!C64] × Med i totalen Sau [Oversikt!B23 → 1/0] + Dekningsbidrag (DB) utan tilskot [Geit!C52] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
+          <t>Sum eigen grovfôrkostnad (fordelingsnøkkel areal) = Eigen grovfôrkostnad – Mjølk [C43] + Eigen grovfôrkostnad – Oksar [C44] + Eigen grovfôrkostnad – Mellomkalv [C45] + Eigen grovfôrkostnad – Ammekyr [C46] + Eigen grovfôrkostnad – Sau [C47] + Eigen grovfôrkostnad – Geit [C48]</t>
         </is>
       </c>
       <c r="F49" s="24" t="inlineStr">
         <is>
-          <t>='Mjølk'!C56*IF(Oversikt!$B$16="J",1,0)+Oksar!C53*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C53*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C58*IF(Oversikt!$B$19="J",1,0)+Sau!C64*IF(Oversikt!$B$23="J",1,0)+Geit!C52*IF(Oversikt!$B$24="J",1,0)</t>
+          <t>=C43+C44+C45+C46+C47+C48</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="20" t="inlineStr">
         <is>
-          <t>DB grovfôrbaserte husdyr m/tilskot</t>
+          <t>Sum variabel grovfôrkostnad (utan plast)</t>
         </is>
       </c>
       <c r="B50" s="21" t="inlineStr">
@@ -46438,7 +46717,7 @@
         </is>
       </c>
       <c r="C50" s="22">
-        <f>'Mjølk'!C57*IF(Oversikt!$B$16="J",1,0)+Oksar!C54*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C54*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C59*IF(Oversikt!$B$19="J",1,0)+Sau!C65*IF(Oversikt!$B$23="J",1,0)+Geit!C53*IF(Oversikt!$B$24="J",1,0)</f>
+        <f>'Mjølk'!C52*IF(Oversikt!$B$16="J",1,0)+Oksar!C49*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C49*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C54*IF(Oversikt!$B$19="J",1,0)+Sau!C60*IF(Oversikt!$B$23="J",1,0)+Geit!C48*IF(Oversikt!$B$24="J",1,0)</f>
         <v/>
       </c>
       <c r="D50" s="12" t="inlineStr">
@@ -46448,31 +46727,50 @@
       </c>
       <c r="E50" s="23" t="inlineStr">
         <is>
-          <t>DB grovfôrbaserte husdyr m/tilskot = Dekningsbidrag (DB) med tilskot [Mjølk!C57] × Med i totalen Mjølk [Oversikt!B16 → 1/0] + Dekningsbidrag (DB) med tilskot [Oksar!C54] × Med i totalen Oksar [Oversikt!B17 → 1/0] + Dekningsbidrag (DB) med tilskot [Mellomkalv!C54] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0] + Dekningsbidrag (DB) med tilskot [Ammekyr!C59] × Med i totalen Ammekyr [Oversikt!B19 → 1/0] + Dekningsbidrag (DB) med tilskot [Sau!C65] × Med i totalen Sau [Oversikt!B23 → 1/0] + Dekningsbidrag (DB) med tilskot [Geit!C53] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
+          <t>Sum variabel grovfôrkostnad (utan plast) = Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Mjølk!C52] × Med i totalen Mjølk [Oversikt!B16 → 1/0] + Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Oksar!C49] × Med i totalen Oksar [Oversikt!B17 → 1/0] + Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Mellomkalv!C49] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0] + Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Ammekyr!C54] × Med i totalen Ammekyr [Oversikt!B19 → 1/0] + Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Sau!C60] × Med i totalen Sau [Oversikt!B23 → 1/0] + Variabel grovfôrkostnad (utan plast og lagerendring eigenprodusert) [Geit!C48] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
         </is>
       </c>
       <c r="F50" s="24" t="inlineStr">
         <is>
-          <t>='Mjølk'!C57*IF(Oversikt!$B$16="J",1,0)+Oksar!C54*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C54*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C59*IF(Oversikt!$B$19="J",1,0)+Sau!C65*IF(Oversikt!$B$23="J",1,0)+Geit!C53*IF(Oversikt!$B$24="J",1,0)</t>
+          <t>='Mjølk'!C52*IF(Oversikt!$B$16="J",1,0)+Oksar!C49*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C49*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C54*IF(Oversikt!$B$19="J",1,0)+Sau!C60*IF(Oversikt!$B$23="J",1,0)+Geit!C48*IF(Oversikt!$B$24="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="18" t="inlineStr">
-        <is>
-          <t>4b. UTREKNING – Arealbehov etter fôrnorm (kontroll av grovfôrbalansen)</t>
-        </is>
-      </c>
-      <c r="B51" s="19" t="n"/>
-      <c r="C51" s="19" t="n"/>
-      <c r="D51" s="19" t="n"/>
-      <c r="E51" s="19" t="n"/>
-      <c r="F51" s="19" t="n"/>
+      <c r="A51" s="20" t="inlineStr">
+        <is>
+          <t>Maskinkostnader i grovfôrproduksjonane</t>
+        </is>
+      </c>
+      <c r="B51" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C51" s="22">
+        <f>'Faste kostnader'!C46*IF(Oversikt!$B$16="J",1,0)+'Faste kostnader'!C47*IF(Oversikt!$B$17="J",1,0)+'Faste kostnader'!C48*IF(Oversikt!$B$18="J",1,0)+'Faste kostnader'!C49*IF(Oversikt!$B$19="J",1,0)+'Faste kostnader'!C53*IF(Oversikt!$B$23="J",1,0)+'Faste kostnader'!C54*IF(Oversikt!$B$24="J",1,0)</f>
+        <v/>
+      </c>
+      <c r="D51" s="12" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E51" s="23" t="inlineStr">
+        <is>
+          <t>Maskinkostnader i grovfôrproduksjonane = Maskinkostnader – Mjølk [Faste kostnader!C46] × Med i totalen Mjølk [Oversikt!B16 → 1/0] + Maskinkostnader – Oksar [Faste kostnader!C47] × Med i totalen Oksar [Oversikt!B17 → 1/0] + Maskinkostnader – Mellomkalv [Faste kostnader!C48] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0] + Maskinkostnader – Ammekyr [Faste kostnader!C49] × Med i totalen Ammekyr [Oversikt!B19 → 1/0] + Maskinkostnader – Sau [Faste kostnader!C53] × Med i totalen Sau [Oversikt!B23 → 1/0] + Maskinkostnader – Geit [Faste kostnader!C54] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
+        </is>
+      </c>
+      <c r="F51" s="24" t="inlineStr">
+        <is>
+          <t>='Faste kostnader'!C46*IF(Oversikt!$B$16="J",1,0)+'Faste kostnader'!C47*IF(Oversikt!$B$17="J",1,0)+'Faste kostnader'!C48*IF(Oversikt!$B$18="J",1,0)+'Faste kostnader'!C49*IF(Oversikt!$B$19="J",1,0)+'Faste kostnader'!C53*IF(Oversikt!$B$23="J",1,0)+'Faste kostnader'!C54*IF(Oversikt!$B$24="J",1,0)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="20" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Mjølk</t>
+          <t>DB grovfôrbaserte husdyr u/tilskot</t>
         </is>
       </c>
       <c r="B52" s="21" t="inlineStr">
@@ -46480,30 +46778,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C52" s="36">
-        <f>'Mjølk'!C7*('Mjølk'!C17/625+'Mjølk'!C18/650)*IF(Oversikt!$B$16="J",1,0)</f>
+      <c r="C52" s="22">
+        <f>'Mjølk'!C56*IF(Oversikt!$B$16="J",1,0)+Oksar!C53*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C53*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C58*IF(Oversikt!$B$19="J",1,0)+Sau!C64*IF(Oversikt!$B$23="J",1,0)+Geit!C52*IF(Oversikt!$B$24="J",1,0)</f>
         <v/>
       </c>
       <c r="D52" s="12" t="inlineStr">
         <is>
-          <t>da</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E52" s="23" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Mjølk = Tal årskyr [Mjølk!C7] × (Fôrnorm beite (FEm) [Mjølk!C17] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Mjølk!C18] / 650) × Med i totalen Mjølk [Oversikt!B16 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
+          <t>DB grovfôrbaserte husdyr u/tilskot = Dekningsbidrag (DB) utan tilskot [Mjølk!C56] × Med i totalen Mjølk [Oversikt!B16 → 1/0] + Dekningsbidrag (DB) utan tilskot [Oksar!C53] × Med i totalen Oksar [Oversikt!B17 → 1/0] + Dekningsbidrag (DB) utan tilskot [Mellomkalv!C53] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0] + Dekningsbidrag (DB) utan tilskot [Ammekyr!C58] × Med i totalen Ammekyr [Oversikt!B19 → 1/0] + Dekningsbidrag (DB) utan tilskot [Sau!C64] × Med i totalen Sau [Oversikt!B23 → 1/0] + Dekningsbidrag (DB) utan tilskot [Geit!C52] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
         </is>
       </c>
       <c r="F52" s="24" t="inlineStr">
         <is>
-          <t>='Mjølk'!C7*('Mjølk'!C17/625+'Mjølk'!C18/650)*IF(Oversikt!$B$16="J",1,0)</t>
+          <t>='Mjølk'!C56*IF(Oversikt!$B$16="J",1,0)+Oksar!C53*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C53*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C58*IF(Oversikt!$B$19="J",1,0)+Sau!C64*IF(Oversikt!$B$23="J",1,0)+Geit!C52*IF(Oversikt!$B$24="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="20" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Oksar</t>
+          <t>DB grovfôrbaserte husdyr m/tilskot</t>
         </is>
       </c>
       <c r="B53" s="21" t="inlineStr">
@@ -46511,61 +46809,42 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C53" s="36">
-        <f>Oksar!C7*(Oksar!C16/625+Oksar!C17/650)*IF(Oversikt!$B$17="J",1,0)</f>
+      <c r="C53" s="22">
+        <f>'Mjølk'!C57*IF(Oversikt!$B$16="J",1,0)+Oksar!C54*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C54*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C59*IF(Oversikt!$B$19="J",1,0)+Sau!C65*IF(Oversikt!$B$23="J",1,0)+Geit!C53*IF(Oversikt!$B$24="J",1,0)</f>
         <v/>
       </c>
       <c r="D53" s="12" t="inlineStr">
         <is>
-          <t>da</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E53" s="23" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Oksar = Tal produserte oksar [Oksar!C7] × (Fôrnorm beite (FEm) [Oksar!C16] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Oksar!C17] / 650) × Med i totalen Oksar [Oversikt!B17 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
+          <t>DB grovfôrbaserte husdyr m/tilskot = Dekningsbidrag (DB) med tilskot [Mjølk!C57] × Med i totalen Mjølk [Oversikt!B16 → 1/0] + Dekningsbidrag (DB) med tilskot [Oksar!C54] × Med i totalen Oksar [Oversikt!B17 → 1/0] + Dekningsbidrag (DB) med tilskot [Mellomkalv!C54] × Med i totalen Mellomkalv [Oversikt!B18 → 1/0] + Dekningsbidrag (DB) med tilskot [Ammekyr!C59] × Med i totalen Ammekyr [Oversikt!B19 → 1/0] + Dekningsbidrag (DB) med tilskot [Sau!C65] × Med i totalen Sau [Oversikt!B23 → 1/0] + Dekningsbidrag (DB) med tilskot [Geit!C53] × Med i totalen Geit [Oversikt!B24 → 1/0]</t>
         </is>
       </c>
       <c r="F53" s="24" t="inlineStr">
         <is>
-          <t>=Oksar!C7*(Oksar!C16/625+Oksar!C17/650)*IF(Oversikt!$B$17="J",1,0)</t>
+          <t>='Mjølk'!C57*IF(Oversikt!$B$16="J",1,0)+Oksar!C54*IF(Oversikt!$B$17="J",1,0)+Mellomkalv!C54*IF(Oversikt!$B$18="J",1,0)+Ammekyr!C59*IF(Oversikt!$B$19="J",1,0)+Sau!C65*IF(Oversikt!$B$23="J",1,0)+Geit!C53*IF(Oversikt!$B$24="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="20" t="inlineStr">
-        <is>
-          <t>Arealbehov etter fôrnorm – Mellomkalv</t>
-        </is>
-      </c>
-      <c r="B54" s="21" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C54" s="36">
-        <f>Mellomkalv!C7*(Mellomkalv!C16/625+Mellomkalv!C17/650)*IF(Oversikt!$B$18="J",1,0)</f>
-        <v/>
-      </c>
-      <c r="D54" s="12" t="inlineStr">
-        <is>
-          <t>da</t>
-        </is>
-      </c>
-      <c r="E54" s="23" t="inlineStr">
-        <is>
-          <t>Arealbehov etter fôrnorm – Mellomkalv = Tal produserte kalvar [Mellomkalv!C7] × (Fôrnorm beite (FEm) [Mellomkalv!C16] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Mellomkalv!C17] / 650) × Med i totalen Mellomkalv [Oversikt!B18 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
-        </is>
-      </c>
-      <c r="F54" s="24" t="inlineStr">
-        <is>
-          <t>=Mellomkalv!C7*(Mellomkalv!C16/625+Mellomkalv!C17/650)*IF(Oversikt!$B$18="J",1,0)</t>
-        </is>
-      </c>
+      <c r="A54" s="18" t="inlineStr">
+        <is>
+          <t>4b. UTREKNING – Arealbehov etter fôrnorm (kontroll av grovfôrbalansen)</t>
+        </is>
+      </c>
+      <c r="B54" s="19" t="n"/>
+      <c r="C54" s="19" t="n"/>
+      <c r="D54" s="19" t="n"/>
+      <c r="E54" s="19" t="n"/>
+      <c r="F54" s="19" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="20" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Ammekyr</t>
+          <t>Arealbehov etter fôrnorm – Mjølk</t>
         </is>
       </c>
       <c r="B55" s="21" t="inlineStr">
@@ -46574,7 +46853,7 @@
         </is>
       </c>
       <c r="C55" s="36">
-        <f>Ammekyr!C7*(Ammekyr!C21/625+Ammekyr!C22/650)*IF(Oversikt!$B$19="J",1,0)</f>
+        <f>'Mjølk'!C7*('Mjølk'!C17/625+'Mjølk'!C18/650)*IF(Oversikt!$B$16="J",1,0)</f>
         <v/>
       </c>
       <c r="D55" s="12" t="inlineStr">
@@ -46584,19 +46863,19 @@
       </c>
       <c r="E55" s="23" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Ammekyr = Tal ammekyr [Ammekyr!C7] × (Fôrnorm beite (FEm) [Ammekyr!C21] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Ammekyr!C22] / 650) × Med i totalen Ammekyr [Oversikt!B19 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
+          <t>Arealbehov etter fôrnorm – Mjølk = Tal årskyr [Mjølk!C7] × (Fôrnorm beite (FEm) [Mjølk!C17] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Mjølk!C18] / 650) × Med i totalen Mjølk [Oversikt!B16 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
         </is>
       </c>
       <c r="F55" s="24" t="inlineStr">
         <is>
-          <t>=Ammekyr!C7*(Ammekyr!C21/625+Ammekyr!C22/650)*IF(Oversikt!$B$19="J",1,0)</t>
+          <t>='Mjølk'!C7*('Mjølk'!C17/625+'Mjølk'!C18/650)*IF(Oversikt!$B$16="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="20" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Sau</t>
+          <t>Arealbehov etter fôrnorm – Oksar</t>
         </is>
       </c>
       <c r="B56" s="21" t="inlineStr">
@@ -46605,7 +46884,7 @@
         </is>
       </c>
       <c r="C56" s="36">
-        <f>Sau!C7*(Sau!C25/625+Sau!C26/650)*IF(Oversikt!$B$23="J",1,0)</f>
+        <f>Oksar!C7*(Oksar!C16/625+Oksar!C17/650)*IF(Oversikt!$B$17="J",1,0)</f>
         <v/>
       </c>
       <c r="D56" s="12" t="inlineStr">
@@ -46615,19 +46894,19 @@
       </c>
       <c r="E56" s="23" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Sau = Tal vinterfôra sau [Sau!C7] × (Fôrnorm beite (FEm) [Sau!C25] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Sau!C26] / 650) × Med i totalen Sau [Oversikt!B23 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
+          <t>Arealbehov etter fôrnorm – Oksar = Tal produserte oksar [Oksar!C7] × (Fôrnorm beite (FEm) [Oksar!C16] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Oksar!C17] / 650) × Med i totalen Oksar [Oversikt!B17 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
         </is>
       </c>
       <c r="F56" s="24" t="inlineStr">
         <is>
-          <t>=Sau!C7*(Sau!C25/625+Sau!C26/650)*IF(Oversikt!$B$23="J",1,0)</t>
+          <t>=Oksar!C7*(Oksar!C16/625+Oksar!C17/650)*IF(Oversikt!$B$17="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="20" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Geit</t>
+          <t>Arealbehov etter fôrnorm – Mellomkalv</t>
         </is>
       </c>
       <c r="B57" s="21" t="inlineStr">
@@ -46636,7 +46915,7 @@
         </is>
       </c>
       <c r="C57" s="36">
-        <f>Geit!C7*(Geit!C14/625+Geit!C15/650)*IF(Oversikt!$B$24="J",1,0)</f>
+        <f>Mellomkalv!C7*(Mellomkalv!C16/625+Mellomkalv!C17/650)*IF(Oversikt!$B$18="J",1,0)</f>
         <v/>
       </c>
       <c r="D57" s="12" t="inlineStr">
@@ -46646,155 +46925,155 @@
       </c>
       <c r="E57" s="23" t="inlineStr">
         <is>
-          <t>Arealbehov etter fôrnorm – Geit = Tal årsgeiter [Geit!C7] × (Fôrnorm beite (FEm) [Geit!C14] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Geit!C15] / 650) × Med i totalen Geit [Oversikt!B24 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
+          <t>Arealbehov etter fôrnorm – Mellomkalv = Tal produserte kalvar [Mellomkalv!C7] × (Fôrnorm beite (FEm) [Mellomkalv!C16] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Mellomkalv!C17] / 650) × Med i totalen Mellomkalv [Oversikt!B18 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
         </is>
       </c>
       <c r="F57" s="24" t="inlineStr">
         <is>
-          <t>=Geit!C7*(Geit!C14/625+Geit!C15/650)*IF(Oversikt!$B$24="J",1,0)</t>
+          <t>=Mellomkalv!C7*(Mellomkalv!C16/625+Mellomkalv!C17/650)*IF(Oversikt!$B$18="J",1,0)</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="20" t="inlineStr">
         <is>
+          <t>Arealbehov etter fôrnorm – Ammekyr</t>
+        </is>
+      </c>
+      <c r="B58" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C58" s="36">
+        <f>Ammekyr!C7*(Ammekyr!C21/625+Ammekyr!C22/650)*IF(Oversikt!$B$19="J",1,0)</f>
+        <v/>
+      </c>
+      <c r="D58" s="12" t="inlineStr">
+        <is>
+          <t>da</t>
+        </is>
+      </c>
+      <c r="E58" s="23" t="inlineStr">
+        <is>
+          <t>Arealbehov etter fôrnorm – Ammekyr = Tal ammekyr [Ammekyr!C7] × (Fôrnorm beite (FEm) [Ammekyr!C21] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Ammekyr!C22] / 650) × Med i totalen Ammekyr [Oversikt!B19 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
+        </is>
+      </c>
+      <c r="F58" s="24" t="inlineStr">
+        <is>
+          <t>=Ammekyr!C7*(Ammekyr!C21/625+Ammekyr!C22/650)*IF(Oversikt!$B$19="J",1,0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="20" t="inlineStr">
+        <is>
+          <t>Arealbehov etter fôrnorm – Sau</t>
+        </is>
+      </c>
+      <c r="B59" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C59" s="36">
+        <f>Sau!C7*(Sau!C25/625+Sau!C26/650)*IF(Oversikt!$B$23="J",1,0)</f>
+        <v/>
+      </c>
+      <c r="D59" s="12" t="inlineStr">
+        <is>
+          <t>da</t>
+        </is>
+      </c>
+      <c r="E59" s="23" t="inlineStr">
+        <is>
+          <t>Arealbehov etter fôrnorm – Sau = Tal vinterfôra sau [Sau!C7] × (Fôrnorm beite (FEm) [Sau!C25] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Sau!C26] / 650) × Med i totalen Sau [Oversikt!B23 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
+        </is>
+      </c>
+      <c r="F59" s="24" t="inlineStr">
+        <is>
+          <t>=Sau!C7*(Sau!C25/625+Sau!C26/650)*IF(Oversikt!$B$23="J",1,0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="20" t="inlineStr">
+        <is>
+          <t>Arealbehov etter fôrnorm – Geit</t>
+        </is>
+      </c>
+      <c r="B60" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C60" s="36">
+        <f>Geit!C7*(Geit!C14/625+Geit!C15/650)*IF(Oversikt!$B$24="J",1,0)</f>
+        <v/>
+      </c>
+      <c r="D60" s="12" t="inlineStr">
+        <is>
+          <t>da</t>
+        </is>
+      </c>
+      <c r="E60" s="23" t="inlineStr">
+        <is>
+          <t>Arealbehov etter fôrnorm – Geit = Tal årsgeiter [Geit!C7] × (Fôrnorm beite (FEm) [Geit!C14] / 625 + Fôrnorm eige grovfôr vinter (FEm) [Geit!C15] / 650) × Med i totalen Geit [Oversikt!B24 → 1/0]   (Beite 250 FEm/da delt på 2,5 og eige grovfôr 650 FEm/da – same omrekning som korrigert areal)</t>
+        </is>
+      </c>
+      <c r="F60" s="24" t="inlineStr">
+        <is>
+          <t>=Geit!C7*(Geit!C14/625+Geit!C15/650)*IF(Oversikt!$B$24="J",1,0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="20" t="inlineStr">
+        <is>
           <t>Sum arealbehov etter fôrnorm</t>
         </is>
       </c>
-      <c r="B58" s="21" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C58" s="36">
-        <f>C52+C53+C54+C55+C56+C57</f>
-        <v/>
-      </c>
-      <c r="D58" s="12" t="inlineStr">
+      <c r="B61" s="21" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C61" s="36">
+        <f>C55+C56+C57+C58+C59+C60</f>
+        <v/>
+      </c>
+      <c r="D61" s="12" t="inlineStr">
         <is>
           <t>da</t>
         </is>
       </c>
-      <c r="E58" s="23" t="inlineStr">
-        <is>
-          <t>Sum arealbehov etter fôrnorm = Arealbehov etter fôrnorm – Mjølk [C52] + Arealbehov etter fôrnorm – Oksar [C53] + Arealbehov etter fôrnorm – Mellomkalv [C54] + Arealbehov etter fôrnorm – Ammekyr [C55] + Arealbehov etter fôrnorm – Sau [C56] + Arealbehov etter fôrnorm – Geit [C57]</t>
-        </is>
-      </c>
-      <c r="F58" s="24" t="inlineStr">
-        <is>
-          <t>=C52+C53+C54+C55+C56+C57</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="18" t="inlineStr">
+      <c r="E61" s="23" t="inlineStr">
+        <is>
+          <t>Sum arealbehov etter fôrnorm = Arealbehov etter fôrnorm – Mjølk [C55] + Arealbehov etter fôrnorm – Oksar [C56] + Arealbehov etter fôrnorm – Mellomkalv [C57] + Arealbehov etter fôrnorm – Ammekyr [C58] + Arealbehov etter fôrnorm – Sau [C59] + Arealbehov etter fôrnorm – Geit [C60]</t>
+        </is>
+      </c>
+      <c r="F61" s="24" t="inlineStr">
+        <is>
+          <t>=C55+C56+C57+C58+C59+C60</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="18" t="inlineStr">
         <is>
           <t>5. OUTPUT – Nøkkeltal grovfôr</t>
         </is>
       </c>
-      <c r="B59" s="19" t="n"/>
-      <c r="C59" s="19" t="n"/>
-      <c r="D59" s="19" t="n"/>
-      <c r="E59" s="19" t="n"/>
-      <c r="F59" s="19" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="25" t="inlineStr">
-        <is>
-          <t>Variabel grovfôrkostnad pr korrigert dekar</t>
-        </is>
-      </c>
-      <c r="B60" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C60" s="39">
-        <f>IF((C22)=0,0,(C47)/(C22))</f>
-        <v/>
-      </c>
-      <c r="D60" s="28" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E60" s="29" t="inlineStr">
-        <is>
-          <t>Variabel grovfôrkostnad pr korrigert dekar = Sum variabel grovfôrkostnad (utan plast) [C47] ÷ Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C22]</t>
-        </is>
-      </c>
-      <c r="F60" s="30" t="inlineStr">
-        <is>
-          <t>=IF((C22)=0,0,(C47)/(C22))</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="25" t="inlineStr">
-        <is>
-          <t>Maskinkostnader pr dekar grovfôr</t>
-        </is>
-      </c>
-      <c r="B61" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C61" s="39">
-        <f>IF((C25)=0,0,(C48)/(C25))</f>
-        <v/>
-      </c>
-      <c r="D61" s="28" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E61" s="29" t="inlineStr">
-        <is>
-          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader i grovfôrproduksjonane [C48] ÷ Dekar grovfôr – maskinkostnadsgrunnlag (overflate/2 + fulldyrka + kulturbeite×10 %) [C25]</t>
-        </is>
-      </c>
-      <c r="F61" s="30" t="inlineStr">
-        <is>
-          <t>=IF((C25)=0,0,(C48)/(C25))</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="25" t="inlineStr">
-        <is>
-          <t>Korrigerte dekar pr «kueining»</t>
-        </is>
-      </c>
-      <c r="B62" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C62" s="39">
-        <f>IF((C39)=0,0,(C22)/(C39))</f>
-        <v/>
-      </c>
-      <c r="D62" s="28" t="inlineStr">
-        <is>
-          <t>da</t>
-        </is>
-      </c>
-      <c r="E62" s="29" t="inlineStr">
-        <is>
-          <t>Korrigerte dekar pr «kueining» = Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C22] ÷ Sum «kueiningar» [C39]</t>
-        </is>
-      </c>
-      <c r="F62" s="30" t="inlineStr">
-        <is>
-          <t>=IF((C39)=0,0,(C22)/(C39))</t>
-        </is>
-      </c>
+      <c r="B62" s="19" t="n"/>
+      <c r="C62" s="19" t="n"/>
+      <c r="D62" s="19" t="n"/>
+      <c r="E62" s="19" t="n"/>
+      <c r="F62" s="19" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>Dekar fulldyrka pr «kueining»</t>
+          <t>Variabel grovfôrkostnad pr korrigert dekar</t>
         </is>
       </c>
       <c r="B63" s="26" t="inlineStr">
@@ -46803,29 +47082,29 @@
         </is>
       </c>
       <c r="C63" s="39">
-        <f>IF((C39)=0,0,(C18)/(C39))</f>
+        <f>IF((C22)=0,0,(C50)/(C22))</f>
         <v/>
       </c>
       <c r="D63" s="28" t="inlineStr">
         <is>
-          <t>da</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E63" s="29" t="inlineStr">
         <is>
-          <t>Dekar fulldyrka pr «kueining» = Fulldyrka til eigen grovfôrbasert husdyrproduksjon [C18] ÷ Sum «kueiningar» [C39]</t>
+          <t>Variabel grovfôrkostnad pr korrigert dekar = Sum variabel grovfôrkostnad (utan plast) [C50] ÷ Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C22]</t>
         </is>
       </c>
       <c r="F63" s="30" t="inlineStr">
         <is>
-          <t>=IF((C39)=0,0,(C18)/(C39))</t>
+          <t>=IF((C22)=0,0,(C50)/(C22))</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="25" t="inlineStr">
         <is>
-          <t>Dekar kulturbeite pr «kueining»</t>
+          <t>Maskinkostnader pr dekar grovfôr</t>
         </is>
       </c>
       <c r="B64" s="26" t="inlineStr">
@@ -46834,29 +47113,29 @@
         </is>
       </c>
       <c r="C64" s="39">
-        <f>IF((C39)=0,0,(C19)/(C39))</f>
+        <f>IF((C25)=0,0,(C51)/(C25))</f>
         <v/>
       </c>
       <c r="D64" s="28" t="inlineStr">
         <is>
-          <t>da</t>
+          <t>kr</t>
         </is>
       </c>
       <c r="E64" s="29" t="inlineStr">
         <is>
-          <t>Dekar kulturbeite pr «kueining» = Kulturbeite til eige bruk [C19] ÷ Sum «kueiningar» [C39]</t>
+          <t>Maskinkostnader pr dekar grovfôr = Maskinkostnader i grovfôrproduksjonane [C51] ÷ Dekar grovfôr – maskinkostnadsgrunnlag (overflate/2 + fulldyrka + kulturbeite×10 %) [C25]</t>
         </is>
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>=IF((C39)=0,0,(C19)/(C39))</t>
+          <t>=IF((C25)=0,0,(C51)/(C25))</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="25" t="inlineStr">
         <is>
-          <t>FEm frå utmark pr «kueining»</t>
+          <t>Korrigerte dekar pr «kueining»</t>
         </is>
       </c>
       <c r="B65" s="26" t="inlineStr">
@@ -46864,30 +47143,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C65" s="27">
-        <f>IF((C39)=0,0,(C28)/(C39))</f>
+      <c r="C65" s="39">
+        <f>IF((C40)=0,0,(C22)/(C40))</f>
         <v/>
       </c>
       <c r="D65" s="28" t="inlineStr">
         <is>
-          <t>FEm</t>
+          <t>da</t>
         </is>
       </c>
       <c r="E65" s="29" t="inlineStr">
         <is>
-          <t>FEm frå utmark pr «kueining» = Fôreiningar (FEm) henta frå utmark [C28] ÷ Sum «kueiningar» [C39]</t>
+          <t>Korrigerte dekar pr «kueining» = Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C22] ÷ Sum «kueiningar» [C40]</t>
         </is>
       </c>
       <c r="F65" s="30" t="inlineStr">
         <is>
-          <t>=IF((C39)=0,0,(C28)/(C39))</t>
+          <t>=IF((C40)=0,0,(C22)/(C40))</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="25" t="inlineStr">
         <is>
-          <t>DB grovfôrbaserte husdyr u/tilskot pr korrigert dekar</t>
+          <t>Dekar fulldyrka pr «kueining»</t>
         </is>
       </c>
       <c r="B66" s="26" t="inlineStr">
@@ -46896,29 +47175,29 @@
         </is>
       </c>
       <c r="C66" s="39">
-        <f>IF((C22)=0,0,(C49)/(C22))</f>
+        <f>IF((C40)=0,0,(C18)/(C40))</f>
         <v/>
       </c>
       <c r="D66" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>da</t>
         </is>
       </c>
       <c r="E66" s="29" t="inlineStr">
         <is>
-          <t>DB grovfôrbaserte husdyr u/tilskot pr korrigert dekar = DB grovfôrbaserte husdyr u/tilskot [C49] ÷ Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C22]</t>
+          <t>Dekar fulldyrka pr «kueining» = Fulldyrka til eigen grovfôrbasert husdyrproduksjon [C18] ÷ Sum «kueiningar» [C40]</t>
         </is>
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>=IF((C22)=0,0,(C49)/(C22))</t>
+          <t>=IF((C40)=0,0,(C18)/(C40))</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="25" t="inlineStr">
         <is>
-          <t>DB grovfôrbaserte husdyr m/tilskot pr korrigert dekar</t>
+          <t>Dekar kulturbeite pr «kueining»</t>
         </is>
       </c>
       <c r="B67" s="26" t="inlineStr">
@@ -46927,53 +47206,146 @@
         </is>
       </c>
       <c r="C67" s="39">
-        <f>IF((C22)=0,0,(C50)/(C22))</f>
+        <f>IF((C40)=0,0,(C19)/(C40))</f>
         <v/>
       </c>
       <c r="D67" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>da</t>
         </is>
       </c>
       <c r="E67" s="29" t="inlineStr">
         <is>
-          <t>DB grovfôrbaserte husdyr m/tilskot pr korrigert dekar = DB grovfôrbaserte husdyr m/tilskot [C50] ÷ Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C22]</t>
+          <t>Dekar kulturbeite pr «kueining» = Kulturbeite til eige bruk [C19] ÷ Sum «kueiningar» [C40]</t>
         </is>
       </c>
       <c r="F67" s="30" t="inlineStr">
         <is>
-          <t>=IF((C22)=0,0,(C50)/(C22))</t>
+          <t>=IF((C40)=0,0,(C19)/(C40))</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="25" t="inlineStr">
         <is>
+          <t>FEm frå utmark pr «kueining»</t>
+        </is>
+      </c>
+      <c r="B68" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C68" s="27">
+        <f>IF((C40)=0,0,(C29)/(C40))</f>
+        <v/>
+      </c>
+      <c r="D68" s="28" t="inlineStr">
+        <is>
+          <t>FEm</t>
+        </is>
+      </c>
+      <c r="E68" s="29" t="inlineStr">
+        <is>
+          <t>FEm frå utmark pr «kueining» = Fôreiningar (FEm) henta frå utmark [C29] ÷ Sum «kueiningar» [C40]</t>
+        </is>
+      </c>
+      <c r="F68" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C40)=0,0,(C29)/(C40))</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="25" t="inlineStr">
+        <is>
+          <t>DB grovfôrbaserte husdyr u/tilskot pr korrigert dekar</t>
+        </is>
+      </c>
+      <c r="B69" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C69" s="39">
+        <f>IF((C22)=0,0,(C52)/(C22))</f>
+        <v/>
+      </c>
+      <c r="D69" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E69" s="29" t="inlineStr">
+        <is>
+          <t>DB grovfôrbaserte husdyr u/tilskot pr korrigert dekar = DB grovfôrbaserte husdyr u/tilskot [C52] ÷ Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C22]</t>
+        </is>
+      </c>
+      <c r="F69" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C22)=0,0,(C52)/(C22))</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="25" t="inlineStr">
+        <is>
+          <t>DB grovfôrbaserte husdyr m/tilskot pr korrigert dekar</t>
+        </is>
+      </c>
+      <c r="B70" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C70" s="39">
+        <f>IF((C22)=0,0,(C53)/(C22))</f>
+        <v/>
+      </c>
+      <c r="D70" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E70" s="29" t="inlineStr">
+        <is>
+          <t>DB grovfôrbaserte husdyr m/tilskot pr korrigert dekar = DB grovfôrbaserte husdyr m/tilskot [C53] ÷ Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C22]</t>
+        </is>
+      </c>
+      <c r="F70" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C22)=0,0,(C53)/(C22))</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="25" t="inlineStr">
+        <is>
           <t>Korrigert grovfôrareal i % av arealbehov etter fôrnorm</t>
         </is>
       </c>
-      <c r="B68" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C68" s="33">
-        <f>IF((C58)=0,0,(C22)/(C58))</f>
-        <v/>
-      </c>
-      <c r="D68" s="28" t="inlineStr">
+      <c r="B71" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C71" s="33">
+        <f>IF((C61)=0,0,(C22)/(C61))</f>
+        <v/>
+      </c>
+      <c r="D71" s="28" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E68" s="29" t="inlineStr">
-        <is>
-          <t>Korrigert grovfôrareal i % av arealbehov etter fôrnorm = Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C22] ÷ Sum arealbehov etter fôrnorm [C58]   (Under 100 % tyder på kjøpt fôr eller høge avlingar, over 100 % på overskot av areal)</t>
-        </is>
-      </c>
-      <c r="F68" s="30" t="inlineStr">
-        <is>
-          <t>=IF((C58)=0,0,(C22)/(C58))</t>
+      <c r="E71" s="29" t="inlineStr">
+        <is>
+          <t>Korrigert grovfôrareal i % av arealbehov etter fôrnorm = Korrigert grovfôrareal (overflate/1,25 + fulldyrka + kulturbeite/2,5) [C22] ÷ Sum arealbehov etter fôrnorm [C61]   (Under 100 % tyder på kjøpt fôr eller høge avlingar, over 100 % på overskot av areal)</t>
+        </is>
+      </c>
+      <c r="F71" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C61)=0,0,(C22)/(C61))</t>
         </is>
       </c>
     </row>
@@ -46989,7 +47361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -48263,7 +48635,7 @@
     <row r="53">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar</t>
+          <t>Seld avling pr dekar (kg)</t>
         </is>
       </c>
       <c r="B53" s="26" t="inlineStr">
@@ -48271,52 +48643,83 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C53" s="39">
-        <f>IF((C7)=0,0,(C22)/(C7))</f>
+      <c r="C53" s="37">
+        <f>IF((C7)=0,0,(C9)/(C7))</f>
         <v/>
       </c>
       <c r="D53" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E53" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar = Maskinkostnader fordelt [C22] ÷ Tal dekar [C7]</t>
+          <t>Seld avling pr dekar (kg) = Seld mengd [C9] ÷ Tal dekar [C7]</t>
         </is>
       </c>
       <c r="F53" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C22)/(C7))</t>
+          <t>=IF((C7)=0,0,(C9)/(C7))</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="25" t="inlineStr">
         <is>
+          <t>Maskinkostnader pr dekar</t>
+        </is>
+      </c>
+      <c r="B54" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C54" s="39">
+        <f>IF((C7)=0,0,(C22)/(C7))</f>
+        <v/>
+      </c>
+      <c r="D54" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E54" s="29" t="inlineStr">
+        <is>
+          <t>Maskinkostnader pr dekar = Maskinkostnader fordelt [C22] ÷ Tal dekar [C7]</t>
+        </is>
+      </c>
+      <c r="F54" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C7)=0,0,(C22)/(C7))</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="25" t="inlineStr">
+        <is>
           <t>DB etter maskinkostnader pr dekar</t>
         </is>
       </c>
-      <c r="B54" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C54" s="39">
+      <c r="B55" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C55" s="39">
         <f>IF((C7)=0,0,(C28)/(C7))</f>
         <v/>
       </c>
-      <c r="D54" s="28" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E54" s="29" t="inlineStr">
+      <c r="D55" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E55" s="29" t="inlineStr">
         <is>
           <t>DB etter maskinkostnader pr dekar = DB m/tilskot etter maskinkostnader [C28] ÷ Tal dekar [C7]</t>
         </is>
       </c>
-      <c r="F54" s="30" t="inlineStr">
+      <c r="F55" s="30" t="inlineStr">
         <is>
           <t>=IF((C7)=0,0,(C28)/(C7))</t>
         </is>
@@ -48334,7 +48737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -49603,7 +50006,7 @@
     <row r="53">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar</t>
+          <t>Seld avling pr dekar (kg)</t>
         </is>
       </c>
       <c r="B53" s="26" t="inlineStr">
@@ -49611,30 +50014,30 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C53" s="39">
-        <f>IF((C7)=0,0,(C23)/(C7))</f>
+      <c r="C53" s="37">
+        <f>IF((C7)=0,0,(C9)/(C7))</f>
         <v/>
       </c>
       <c r="D53" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E53" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar = Maskinkostnader fordelt [C23] ÷ Tal dekar [C7]</t>
+          <t>Seld avling pr dekar (kg) = Seld mengd [C9] ÷ Tal dekar [C7]</t>
         </is>
       </c>
       <c r="F53" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C23)/(C7))</t>
+          <t>=IF((C7)=0,0,(C9)/(C7))</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>DB etter maskinkostnader pr dekar</t>
+          <t>Maskinkostnader pr dekar</t>
         </is>
       </c>
       <c r="B54" s="26" t="inlineStr">
@@ -49643,7 +50046,7 @@
         </is>
       </c>
       <c r="C54" s="39">
-        <f>IF((C7)=0,0,(C29)/(C7))</f>
+        <f>IF((C7)=0,0,(C23)/(C7))</f>
         <v/>
       </c>
       <c r="D54" s="28" t="inlineStr">
@@ -49653,19 +50056,19 @@
       </c>
       <c r="E54" s="29" t="inlineStr">
         <is>
-          <t>DB etter maskinkostnader pr dekar = DB m/tilskot etter maskinkostnader [C29] ÷ Tal dekar [C7]</t>
+          <t>Maskinkostnader pr dekar = Maskinkostnader fordelt [C23] ÷ Tal dekar [C7]</t>
         </is>
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C29)/(C7))</t>
+          <t>=IF((C7)=0,0,(C23)/(C7))</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>Oppnådd pris pr siloballe</t>
+          <t>DB etter maskinkostnader pr dekar</t>
         </is>
       </c>
       <c r="B55" s="26" t="inlineStr">
@@ -49674,7 +50077,7 @@
         </is>
       </c>
       <c r="C55" s="39">
-        <f>IF((C10)=0,0,(C14)/(C10))</f>
+        <f>IF((C7)=0,0,(C29)/(C7))</f>
         <v/>
       </c>
       <c r="D55" s="28" t="inlineStr">
@@ -49684,41 +50087,72 @@
       </c>
       <c r="E55" s="29" t="inlineStr">
         <is>
-          <t>Oppnådd pris pr siloballe = Sal av silofôr [C14] ÷ Tal siloballar seld [C10]</t>
+          <t>DB etter maskinkostnader pr dekar = DB m/tilskot etter maskinkostnader [C29] ÷ Tal dekar [C7]</t>
         </is>
       </c>
       <c r="F55" s="30" t="inlineStr">
         <is>
-          <t>=IF((C10)=0,0,(C14)/(C10))</t>
+          <t>=IF((C7)=0,0,(C29)/(C7))</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="25" t="inlineStr">
         <is>
+          <t>Oppnådd pris pr siloballe</t>
+        </is>
+      </c>
+      <c r="B56" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C56" s="39">
+        <f>IF((C10)=0,0,(C14)/(C10))</f>
+        <v/>
+      </c>
+      <c r="D56" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E56" s="29" t="inlineStr">
+        <is>
+          <t>Oppnådd pris pr siloballe = Sal av silofôr [C14] ÷ Tal siloballar seld [C10]</t>
+        </is>
+      </c>
+      <c r="F56" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C10)=0,0,(C14)/(C10))</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="25" t="inlineStr">
+        <is>
           <t>Tal siloballar pr dekar</t>
         </is>
       </c>
-      <c r="B56" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C56" s="39">
+      <c r="B57" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C57" s="39">
         <f>IF((C7)=0,0,(C10+C11/750)/(C7))</f>
         <v/>
       </c>
-      <c r="D56" s="28" t="inlineStr">
+      <c r="D57" s="28" t="inlineStr">
         <is>
           <t>stk</t>
         </is>
       </c>
-      <c r="E56" s="29" t="inlineStr">
+      <c r="E57" s="29" t="inlineStr">
         <is>
           <t>Tal siloballar pr dekar = (Tal siloballar seld [C10] + Auke i varelager (kg) [C11] / 750) ÷ Tal dekar [C7]   (Lagerauke i kg er rekna om til ballar med 750 kg pr balle)</t>
         </is>
       </c>
-      <c r="F56" s="30" t="inlineStr">
+      <c r="F57" s="30" t="inlineStr">
         <is>
           <t>=IF((C7)=0,0,(C10+C11/750)/(C7))</t>
         </is>
@@ -49736,7 +50170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -50953,7 +51387,7 @@
     <row r="51">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar</t>
+          <t>Seld avling pr dekar (kg)</t>
         </is>
       </c>
       <c r="B51" s="26" t="inlineStr">
@@ -50961,52 +51395,83 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C51" s="39">
-        <f>IF((C7)=0,0,(C21)/(C7))</f>
+      <c r="C51" s="37">
+        <f>IF((C7)=0,0,(C9)/(C7))</f>
         <v/>
       </c>
       <c r="D51" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E51" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar = Maskinkostnader fordelt [C21] ÷ Tal dekar [C7]</t>
+          <t>Seld avling pr dekar (kg) = Seld mengd [C9] ÷ Tal dekar [C7]</t>
         </is>
       </c>
       <c r="F51" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C21)/(C7))</t>
+          <t>=IF((C7)=0,0,(C9)/(C7))</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="25" t="inlineStr">
         <is>
+          <t>Maskinkostnader pr dekar</t>
+        </is>
+      </c>
+      <c r="B52" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C52" s="39">
+        <f>IF((C7)=0,0,(C21)/(C7))</f>
+        <v/>
+      </c>
+      <c r="D52" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E52" s="29" t="inlineStr">
+        <is>
+          <t>Maskinkostnader pr dekar = Maskinkostnader fordelt [C21] ÷ Tal dekar [C7]</t>
+        </is>
+      </c>
+      <c r="F52" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C7)=0,0,(C21)/(C7))</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="25" t="inlineStr">
+        <is>
           <t>DB etter maskinkostnader pr dekar</t>
         </is>
       </c>
-      <c r="B52" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C52" s="39">
+      <c r="B53" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C53" s="39">
         <f>IF((C7)=0,0,(C27)/(C7))</f>
         <v/>
       </c>
-      <c r="D52" s="28" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E52" s="29" t="inlineStr">
+      <c r="D53" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E53" s="29" t="inlineStr">
         <is>
           <t>DB etter maskinkostnader pr dekar = DB m/tilskot etter maskinkostnader [C27] ÷ Tal dekar [C7]</t>
         </is>
       </c>
-      <c r="F52" s="30" t="inlineStr">
+      <c r="F53" s="30" t="inlineStr">
         <is>
           <t>=IF((C7)=0,0,(C27)/(C7))</t>
         </is>
@@ -51024,7 +51489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -52298,7 +52763,7 @@
     <row r="53">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar</t>
+          <t>Seld avling pr dekar (kg)</t>
         </is>
       </c>
       <c r="B53" s="26" t="inlineStr">
@@ -52306,52 +52771,83 @@
           <t>Utrekna</t>
         </is>
       </c>
-      <c r="C53" s="39">
-        <f>IF((C7)=0,0,(C22)/(C7))</f>
+      <c r="C53" s="37">
+        <f>IF((C7)=0,0,(C9)/(C7))</f>
         <v/>
       </c>
       <c r="D53" s="28" t="inlineStr">
         <is>
-          <t>kr</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E53" s="29" t="inlineStr">
         <is>
-          <t>Maskinkostnader pr dekar = Maskinkostnader fordelt [C22] ÷ Tal dekar [C7]</t>
+          <t>Seld avling pr dekar (kg) = Seld mengd [C9] ÷ Tal dekar [C7]</t>
         </is>
       </c>
       <c r="F53" s="30" t="inlineStr">
         <is>
-          <t>=IF((C7)=0,0,(C22)/(C7))</t>
+          <t>=IF((C7)=0,0,(C9)/(C7))</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="25" t="inlineStr">
         <is>
+          <t>Maskinkostnader pr dekar</t>
+        </is>
+      </c>
+      <c r="B54" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C54" s="39">
+        <f>IF((C7)=0,0,(C22)/(C7))</f>
+        <v/>
+      </c>
+      <c r="D54" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E54" s="29" t="inlineStr">
+        <is>
+          <t>Maskinkostnader pr dekar = Maskinkostnader fordelt [C22] ÷ Tal dekar [C7]</t>
+        </is>
+      </c>
+      <c r="F54" s="30" t="inlineStr">
+        <is>
+          <t>=IF((C7)=0,0,(C22)/(C7))</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="25" t="inlineStr">
+        <is>
           <t>DB etter maskinkostnader pr dekar</t>
         </is>
       </c>
-      <c r="B54" s="26" t="inlineStr">
-        <is>
-          <t>Utrekna</t>
-        </is>
-      </c>
-      <c r="C54" s="39">
+      <c r="B55" s="26" t="inlineStr">
+        <is>
+          <t>Utrekna</t>
+        </is>
+      </c>
+      <c r="C55" s="39">
         <f>IF((C7)=0,0,(C28)/(C7))</f>
         <v/>
       </c>
-      <c r="D54" s="28" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="E54" s="29" t="inlineStr">
+      <c r="D55" s="28" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="E55" s="29" t="inlineStr">
         <is>
           <t>DB etter maskinkostnader pr dekar = DB m/tilskot etter maskinkostnader [C28] ÷ Tal dekar [C7]</t>
         </is>
       </c>
-      <c r="F54" s="30" t="inlineStr">
+      <c r="F55" s="30" t="inlineStr">
         <is>
           <t>=IF((C7)=0,0,(C28)/(C7))</t>
         </is>

</xml_diff>